<commit_message>
feat(roles): derive sourced engineering-management ladder
Fully sources all 43 competencies x 6 levels (258 mappings) with bibliography
citations and per-level why text, grounded in the catalog's P1-P6 profiles.
Harvests role evidence from the prior authored ladder where it passes the
cell-derivation instance test; re-maps STRAT-01 M4 from P5 to P4 to match the
sub-org scope band, mirroring the same fix already applied on the platform
engineering management ladder. Marks the role derived and regenerates
ladder.md/ladder.csv/ladder.xlsx.
</commit_message>
<xml_diff>
--- a/roles/engineering-management/ladder.xlsx
+++ b/roles/engineering-management/ladder.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Overview" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Competency Matrix" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Rating Template" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Sources" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Sources &amp; Theory" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -696,20 +696,21 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K44"/>
+  <dimension ref="A1:L44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
     <col width="18" customWidth="1" min="2" max="2"/>
     <col width="24" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="40" customWidth="1" min="5" max="5"/>
-    <col width="55" customWidth="1" min="6" max="6"/>
+    <col width="45" customWidth="1" min="5" max="5"/>
+    <col width="45" customWidth="1" min="6" max="6"/>
     <col width="55" customWidth="1" min="7" max="7"/>
     <col width="55" customWidth="1" min="8" max="8"/>
     <col width="55" customWidth="1" min="9" max="9"/>
     <col width="55" customWidth="1" min="10" max="10"/>
     <col width="55" customWidth="1" min="11" max="11"/>
+    <col width="55" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -735,35 +736,40 @@
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>Theory Anchor</t>
+          <t>What it covers</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
+          <t>Theory anchor &amp; why</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
           <t>M1</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>M2</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>M3</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>M4</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>M5</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>M6</t>
         </is>
@@ -792,37 +798,42 @@
       </c>
       <c r="E2" s="4" t="inlineStr">
         <is>
-          <t>Rumelt, Good Strategy Bad Strategy (2011)</t>
+          <t>Define enterprise direction, scope, and competitive positioning to create durable advantage.</t>
         </is>
       </c>
       <c r="F2" s="4" t="inlineStr">
         <is>
-          <t>Depth: Writes a team charter that names the problem the team exists to solve and ties each quarter's plan to an honest diagnosis of the team's real constraints; explains in planning why this, why now — and why not the alternatives. Scope: one team's plan, traceable to org priorities.</t>
+          <t>Rumelt, Good Strategy Bad Strategy: The Difference and Why It Matters (Crown Business, 2011) — real strategy is a diagnosis plus a coherent guiding policy and actions, not goals restated as ambition</t>
         </is>
       </c>
       <c r="G2" s="4" t="inlineStr">
         <is>
-          <t>Depth: Frames a critical team's strategy as diagnosis, guiding policy, and coherent action in a document others can challenge; spots when a "strategy" is goals restated as ambition and reframes it around the actual obstacle; kills or re-scopes work that fails the test. Scope: a complex / critical team; peer managers borrow the framing.</t>
+          <t>Depth: Develops components of strategy and standard analyses independently with normal review. Evidenced by: Writes a team charter that names the problem the team exists to solve, not just its goals. Scope: one team.</t>
         </is>
       </c>
       <c r="H2" s="4" t="inlineStr">
         <is>
-          <t>Depth: Writes the domain strategy several teams plan against, naming the bets, explicit non-goals, and rejected alternatives; kills initiatives that do not serve it, saying why in the open. Scope: a cross-team domain; cited by teams the author does not run.</t>
+          <t>Depth: Frames ambiguous strategic problems and shapes coherent strategy autonomously; the go-to strategist. Evidenced by: Reframes a team's stalled 'strategy' around its actual obstacle after spotting it was really just goals restated as ambition. Scope: a complex / critical team.</t>
         </is>
       </c>
       <c r="I2" s="4" t="inlineStr">
         <is>
-          <t>Depth: Reconciles competing team strategies into one coherent investment thesis, cutting real programs to fund the guiding policy; leaders they coach write strategies that pass the same test. Scope: a sub-org's portfolio; funding and staffing follow the document.</t>
+          <t>Depth: Defines strategy-formulation approaches others adopt; resolves the hardest strategic trade-offs. Evidenced by: Publishes the domain strategy several teams plan against, naming the bets, non-goals, and rejected alternatives. Scope: a domain (cross-team).</t>
         </is>
       </c>
       <c r="J2" s="4" t="inlineStr">
         <is>
-          <t>Depth: Sets multi-year direction for a function and defends its trade-offs at the executive table with market and delivery evidence; product and finance plans reference its bets. Scope: a function; the strategy shapes decisions in rooms they are not in.</t>
+          <t>Depth: Defines strategy-formulation approaches others adopt; resolves the hardest strategic trade-offs. Evidenced by: Reconciles competing team strategies into one coherent investment thesis, cutting real programs to fund the guiding policy. Scope: a sub-org.</t>
         </is>
       </c>
       <c r="K2" s="4" t="inlineStr">
         <is>
-          <t>Depth: Frames the company-level technical bets the executive team commits to, revising the diagnosis publicly when it changes; leaders at every level can defend the logic. Scope: org-wide; visible in board-level material.</t>
+          <t>Depth: Sets the enterprise strategic direction; anticipates major shifts reshaping the competitive landscape. Evidenced by: Sets multi-year direction for a function and defends its trade-offs at the executive table with market and delivery evidence. Scope: a function.</t>
+        </is>
+      </c>
+      <c r="L2" s="4" t="inlineStr">
+        <is>
+          <t>Depth: Defines corporate-strategy practice recognized industry-wide; externally cited thought leader. Evidenced by: Frames the company-level bets the executive team commits to, and revises the diagnosis publicly when it changes. Scope: org-wide.</t>
         </is>
       </c>
     </row>
@@ -849,37 +860,42 @@
       </c>
       <c r="E3" s="4" t="inlineStr">
         <is>
-          <t>Locke &amp; Latham, goal-setting theory (2002); Collins &amp; Porras (1996)</t>
+          <t>Translate strategy into multi-horizon plans and cascading objectives across the enterprise.</t>
         </is>
       </c>
       <c r="F3" s="4" t="inlineStr">
         <is>
-          <t>Depth: Translates org direction into team goals specific enough that anyone can say whether they were hit, restates the why at kickoffs so every engineer can explain it to an outsider, and flags work that ladders to no goal. Scope: one team's goals and their upward trace.</t>
+          <t>Doerr, Measure What Matters: How Google, Bono, and the Gates Foundation Rock the World with OKRs (Portfolio/Penguin, 2018) — cascading objectives is how strategy becomes goals people can hit or miss, not just a slogan</t>
         </is>
       </c>
       <c r="G3" s="4" t="inlineStr">
         <is>
-          <t>Depth: Paints a one-page picture of where the team is heading in 12–18 months and repairs vague or sandbagged goals during planning — leading indicators, counter-metrics against gaming; resets targets publicly when the situation changes rather than quietly redefining success. Scope: a critical team; partners repeat the picture unprompted.</t>
+          <t>Depth: Runs standard planning cycles and cascades objectives independently with normal review. Evidenced by: Translates org direction into team goals specific enough that anyone can say whether they were hit. Scope: one team.</t>
         </is>
       </c>
       <c r="H3" s="4" t="inlineStr">
         <is>
-          <t>Depth: Runs the goal cadence a domain uses so objectives interlock across teams, catching collisions — one team's target is another's counter-metric — before the quarter starts. Scope: cross-team; teams outside their span adopt the cascade format.</t>
+          <t>Depth: Designs planning for complex, interdependent units and resolves misalignment autonomously. Evidenced by: Repairs a vague or sandbagged goal during planning by adding leading indicators and a counter-metric against gaming. Scope: a complex / critical team.</t>
         </is>
       </c>
       <c r="I3" s="4" t="inlineStr">
         <is>
-          <t>Depth: Builds the goal architecture a sub-org runs on — drafting, calibration, and scoring rituals that function without them in the room — and aligns leaders with conflicting incentives around one destination. Scope: a sub-org; the cascade holds without their weekly presence.</t>
+          <t>Depth: Defines the planning and goal-cascade methodology others adopt; fixes the hardest alignment failures. Evidenced by: Runs the goal cadence a domain uses so objectives interlock across teams, catching collisions before the quarter starts. Scope: a domain (cross-team).</t>
         </is>
       </c>
       <c r="J3" s="4" t="inlineStr">
         <is>
-          <t>Depth: Sets function-level outcomes the business plans around, brokering trade-offs with product and finance and holding the line when teams optimize local metrics against them. Scope: a function; company scorecards carry their measures.</t>
+          <t>Depth: Defines the planning and goal-cascade methodology others adopt; fixes the hardest alignment failures. Evidenced by: Builds the goal architecture a sub-org runs on, calibration and scoring rituals included, that functions without them in the room. Scope: a sub-org.</t>
         </is>
       </c>
       <c r="K3" s="4" t="inlineStr">
         <is>
-          <t>Depth: Audits the line of sight from mission to every level's goals and publicly retires goals that no longer serve it; the org's identity — what it intends to be known for — is repeated until hiring and architecture visibly bend toward it. Scope: org-wide; annual planning starts from their frame.</t>
+          <t>Depth: Sets the enterprise planning operating model; anticipates shifts in how strategy translates to execution. Evidenced by: Sets function-level outcomes the business plans around, brokering trade-offs with product and finance. Scope: a function.</t>
+        </is>
+      </c>
+      <c r="L3" s="4" t="inlineStr">
+        <is>
+          <t>Depth: Defines strategic-planning best practice recognized across the field; externally credible authority. Evidenced by: Audits the line of sight from mission to every level's goals, and publicly retires goals that no longer serve it. Scope: org-wide.</t>
         </is>
       </c>
     </row>
@@ -906,37 +922,42 @@
       </c>
       <c r="E4" s="4" t="inlineStr">
         <is>
-          <t>Kotter, Leading Change (1996)</t>
+          <t>Leading teams through reorganization, process change, and shifting priorities.</t>
         </is>
       </c>
       <c r="F4" s="4" t="inlineStr">
         <is>
-          <t>Depth: Lands a team-level change by naming the why, piloting it, and following through past the initial dip; the team can explain the reason, not just the rule. Scope: one team; the change sticks after attention moves on.</t>
+          <t>Kotter, Leading Change (Harvard Business School Press, 1996) — durable change needs urgency, a guiding coalition, and follow-through, not a mandate</t>
         </is>
       </c>
       <c r="G4" s="4" t="inlineStr">
         <is>
-          <t>Depth: Sequences a disruptive change on a critical team — migration, re-team, practice overhaul — with a stated case for urgency and staged early wins, and publicly kills a change that is not working rather than letting it linger. Scope: a complex team; peers copy the rollout plan.</t>
+          <t>Depth: Leads a contained team change with normal review. Evidenced by: Lands a team-level change by naming the why, piloting it, and following through past the initial dip. Scope: one team.</t>
         </is>
       </c>
       <c r="H4" s="4" t="inlineStr">
         <is>
-          <t>Depth: Builds the coalition for a cross-team change before announcing it — recruits early adopters, arms them with evidence, converts skeptics on the record; adoption is voluntary before it is mandatory. Scope: a domain; teams they do not run adopt the change.</t>
+          <t>Depth: Independently drives significant change through resistance to durable adoption. Evidenced by: Sequences a disruptive change on a critical team with a stated case for urgency and staged early wins, and kills it publicly if it is not working. Scope: a complex / critical team.</t>
         </is>
       </c>
       <c r="I4" s="4" t="inlineStr">
         <is>
-          <t>Depth: Runs multiple concurrent changes without exceeding the org's absorption capacity, with explicit reversal criteria and a communication plan that reaches every affected person before the rumor does; grows the leaders who run the workstreams. Scope: a sub-org; the change sticks after they stop pushing.</t>
+          <t>Depth: Defines change approaches others adopt and rescues stalled transformations. Evidenced by: Builds the coalition for a cross-team change before announcing it, recruiting early adopters and converting skeptics on the record. Scope: a domain (cross-team).</t>
         </is>
       </c>
       <c r="J4" s="4" t="inlineStr">
         <is>
-          <t>Depth: Leads function-wide transformation with an honest cost narrative executives sign up for, anchoring the change in reviews, incentives, and hiring criteria so the old way cannot quietly return. Scope: a function; the change model is reused for the next transformation.</t>
+          <t>Depth: Defines change approaches others adopt and rescues stalled transformations. Evidenced by: Runs multiple concurrent changes across a sub-org without exceeding its absorption capacity, with explicit reversal criteria. Scope: a sub-org.</t>
         </is>
       </c>
       <c r="K4" s="4" t="inlineStr">
         <is>
-          <t>Depth: Times and frames org-wide change against market conditions, absorbing the political cost personally so teams can execute; the change survives leadership churn because it lives in mechanisms and culture, not in their presence. Scope: org-wide, including external partners and customers.</t>
+          <t>Depth: Sets the org's transformation strategy and anticipates where change is needed next. Evidenced by: Leads function-wide transformation with an honest cost narrative executives sign up for, anchored in reviews and incentives. Scope: a function.</t>
+        </is>
+      </c>
+      <c r="L4" s="4" t="inlineStr">
+        <is>
+          <t>Depth: Defines effective engineering transformation for the discipline and shapes external practice. Evidenced by: Times and frames org-wide change against market conditions, absorbing the political cost personally so teams can execute. Scope: org-wide.</t>
         </is>
       </c>
     </row>
@@ -963,37 +984,42 @@
       </c>
       <c r="E5" s="4" t="inlineStr">
         <is>
-          <t>Skelton &amp; Pais, Team Topologies (2019); Conway (1968)</t>
+          <t>Shaping team topologies, roles, and reporting lines to fit the work and scale.</t>
         </is>
       </c>
       <c r="F5" s="4" t="inlineStr">
         <is>
-          <t>Depth: Shapes roles, ownership boundaries, and on-call load inside the team so work flows without waiting on one person; flags cognitive overload with evidence — missed reviews, hero patterns — before it burns people out. Scope: one team's internal structure.</t>
+          <t>Skelton &amp; Pais, Team Topologies (IT Revolution, 2019) — team boundaries, cognitive load, and interaction modes determine architecture and flow</t>
         </is>
       </c>
       <c r="G5" s="4" t="inlineStr">
         <is>
-          <t>Depth: Redraws a team's boundaries and interfaces when the system outgrows them, proposing splits or charter changes with a written rationale and showing the load reduction afterward — fewer handoffs, fewer pages, clearer ownership. Scope: a critical team and the seams it shares with neighbors.</t>
+          <t>Depth: Designs a sound structure for one team with normal review. Evidenced by: Shapes roles, ownership boundaries, and on-call load inside the team so work flows without waiting on one person. Scope: one team.</t>
         </is>
       </c>
       <c r="H5" s="4" t="inlineStr">
         <is>
-          <t>Depth: Designs multi-team boundaries for a domain with the Conway's-law consequences named, grounded in dependency and flow evidence; neighboring leads co-sign the design, and predicted interface fractures are named before they happen. Scope: a domain's topology; adopted by managers who do not answer to them.</t>
+          <t>Depth: Independently restructures teams to fit changing work and resolves boundary conflicts. Evidenced by: Redraws a team's boundaries when the system outgrows them, showing the load reduction afterward -- fewer handoffs, fewer pages. Scope: a complex / critical team.</t>
         </is>
       </c>
       <c r="I5" s="4" t="inlineStr">
         <is>
-          <t>Depth: Designs a sub-org's structure around the work rather than around people — platform versus stream teams, interaction contracts, new leadership seats — modeling transition costs and dependencies before the announcement. Scope: a sub-org; the structure outlives them.</t>
+          <t>Depth: Defines org-design approaches others adopt and reshapes the most tangled structures. Evidenced by: Designs multi-team boundaries for a domain with the Conway's-law consequences named; neighboring leads co-sign the design. Scope: a domain (cross-team).</t>
         </is>
       </c>
       <c r="J5" s="4" t="inlineStr">
         <is>
-          <t>Depth: Sets the function's principles for when to split, merge, or platformize teams, evolving its shape ahead of scale inflections; structural decisions below them come out consistent without escalation. Scope: a function's topology.</t>
+          <t>Depth: Defines org-design approaches others adopt and reshapes the most tangled structures. Evidenced by: Designs a sub-org's structure around the work rather than around people, modeling transition costs before the announcement. Scope: a sub-org.</t>
         </is>
       </c>
       <c r="K5" s="4" t="inlineStr">
         <is>
-          <t>Depth: Publishes the org-wide design principles other leaders use for their own restructures and times structural change to strategy rather than crisis. Scope: org-wide; Conway effects are anticipated in company architecture.</t>
+          <t>Depth: Sets org-structuring strategy across the org and anticipates scaling inflection points. Evidenced by: Sets the function's principles for when to split, merge, or platformize teams, evolving shape ahead of scale inflections. Scope: a function.</t>
+        </is>
+      </c>
+      <c r="L5" s="4" t="inlineStr">
+        <is>
+          <t>Depth: Defines effective engineering-org design for the discipline and is cited externally on it. Evidenced by: Publishes the org-wide design principles other leaders use for their own restructures. Scope: org-wide.</t>
         </is>
       </c>
     </row>
@@ -1020,37 +1046,42 @@
       </c>
       <c r="E6" s="4" t="inlineStr">
         <is>
-          <t>Bungay, The Art of Action (2011)</t>
+          <t>Gets people moving in the same direction.</t>
         </is>
       </c>
       <c r="F6" s="4" t="inlineStr">
         <is>
-          <t>Depth: Closes decisions in the room — states the call, the owner, the revisit date — and writes it down where the team works; ambiguous threads get converted to decisions or killed. Scope: one team's decision log.</t>
+          <t>Bungay, The Art of Action: How Leaders Close the Gaps between Plans, Actions and Results (Nicholas Brealey, 2011) — mission command closes the knowledge, alignment, and effects gaps by briefing intent and freeing method</t>
         </is>
       </c>
       <c r="G6" s="4" t="inlineStr">
         <is>
-          <t>Depth: Briefs intent so well the team makes correct calls in their absence — the what and why stated, the how left free; drift is caught at the weekly, not the postmortem. Scope: a critical team under ambiguity.</t>
+          <t>Depth: Aligns direct partners on scoped decisions. Evidenced by: Closes decisions in the room and writes down the call, the owner, and the revisit date where the team works. Scope: one team.</t>
         </is>
       </c>
       <c r="H6" s="4" t="inlineStr">
         <is>
-          <t>Depth: Aligns teams they do not run on shared intent — one-page briefs, decision forums with real closure rules; disagreement moves to disagree-and-commit on record instead of slow-rolling. Scope: cross-team execution.</t>
+          <t>Depth: Drives alignment across a domain; turns disagreement into committed direction. Evidenced by: Briefs intent so well the team makes correct calls in their absence, catching drift at the weekly instead of the postmortem. Scope: a complex / critical team.</t>
         </is>
       </c>
       <c r="I6" s="4" t="inlineStr">
         <is>
-          <t>Depth: Builds a sub-org's decision architecture — what gets decided where, by whom, how fast — and unblocks stuck decisions by fixing the process, not just the decision. Scope: a sub-org.</t>
+          <t>Depth: Aligns multiple teams and leadership behind a direction. Evidenced by: Aligns teams they do not run on shared intent through one-page briefs and decision forums with real closure rules. Scope: a domain (cross-team).</t>
         </is>
       </c>
       <c r="J6" s="4" t="inlineStr">
         <is>
-          <t>Depth: Aligns a function with company strategy through briefed intent that executives and engineers repeat verbatim — the strategy survives three retellings intact. Scope: a function.</t>
+          <t>Depth: Aligns multiple teams and leadership behind a direction. Evidenced by: Builds a sub-org's decision architecture and unblocks stuck decisions by fixing the process, not just the decision. Scope: a sub-org.</t>
         </is>
       </c>
       <c r="K6" s="4" t="inlineStr">
         <is>
-          <t>Depth: Keeps an entire org pointed at the same intent through noise — repeats the direction until bored, then repeats it again; org-wide decisions visibly trace to it. Scope: org-wide coherence.</t>
+          <t>Depth: Creates forums/narratives through which the org aligns. Evidenced by: Aligns a function with company strategy through briefed intent that executives and engineers repeat verbatim. Scope: a function.</t>
+        </is>
+      </c>
+      <c r="L6" s="4" t="inlineStr">
+        <is>
+          <t>Depth: Aligns the company behind direction; externally persuasive. Evidenced by: Keeps an entire org pointed at the same intent through noise, repeating the direction until org-wide decisions visibly trace to it. Scope: org-wide.</t>
         </is>
       </c>
     </row>
@@ -1077,37 +1108,42 @@
       </c>
       <c r="E7" s="4" t="inlineStr">
         <is>
-          <t>Hersey &amp; Blanchard (1969); Heifetz (1994)</t>
+          <t>Reads what the person, team, and moment need and flexes leadership approach — directing, coaching, supporting, delegating — from a grounded, authentic center; distinguishes technical from adaptive challenges.</t>
         </is>
       </c>
       <c r="F7" s="4" t="inlineStr">
         <is>
-          <t>Depth: Matches direction and support to each person's readiness on each task — directing, coaching, supporting, or delegating deliberately — and tells technical problems from adaptive ones before choosing a fix. Scope: one team's range of people and situations.</t>
+          <t>Hersey &amp; Blanchard, Management of Organizational Behavior: Utilizing Human Resources (Prentice-Hall, 1969) — there is no single right style; the meta-skill is reading what the person, team, and moment need</t>
         </is>
       </c>
       <c r="G7" s="4" t="inlineStr">
         <is>
-          <t>Depth: Flexes skillfully across a wider range of people and harder situations without losing a grounded center; refuses to force technical fixes onto adaptive challenges and names the difference in the room. Scope: a critical team under conflicting demands.</t>
+          <t>Depth: Matches direction and support to each person's readiness per task — directing, coaching, supporting, or delegating deliberately — and tells technical problems from adaptive ones. Evidenced by: Delegates a familiar task to a seasoned engineer and coaches a struggling new hire through the same kind of task step by step, in the same week. Scope: one team.</t>
         </is>
       </c>
       <c r="H7" s="4" t="inlineStr">
         <is>
-          <t>Depth: Coaches other leads to read what a person, team, or moment needs, adapting their own approach across diverse teams while staying recognizably consistent in values. Scope: a domain; leaders cite their situational reads.</t>
+          <t>Depth: Flexes skillfully across a wide range of people and hard situations without losing a grounded center; refuses to force technical fixes onto adaptive challenges and names the difference. Evidenced by: Refuses to force a technical fix onto an adaptive challenge on a critical team, and names the difference in the room. Scope: a complex / critical team.</t>
         </is>
       </c>
       <c r="I7" s="4" t="inlineStr">
         <is>
-          <t>Depth: Develops adaptive leadership as a discipline across a sub-org — teaches leaders to diagnose technical-versus-adaptive at scale and models changing approach when the situation changes. Scope: a sub-org's leadership practice.</t>
+          <t>Depth: Coaches other leaders to read what a person, team, or moment needs; adapts across diverse teams while staying recognizably consistent in values. Evidenced by: Coaches a peer lead who defaults to hands-on rescue to recognize when a team's problem is adaptive, not technical, and to back off instead of fixing it themselves. Scope: a domain (cross-team).</t>
         </is>
       </c>
       <c r="J7" s="4" t="inlineStr">
         <is>
-          <t>Depth: Sets the tone for adaptive, authentic leadership across a function, adjusting their own leadership to what the function needs now rather than what worked last time. Scope: a function.</t>
+          <t>Depth: Coaches other leaders to read what a person, team, or moment needs; adapts across diverse teams while staying recognizably consistent in values. Evidenced by: Develops adaptive leadership as a discipline across a sub-org, teaching leaders to diagnose technical-versus-adaptive at scale. Scope: a sub-org.</t>
         </is>
       </c>
       <c r="K7" s="4" t="inlineStr">
         <is>
-          <t>Depth: Shapes an adaptive, grounded leadership culture org-wide, keeping the org's leadership style plastic to conditions while its values stay fixed. Scope: org-wide.</t>
+          <t>Depth: Develops adaptive leadership as an organizational discipline — leaders diagnose technical-versus-adaptive at scale, and the leadership style changes when the situation does. Evidenced by: Sets the tone for adaptive, authentic leadership across a function, adjusting their own approach to what the function needs now. Scope: a function.</t>
+        </is>
+      </c>
+      <c r="L7" s="4" t="inlineStr">
+        <is>
+          <t>Depth: Shapes an adaptive, grounded leadership culture across an organization — style stays plastic to conditions while values stay fixed; the approach is emulated beyond the organization. Evidenced by: Keeps the org's leadership style recognizable through a merger that could have imported a completely different culture. Scope: org-wide.</t>
         </is>
       </c>
     </row>
@@ -1134,37 +1170,42 @@
       </c>
       <c r="E8" s="4" t="inlineStr">
         <is>
-          <t>McConnell, Software Estimation (2006)</t>
+          <t>Forecasts and plans work credibly.</t>
         </is>
       </c>
       <c r="F8" s="4" t="inlineStr">
         <is>
-          <t>Depth: Publishes a team plan with ranged estimates and named assumptions, breaking goals into a realistic, sequenced plan within capacity; re-plans visibly when reality diverges instead of quietly slipping. Scope: one team's quarter.</t>
+          <t>McConnell, Software Estimation: Demystifying the Black Art (Microsoft Press, 2006) — estimates carry a cone of uncertainty that narrows with knowledge, and honest ranges beat confident points</t>
         </is>
       </c>
       <c r="G8" s="4" t="inlineStr">
         <is>
-          <t>Depth: Plans a critical team through dependency-heavy work — sequencing around external teams, buffering the riskiest items first; their dates are the ones stakeholders trust. Scope: a complex team plus its dependency graph.</t>
+          <t>Depth: Estimates scoped work realistically; plans own 1-3 week projects. Evidenced by: Publishes a team plan with ranged estimates and named assumptions, and re-plans visibly when reality diverges. Scope: one team.</t>
         </is>
       </c>
       <c r="H8" s="4" t="inlineStr">
         <is>
-          <t>Depth: Runs planning across a domain so team plans compose into one deliverable picture; surfaces cross-team collisions weeks early and brokers the re-sequencing. Scope: cross-team; teams they do not run plan on their calendar.</t>
+          <t>Depth: Plans quarter-scale, multi-workstream efforts including dependencies. Evidenced by: Plans a critical team through dependency-heavy work, sequencing around external teams and buffering the riskiest items first. Scope: a complex / critical team.</t>
         </is>
       </c>
       <c r="I8" s="4" t="inlineStr">
         <is>
-          <t>Depth: Builds the planning system a sub-org runs on — cadence, templates, dependency review — and coaches leaders until plan quality is uniform; slips surface in the mechanism, not in hallway surprise. Scope: a sub-org.</t>
+          <t>Depth: Expert at planning large programs; anticipates risk early. Evidenced by: Runs planning across a domain so team plans compose into one deliverable picture, surfacing cross-team collisions weeks early. Scope: a domain (cross-team).</t>
         </is>
       </c>
       <c r="J8" s="4" t="inlineStr">
         <is>
-          <t>Depth: Converts portfolio uncertainty into ranged function-level commitments the business plans around, renegotiating them in the open when the cone of uncertainty narrows. Scope: a function's promises to the company.</t>
+          <t>Depth: Expert at planning large programs; anticipates risk early. Evidenced by: Builds the planning system a sub-org runs on and coaches leaders until plan quality is uniform across it. Scope: a sub-org.</t>
         </is>
       </c>
       <c r="K8" s="4" t="inlineStr">
         <is>
-          <t>Depth: Sets the org's planning philosophy — horizon, cadence, commitment culture — and arbitrates when annual bets collide. Scope: org-wide.</t>
+          <t>Depth: Plans org-level programs across quarters/years. Evidenced by: Converts portfolio uncertainty into ranged function-level commitments the business plans around. Scope: a function.</t>
+        </is>
+      </c>
+      <c r="L8" s="4" t="inlineStr">
+        <is>
+          <t>Depth: Shapes how the company plans major technical change. Evidenced by: Sets the org's planning philosophy -- horizon, cadence, commitment culture -- and arbitrates when annual bets collide. Scope: org-wide.</t>
         </is>
       </c>
     </row>
@@ -1191,37 +1232,42 @@
       </c>
       <c r="E9" s="4" t="inlineStr">
         <is>
-          <t>Reinertsen, The Principles of Product Development Flow (2009)</t>
+          <t>Weighs cost, value, risk and timing.</t>
         </is>
       </c>
       <c r="F9" s="4" t="inlineStr">
         <is>
-          <t>Depth: Ranks the backlog with explicit cost-of-delay reasoning and says no with the reasons attached, showing stakeholders what a new ask displaces; protects committed work from drive-by asks. Scope: one team's queue.</t>
+          <t>Reinertsen, The Principles of Product Development Flow: Second Generation Lean Product Development (Celeritas, 2009) — cost of delay and queue economics make prioritization quantitative instead of loudest-voice-wins</t>
         </is>
       </c>
       <c r="G9" s="4" t="inlineStr">
         <is>
-          <t>Depth: Trades scope, quality, and date on a critical deliverable with the reasoning written down; escalations they raise arrive with options, not just problems. Scope: a complex team; their trade-off memos travel.</t>
+          <t>Depth: Makes sound priority calls within scope; time-boxes uncertain work. Evidenced by: Ranks the backlog with explicit cost-of-delay reasoning and says no to a low-value request with the reasons attached. Scope: one team.</t>
         </is>
       </c>
       <c r="H9" s="4" t="inlineStr">
         <is>
-          <t>Depth: Arbitrates priority conflicts between teams using a shared economic frame they introduced, documenting the trade-offs each team accepted so re-litigations point at the record, not the meeting. Scope: cross-team queues in a domain.</t>
+          <t>Depth: Balances cost/value/risk across a domain; resists hype; decisions hold up over months. Evidenced by: Trades scope, quality, and date on a critical deliverable with the reasoning written down so it travels. Scope: a complex / critical team.</t>
         </is>
       </c>
       <c r="I9" s="4" t="inlineStr">
         <is>
-          <t>Depth: Kills or defers whole initiatives to keep a sub-org's portfolio inside real capacity, delivering the news to sponsors personally and publishing the rationale so the decision teaches; leaders they develop make the same call one level down. Scope: a sub-org's portfolio.</t>
+          <t>Depth: Expert at portfolio-level trade-offs; surfaces hidden assumptions; trusted tiebreaker. Evidenced by: Arbitrates priority conflicts between teams using a shared economic frame they introduced, with the accepted trade-offs on record. Scope: a domain (cross-team).</t>
         </is>
       </c>
       <c r="J9" s="4" t="inlineStr">
         <is>
-          <t>Depth: Sets the investment split across run, grow, and transform for a function with an economic case finance signs off on, defending it against quarter-to-quarter noise. Scope: a function.</t>
+          <t>Depth: Expert at portfolio-level trade-offs; surfaces hidden assumptions; trusted tiebreaker. Evidenced by: Kills or defers whole initiatives to keep a sub-org's portfolio inside real capacity, delivering the news to sponsors personally. Scope: a sub-org.</t>
         </is>
       </c>
       <c r="K9" s="4" t="inlineStr">
         <is>
-          <t>Depth: Makes the org's few irreversible bets explicitly and stages the reversible ones, saying no to good ideas in public so the org learns the bar. Scope: org-wide capacity and capital.</t>
+          <t>Depth: Sets decision frameworks for the org. Evidenced by: Sets the investment split across run, grow, and transform for a function with an economic case finance signs off on. Scope: a function.</t>
+        </is>
+      </c>
+      <c r="L9" s="4" t="inlineStr">
+        <is>
+          <t>Depth: Influences company strategic direction through judgment. Evidenced by: Makes the org's few irreversible bets explicitly and stages the reversible ones, saying no to good ideas in public. Scope: org-wide.</t>
         </is>
       </c>
     </row>
@@ -1248,37 +1294,42 @@
       </c>
       <c r="E10" s="4" t="inlineStr">
         <is>
-          <t>Forsgren, Humble &amp; Kim, Accelerate (2018)</t>
+          <t>Driving cross-team execution, dependencies, and predictable delivery of programs.</t>
         </is>
       </c>
       <c r="F10" s="4" t="inlineStr">
         <is>
-          <t>Depth: Runs a delivery cadence where commitments are met or renegotiated early, never silently missed; delegates, coordinates, unblocks, and flags slips with options, not apologies. Scope: one team's delivery.</t>
+          <t>Forsgren, Humble &amp; Kim, Accelerate: The Science of Lean Software and DevOps (IT Revolution Press, 2018) — software delivery performance predicts organizational performance and is measurable</t>
         </is>
       </c>
       <c r="G10" s="4" t="inlineStr">
         <is>
-          <t>Depth: Keeps delivery predictable on a system with heavy dependencies and legacy drag, recovering a slipping critical program by re-scoping and communicating the new plan before being asked; runs premortems on critical launches and folds the mitigations into the plan. Scope: a critical path other teams depend on.</t>
+          <t>Depth: Drives delivery of a standard program with normal review. Evidenced by: Runs a delivery cadence where commitments are met or renegotiated early, and flags slips with options, not apologies. Scope: one team.</t>
         </is>
       </c>
       <c r="H10" s="4" t="inlineStr">
         <is>
-          <t>Depth: Runs cross-team delivery with dependencies mapped and integration milestones checked, negotiating buffers and interface contracts between teams before integration, not after. Scope: a domain-wide program.</t>
+          <t>Depth: Independently runs complex multi-team programs and recovers slipping delivery. Evidenced by: Recovers a slipping critical program by re-scoping and communicating the new plan before being asked. Scope: a complex / critical team.</t>
         </is>
       </c>
       <c r="I10" s="4" t="inlineStr">
         <is>
-          <t>Depth: Builds the program mechanisms — dependency maps, integration checkpoints, single-threaded owners — that let multi-quarter, multi-team programs land, and coaches other leads to run them. Scope: sub-org-scale programs; the review runs in their absence.</t>
+          <t>Depth: Defines delivery practices others adopt and rescues the most troubled programs. Evidenced by: Runs cross-team delivery with dependencies mapped, negotiating interface contracts between teams before integration, not after. Scope: a domain (cross-team).</t>
         </is>
       </c>
       <c r="J10" s="4" t="inlineStr">
         <is>
-          <t>Depth: Gives executives delivery forecasts they plan the business on, and early warning the moment a forecast breaks, treating misses as prompts for systemic fixes rather than blame. Scope: a function's commitments and delivery reputation.</t>
+          <t>Depth: Defines delivery practices others adopt and rescues the most troubled programs. Evidenced by: Builds the program mechanisms that let multi-quarter, multi-team programs land, and coaches other leads to run them. Scope: a sub-org.</t>
         </is>
       </c>
       <c r="K10" s="4" t="inlineStr">
         <is>
-          <t>Depth: Sets the org's execution bar — what "on time" and "done" mean — and personally intervenes on the few programs whose failure would be existential. Scope: org-wide.</t>
+          <t>Depth: Sets the org's delivery strategy and anticipates systemic delivery risks. Evidenced by: Gives executives delivery forecasts they plan the business on, with early warning the moment a forecast breaks. Scope: a function.</t>
+        </is>
+      </c>
+      <c r="L10" s="4" t="inlineStr">
+        <is>
+          <t>Depth: Defines what excellent program delivery means and shapes external practice. Evidenced by: Sets the org's execution bar for what 'on time' and 'done' mean, and personally intervenes on the few existential programs. Scope: org-wide.</t>
         </is>
       </c>
     </row>
@@ -1305,37 +1356,42 @@
       </c>
       <c r="E11" s="4" t="inlineStr">
         <is>
-          <t>Beyer, Jones, Petoff &amp; Murphy, Site Reliability Engineering (2016)</t>
+          <t>Establishing on-call, incident response, and risk practices that protect reliability.</t>
         </is>
       </c>
       <c r="F11" s="4" t="inlineStr">
         <is>
-          <t>Depth: Runs blameless postmortems that produce completed actions, not filed documents; keeps on-call humane — load tracked, handoffs clean, pages actionable. Scope: one team's services and pager.</t>
+          <t>Beyer, Jones, Petoff &amp; Murphy (eds.), Site Reliability Engineering: How Google Runs Production Systems (O'Reilly/Google, 2016) — error budgets, blameless postmortems, and toil caps make reliability an engineering discipline</t>
         </is>
       </c>
       <c r="G11" s="4" t="inlineStr">
         <is>
-          <t>Depth: Commands sev-1 incidents on a critical system calmly — clear roles, communication cadence, decision log — and pushes reliability work onto the roadmap with error-budget evidence; failure is rehearsed with game days. Scope: a critical system and its blast radius.</t>
+          <t>Depth: Manages standard incidents and routine operational risk with normal review. Evidenced by: Runs blameless postmortems that produce completed actions, not filed documents, and keeps on-call humane. Scope: one team.</t>
         </is>
       </c>
       <c r="H11" s="4" t="inlineStr">
         <is>
-          <t>Depth: Raises the postmortem and readiness bar across a domain — SLOs and error budgets adopted by teams they do not run — and eliminates recurring incident classes with systemic fixes instead of three local patches. Scope: cross-team reliability.</t>
+          <t>Depth: Independently leads severe incidents and drives durable remediation of risk. Evidenced by: Commands sev-1 incidents on a critical system calmly, with clear roles and a decision log, and pushes reliability work onto the roadmap with error-budget evidence. Scope: a complex / critical team.</t>
         </is>
       </c>
       <c r="I11" s="4" t="inlineStr">
         <is>
-          <t>Depth: Builds a sub-org's reliability operating model — SLO governance, severity taxonomy, escalation design, an incident-commander bench — and rehearses it; the org's worst day runs on mechanisms they installed. Scope: a sub-org.</t>
+          <t>Depth: Defines incident and risk practices others adopt and commands the worst crises calmly. Evidenced by: Raises the postmortem and readiness bar across a domain, so SLOs and error budgets are adopted by teams they do not run. Scope: a domain (cross-team).</t>
         </is>
       </c>
       <c r="J11" s="4" t="inlineStr">
         <is>
-          <t>Depth: Represents operational risk at the executive table in customer and revenue terms, setting risk tolerance with the business and defending reliability investment in budget season. Scope: a function's risk position.</t>
+          <t>Depth: Defines incident and risk practices others adopt and commands the worst crises calmly. Evidenced by: Builds a sub-org's reliability operating model -- SLO governance, severity taxonomy, an incident-commander bench -- and rehearses it. Scope: a sub-org.</t>
         </is>
       </c>
       <c r="K11" s="4" t="inlineStr">
         <is>
-          <t>Depth: Represents the org's operational integrity to customers, regulators, and the board during the worst incidents, and turns them into structural investment. Scope: org-wide trust.</t>
+          <t>Depth: Sets the org's operational-risk strategy and anticipates systemic failure modes. Evidenced by: Represents operational risk at the executive table in customer and revenue terms, setting risk tolerance with the business. Scope: a function.</t>
+        </is>
+      </c>
+      <c r="L11" s="4" t="inlineStr">
+        <is>
+          <t>Depth: Defines what excellent operational risk management means and shapes external practice. Evidenced by: Represents the org's operational integrity to customers, regulators, and the board during the worst incidents. Scope: org-wide.</t>
         </is>
       </c>
     </row>
@@ -1362,37 +1418,42 @@
       </c>
       <c r="E12" s="4" t="inlineStr">
         <is>
-          <t>NIST Cybersecurity Framework (2014); PMI PMBOK (2021)</t>
+          <t>Identify, assess, treat, and monitor risks across the organization within a risk appetite.</t>
         </is>
       </c>
       <c r="F12" s="4" t="inlineStr">
         <is>
-          <t>Depth: Keeps a team risk register with named owners and trigger conditions, treats security and compliance findings as scheduled work with deadlines, and escalates when a trigger fires rather than hoping. Scope: one team's plans and attack surface.</t>
+          <t>NIST, The NIST Cybersecurity Framework (CSF) 2.0, NIST CSWP 29 (2024) — risk fails at the management layer -- unowned exposures, unfunded mitigations -- more often than the technical one</t>
         </is>
       </c>
       <c r="G12" s="4" t="inlineStr">
         <is>
-          <t>Depth: Leads a critical system through real risk events — an audit, a coordinated disclosure, a failed dependency — hardening both the system and the process afterward; near-misses get written up, not shrugged off. Scope: a critical system's risk posture.</t>
+          <t>Depth: Conducts standard risk assessments and updates registers independently with normal review. Evidenced by: Keeps a team risk register with named owners and trigger conditions, and escalates when a trigger fires rather than hoping. Scope: one team.</t>
         </is>
       </c>
       <c r="H12" s="4" t="inlineStr">
         <is>
-          <t>Depth: Normalizes risk practice across a domain — shared register format, review cadence, paved-road controls teams adopt because they are easier than the alternative — and maps dependency risk between teams before integration. Scope: cross-team risk posture.</t>
+          <t>Depth: Assesses complex, interconnected enterprise risks and sets local methodology autonomously. Evidenced by: Leads a critical system through a real risk event -- an audit or a failed dependency -- and hardens the system and process afterward. Scope: a complex / critical team.</t>
         </is>
       </c>
       <c r="I12" s="4" t="inlineStr">
         <is>
-          <t>Depth: Builds a sub-org's risk governance — risk-appetite statements, exception processes with expiry dates, compliance readiness under regulated-industry constraints — surfacing systemic exposures like single points of failure and key-person risk, and funding the mitigations. Scope: a sub-org.</t>
+          <t>Depth: Designs the enterprise risk framework and appetite model others adopt; solves the hardest risk problems. Evidenced by: Normalizes risk practice across a domain -- shared register format, review cadence, paved-road controls teams adopt because they are easier. Scope: a domain (cross-team).</t>
         </is>
       </c>
       <c r="J12" s="4" t="inlineStr">
         <is>
-          <t>Depth: Trades risk against delivery at function scale with explicit executive sign-off on accepted risks — no silent acceptance. Scope: a function.</t>
+          <t>Depth: Designs the enterprise risk framework and appetite model others adopt; solves the hardest risk problems. Evidenced by: Builds a sub-org's risk governance -- risk-appetite statements, exception processes with expiry dates -- and funds the mitigations. Scope: a sub-org.</t>
         </is>
       </c>
       <c r="K12" s="4" t="inlineStr">
         <is>
-          <t>Depth: Sets the org's risk appetite and answers for its posture to the board, regulators, and customers, making the hardest calls — disclosure, shutdown, delay — personally and on record. Scope: org-wide.</t>
+          <t>Depth: Sets enterprise risk strategy and appetite at board level; anticipates emerging systemic risks. Evidenced by: Trades risk against delivery at function scale with explicit executive sign-off on accepted risks -- no silent acceptance. Scope: a function.</t>
+        </is>
+      </c>
+      <c r="L12" s="4" t="inlineStr">
+        <is>
+          <t>Depth: Defines enterprise-risk practice recognized industry-wide; externally cited authority. Evidenced by: Sets the org's risk appetite and answers for its posture to the board, regulators, and customers. Scope: org-wide.</t>
         </is>
       </c>
     </row>
@@ -1419,37 +1480,42 @@
       </c>
       <c r="E13" s="4" t="inlineStr">
         <is>
-          <t>Forsgren, Humble &amp; Kim, Accelerate (2018) - DORA four keys</t>
+          <t>Using delivery and health metrics to diagnose and improve team effectiveness.</t>
         </is>
       </c>
       <c r="F13" s="4" t="inlineStr">
         <is>
-          <t>Depth: Reads the team's core health signals — lead time, deploy frequency, change-fail rate, recovery time, test health — on a cadence and acts on one bottleneck at a time; distinguishes the metric moving from the system improving. Scope: one team's pipeline.</t>
+          <t>Forsgren, Humble &amp; Kim, Accelerate: The Science of Lean Software and DevOps (IT Revolution Press, 2018) — the DORA four keys predict organizational performance, and instrumenting them beats arguing from anecdote</t>
         </is>
       </c>
       <c r="G13" s="4" t="inlineStr">
         <is>
-          <t>Depth: Diagnoses a complex team's delivery drag to root cause — flaky tests, review latency, batch size — and shows the improvement in the numbers, not just the narrative; the fix holds for quarters. Scope: a critical delivery path.</t>
+          <t>Depth: Interprets productivity metrics for one team with normal review. Evidenced by: Reads the team's core health signals on a cadence and acts on one bottleneck at a time, distinguishing the metric moving from the system improving. Scope: one team.</t>
         </is>
       </c>
       <c r="H13" s="4" t="inlineStr">
         <is>
-          <t>Depth: Standardizes delivery measurement across a domain so teams are comparable without being gamed; distinguishes real health from vanity metrics, and managers they do not oversee run retros off the dashboard they built. Scope: cross-team.</t>
+          <t>Depth: Independently designs metric systems and distinguishes real signal from vanity numbers. Evidenced by: Diagnoses a complex team's delivery drag to root cause and shows the improvement in the numbers, not just the narrative. Scope: a complex / critical team.</t>
         </is>
       </c>
       <c r="I13" s="4" t="inlineStr">
         <is>
-          <t>Depth: Sets delivery-health standards and instrumentation for a sub-org and funds the platform work that moves them, using trends to guide investment and protecting improvement capacity from roadmap pressure quarter after quarter. Scope: a sub-org.</t>
+          <t>Depth: Defines the productivity-measurement model others adopt and debunks misleading metrics. Evidenced by: Standardizes delivery measurement across a domain so teams are comparable without being gamed. Scope: a domain (cross-team).</t>
         </is>
       </c>
       <c r="J13" s="4" t="inlineStr">
         <is>
-          <t>Depth: Frames engineering productivity for the executive suite in business terms, resisting vanity metrics; the function's improvement investments trace to measured constraints. Scope: a function.</t>
+          <t>Depth: Defines the productivity-measurement model others adopt and debunks misleading metrics. Evidenced by: Sets delivery-health standards and instrumentation for a sub-org and funds the platform work that moves them. Scope: a sub-org.</t>
         </is>
       </c>
       <c r="K13" s="4" t="inlineStr">
         <is>
-          <t>Depth: Makes delivery capability a board-legible asset, benchmarking the org externally, setting the measurement philosophy, and retiring measures that stop informing decisions. Scope: org-wide.</t>
+          <t>Depth: Sets the org's engineering-metrics strategy and anticipates which signals will matter. Evidenced by: Frames engineering productivity for the executive suite in business terms, resisting vanity metrics. Scope: a function.</t>
+        </is>
+      </c>
+      <c r="L13" s="4" t="inlineStr">
+        <is>
+          <t>Depth: Defines rigorous engineering productivity measurement and influences the field externally. Evidenced by: Makes delivery capability a board-legible asset, benchmarking the org externally and retiring measures that stop informing decisions. Scope: org-wide.</t>
         </is>
       </c>
     </row>
@@ -1466,7 +1532,7 @@
       </c>
       <c r="C14" s="4" t="inlineStr">
         <is>
-          <t>Process Design &amp; Continuous Improvement</t>
+          <t>Process &amp; Continuous Improvement</t>
         </is>
       </c>
       <c r="D14" s="6" t="inlineStr">
@@ -1476,37 +1542,42 @@
       </c>
       <c r="E14" s="4" t="inlineStr">
         <is>
-          <t>Deming, Out of the Crisis (1986)</t>
+          <t>Designing rituals, workflows, and cadences that keep teams effective and aligned.</t>
         </is>
       </c>
       <c r="F14" s="4" t="inlineStr">
         <is>
-          <t>Depth: Designs lightweight processes that make good outcomes repeatable and runs retrospectives that produce changes which stick — the same complaint does not appear three retros running; fixes the actual bottleneck, not everything at once. Scope: one team's system of work.</t>
+          <t>Deming, Out of the Crisis (MIT Center for Advanced Engineering Study, 1986) — improvement comes from acting on the system, not exhorting individuals</t>
         </is>
       </c>
       <c r="G14" s="4" t="inlineStr">
         <is>
-          <t>Depth: Builds robust process and controls for a critical team — reducing variation in quality and delivery while right-sizing governance — and institutionalizes plan-do-study-act learning loops. Scope: a critical team's end-to-end flow.</t>
+          <t>Depth: Runs and tunes a team's operating cadence with normal review. Evidenced by: Runs retrospectives that produce changes which stick, so the same complaint does not appear three retros running. Scope: one team.</t>
         </is>
       </c>
       <c r="H14" s="4" t="inlineStr">
         <is>
-          <t>Depth: Sets consistent process and quality controls across a domain and moves improvements from one team to another with credit given; targets the domain's real constraint so improvement compounds. Scope: a domain; teams volunteer their data.</t>
+          <t>Depth: Independently designs processes that fit the work and removes friction others miss. Evidenced by: Builds robust process for a critical team, reducing variation in quality and delivery while right-sizing governance. Scope: a complex / critical team.</t>
         </is>
       </c>
       <c r="I14" s="4" t="inlineStr">
         <is>
-          <t>Depth: Builds the operations-review rhythm a sub-org trusts — leaders bring their own bad news to it because the response is problem-solving, not punishment; consistency is institutionalized through the leaders who run each team. Scope: a sub-org.</t>
+          <t>Depth: Defines operating-cadence patterns others adopt and fixes broken processes across teams. Evidenced by: Sets consistent process and quality controls across a domain and moves an improvement from one team to another with credit given. Scope: a domain (cross-team).</t>
         </is>
       </c>
       <c r="J14" s="4" t="inlineStr">
         <is>
-          <t>Depth: Sets the function's continuous-improvement strategy and operating-efficiency bar, justifying investments with trend data that survives finance scrutiny. Scope: a function.</t>
+          <t>Depth: Defines operating-cadence patterns others adopt and fixes broken processes across teams. Evidenced by: Builds the operations-review rhythm a sub-org trusts, so leaders bring their own bad news to it. Scope: a sub-org.</t>
         </is>
       </c>
       <c r="K14" s="4" t="inlineStr">
         <is>
-          <t>Depth: Shapes an improvement culture org-wide — process standards, learning loops, and waste elimination that persist because they are cultural, not mandated. Scope: org-wide.</t>
+          <t>Depth: Sets the org's operating model and anticipates where cadence must evolve. Evidenced by: Sets the function's continuous-improvement strategy and operating-efficiency bar, justified with trend data that survives finance scrutiny. Scope: a function.</t>
+        </is>
+      </c>
+      <c r="L14" s="4" t="inlineStr">
+        <is>
+          <t>Depth: Defines effective engineering operating cadence for the discipline and is recognized for it. Evidenced by: Shapes an improvement culture org-wide -- process standards and learning loops that persist because they are cultural, not mandated. Scope: org-wide.</t>
         </is>
       </c>
     </row>
@@ -1533,37 +1604,42 @@
       </c>
       <c r="E15" s="4" t="inlineStr">
         <is>
-          <t>Forsgren et al., The SPACE of Developer Productivity (2021)</t>
+          <t>Build self-service internal platforms and paved paths that streamline delivery.</t>
         </is>
       </c>
       <c r="F15" s="4" t="inlineStr">
         <is>
-          <t>Depth: Removes the team's top friction — flaky CI, slow reviews, meeting load — and measures cycle time before and after. Scope: one team's daily flow.</t>
+          <t>Forsgren, Storey, Maddila, Zimmermann, Houck &amp; Butler, The SPACE of Developer Productivity, ACM Queue 19(1) (2021) — developer productivity is multidimensional, never a single output count, and friction taxes everything</t>
         </is>
       </c>
       <c r="G15" s="4" t="inlineStr">
         <is>
-          <t>Depth: Instruments developer experience on a critical team with surveys plus system metrics and fixes the top pain point each quarter, showing the delta. Scope: a critical team's toolchain and process.</t>
+          <t>Depth: Independently builds and supports standard platform capabilities and templates for routine developer needs with review. Evidenced by: Removes the team's top friction and measures cycle time before and after. Scope: one team.</t>
         </is>
       </c>
       <c r="H15" s="4" t="inlineStr">
         <is>
-          <t>Depth: Prioritizes platform and tooling investment across teams by measured friction, resisting single-metric productivity theater on the record. Scope: a domain's developer platform.</t>
+          <t>Depth: Designs self-service workflows for ambiguous needs, reducing friction and resolving hard abstraction and adoption issues. Evidenced by: Instruments developer experience on a critical team with surveys plus system metrics and fixes the top pain point each quarter. Scope: a complex / critical team.</t>
         </is>
       </c>
       <c r="I15" s="4" t="inlineStr">
         <is>
-          <t>Depth: Builds a developer-experience feedback loop a sub-org acts on quarterly — findings become funded work, and engineers can see it. Scope: a sub-org.</t>
+          <t>Depth: Defines platform architecture and golden paths others adopt, solving deep developer-experience and leverage problems. Evidenced by: Prioritizes platform and tooling investment across teams by measured friction, resisting single-metric productivity theater on the record. Scope: a domain (cross-team).</t>
         </is>
       </c>
       <c r="J15" s="4" t="inlineStr">
         <is>
-          <t>Depth: Makes the function-wide productivity investment case at the executive table with multidimensional evidence, and reports back honestly on what worked. Scope: a function.</t>
+          <t>Depth: Defines platform architecture and golden paths others adopt, solving deep developer-experience and leverage problems. Evidenced by: Builds a developer-experience feedback loop a sub-org acts on quarterly, so findings become funded, visible work. Scope: a sub-org.</t>
         </is>
       </c>
       <c r="K15" s="4" t="inlineStr">
         <is>
-          <t>Depth: Keeps engineering effectiveness a standing strategic priority rather than a slogan; the org budgets for it in bad years too. Scope: org-wide.</t>
+          <t>Depth: Sets organization-wide platform strategy, anticipating how developer-experience engineering should evolve. Evidenced by: Makes the function-wide productivity investment case at the executive table with multidimensional evidence, and reports back honestly on what worked. Scope: a function.</t>
+        </is>
+      </c>
+      <c r="L15" s="4" t="inlineStr">
+        <is>
+          <t>Depth: Defines what excellent platform engineering means for the field, shaping industry developer-experience practice. Evidenced by: Keeps engineering effectiveness a standing strategic priority rather than a slogan; the org budgets for it in bad years too. Scope: org-wide.</t>
         </is>
       </c>
     </row>
@@ -1590,37 +1666,42 @@
       </c>
       <c r="E16" s="4" t="inlineStr">
         <is>
-          <t>Brooks, The Mythical Man-Month (1975)</t>
+          <t>Forecasting staffing needs and allocating people across initiatives and priorities.</t>
         </is>
       </c>
       <c r="F16" s="4" t="inlineStr">
         <is>
-          <t>Depth: Plans the team's quarter against realistic capacity — on-call, ramp time, keep-the-lights-on — and shows the math when asked to take more. Scope: one team's capacity.</t>
+          <t>Brooks, The Mythical Man-Month: Essays on Software Engineering, Anniversary ed. (Addison-Wesley, 1995; orig. 1975) — adding people to a late project makes it later; capacity is nonlinear in headcount</t>
         </is>
       </c>
       <c r="G16" s="4" t="inlineStr">
         <is>
-          <t>Depth: Forecasts capacity across attrition and ramp scenarios, sequencing hiring so the team never lurches between starving and drowning; declines headcount that would slow the team down and says why. Scope: a complex team's pipeline.</t>
+          <t>Depth: Builds a credible headcount plan for one team with normal review. Evidenced by: Plans the team's quarter against realistic capacity and shows the math when asked to take more. Scope: one team.</t>
         </is>
       </c>
       <c r="H16" s="4" t="inlineStr">
         <is>
-          <t>Depth: Models capacity across several teams and proposes moving work or people to where the constraint actually is, with the trade-offs written down. Scope: a domain's capacity allocation.</t>
+          <t>Depth: Independently plans resourcing under uncertainty and defends staffing trade-offs. Evidenced by: Forecasts capacity across attrition and ramp scenarios so the team never lurches between starving and drowning. Scope: a complex / critical team.</t>
         </is>
       </c>
       <c r="I16" s="4" t="inlineStr">
         <is>
-          <t>Depth: Builds the headcount plan a sub-org's budget is built on, defending it line by line and taking cuts strategically rather than spreading them evenly. Scope: a sub-org planning cycle.</t>
+          <t>Depth: Defines resource-planning practices others adopt and resolves cross-team allocation conflicts. Evidenced by: Models capacity across several teams and proposes moving work or people to where the constraint actually is, trade-offs written down. Scope: a domain (cross-team).</t>
         </is>
       </c>
       <c r="J16" s="4" t="inlineStr">
         <is>
-          <t>Depth: Sets the function's location, seniority-mix, and build/contract workforce shape, tying growth to unit economics executives accept. Scope: a function's workforce plan.</t>
+          <t>Depth: Defines resource-planning practices others adopt and resolves cross-team allocation conflicts. Evidenced by: Builds the headcount plan a sub-org's budget is built on, taking cuts strategically rather than spreading them evenly. Scope: a sub-org.</t>
         </is>
       </c>
       <c r="K16" s="4" t="inlineStr">
         <is>
-          <t>Depth: Shapes org-wide workforce strategy across cycles — growing, freezing, or reducing — with the org's long-run capability protected in the plan. Scope: org-wide.</t>
+          <t>Depth: Sets org-wide resourcing strategy and anticipates future capacity demand. Evidenced by: Sets the function's location, seniority-mix, and build/contract workforce shape, tying growth to unit economics executives accept. Scope: a function.</t>
+        </is>
+      </c>
+      <c r="L16" s="4" t="inlineStr">
+        <is>
+          <t>Depth: Defines headcount-planning best practice for the discipline and is recognized for it. Evidenced by: Shapes org-wide workforce strategy across cycles -- growing, freezing, or reducing -- with the org's long-run capability protected. Scope: org-wide.</t>
         </is>
       </c>
     </row>
@@ -1647,37 +1728,42 @@
       </c>
       <c r="E17" s="4" t="inlineStr">
         <is>
-          <t>Korn Ferry Leadership Architect (2014) - Financial Acumen</t>
+          <t>Managing budgets, costs, and external vendor or contractor relationships.</t>
         </is>
       </c>
       <c r="F17" s="4" t="inlineStr">
         <is>
-          <t>Depth: Tracks the team's spend — cloud, tooling, services — and catches anomalies before finance does; makes cost visible on the team's own dashboards. Scope: one team's cost lines.</t>
+          <t>Korn Ferry, Korn Ferry Leadership Architect Global Competency Framework (2014) — engineering leaders are judged on cost lines as well as delivery, and cloud-era spend is an engineering decision</t>
         </is>
       </c>
       <c r="G17" s="4" t="inlineStr">
         <is>
-          <t>Depth: Owns a budget with real variance — forecasts it, explains misses, finds savings that do not damage the roadmap — and negotiates renewals with usage data in hand. Scope: a critical team's budget and vendors.</t>
+          <t>Depth: Manages a team budget and standard vendor relationships with normal review. Evidenced by: Tracks the team's spend and catches anomalies before finance does, making cost visible on the team's own dashboards. Scope: one team.</t>
         </is>
       </c>
       <c r="H17" s="4" t="inlineStr">
         <is>
-          <t>Depth: Finds structural savings across teams — duplicate tooling, idle capacity, overlapping contracts — and lands the consolidation, funding platform work despite feature pressure and defending the split in the open. Scope: domain-level spend.</t>
+          <t>Depth: Independently controls budgets under pressure and negotiates difficult vendor terms. Evidenced by: Owns a budget with real variance, forecasting it and finding savings that do not damage the roadmap. Scope: a complex / critical team.</t>
         </is>
       </c>
       <c r="I17" s="4" t="inlineStr">
         <is>
-          <t>Depth: Runs a full budget cycle for a sub-org, connecting each line to a strategic bet and reallocating mid-year with a rationale the losing team can repeat accurately; kills spend that has outlived its purpose. Scope: a sub-org budget.</t>
+          <t>Depth: Defines budget and vendor practices others adopt and rescues failing vendor relationships. Evidenced by: Finds structural savings across teams -- duplicate tooling, idle capacity, overlapping contracts -- and lands the consolidation. Scope: a domain (cross-team).</t>
         </is>
       </c>
       <c r="J17" s="4" t="inlineStr">
         <is>
-          <t>Depth: Stewards a function's cost structure — unit economics, vendor strategy, location mix — and defends it at the executive and finance table. Scope: a function's economics.</t>
+          <t>Depth: Defines budget and vendor practices others adopt and rescues failing vendor relationships. Evidenced by: Runs a full budget cycle for a sub-org, connecting each line to a strategic bet and reallocating mid-year with a rationale that travels. Scope: a sub-org.</t>
         </is>
       </c>
       <c r="K17" s="4" t="inlineStr">
         <is>
-          <t>Depth: Aligns the org's investment envelope with company strategy and makes its largest financial commitments — deals sized to be existential get diligence sized to match. Scope: org-wide financial exposure.</t>
+          <t>Depth: Sets org-wide budget and vendor strategy and anticipates cost and supplier risks. Evidenced by: Stewards a function's cost structure -- unit economics, vendor strategy, location mix -- and defends it at the executive and finance table. Scope: a function.</t>
+        </is>
+      </c>
+      <c r="L17" s="4" t="inlineStr">
+        <is>
+          <t>Depth: Defines exemplary budget and vendor management for the field and influences practice. Evidenced by: Aligns the org's investment envelope with company strategy and makes its largest financial commitments. Scope: org-wide.</t>
         </is>
       </c>
     </row>
@@ -1704,37 +1790,42 @@
       </c>
       <c r="E18" s="4" t="inlineStr">
         <is>
-          <t>Schmidt &amp; Hunter, selection-methods meta-analysis (1998)</t>
+          <t>Builds the team through hiring and placement.</t>
         </is>
       </c>
       <c r="F18" s="4" t="inlineStr">
         <is>
-          <t>Depth: Runs a structured hiring loop — defined signals per interview, written rubrics, evidence-based debriefs — and closes candidates personally with an honest pitch. Scope: one team's openings.</t>
+          <t>Schmidt &amp; Hunter, The Validity and Utility of Selection Methods in Personnel Psychology, Psychological Bulletin 124(2), 262-274 (1998) — structured interviews and work samples are among the strongest predictors of job performance</t>
         </is>
       </c>
       <c r="G18" s="4" t="inlineStr">
         <is>
-          <t>Depth: Designs the loop itself for senior and hard-to-fill roles — work samples, calibrated rubrics — and defends bar decisions with evidence over gut feel; interviewers they trained staff other loops. Scope: a critical team's talent needs and beyond.</t>
+          <t>Depth: Shapes hiring for a team; designs loops; makes sound staffing calls. Evidenced by: Runs a structured hiring loop with defined signals per interview and evidence-based debriefs, and closes candidates personally. Scope: one team.</t>
         </is>
       </c>
       <c r="H18" s="4" t="inlineStr">
         <is>
-          <t>Depth: Sets the hiring bar across a domain — rubric library, debrief standards, a bar-raiser bench — so teams they do not run make comparable decisions; makes calibration visible with data like pass-through rates and first-year outcomes. Scope: cross-team hiring quality.</t>
+          <t>Depth: Shapes hiring for a team; designs loops; makes sound staffing calls. Evidenced by: Designs the loop itself for senior and hard-to-fill roles and defends bar decisions with evidence over gut feel. Scope: a complex / critical team.</t>
         </is>
       </c>
       <c r="I18" s="4" t="inlineStr">
         <is>
-          <t>Depth: Builds the hiring machinery a sub-org hires through — interviewer training, bar-raiser pools, leveling guides, sourcing strategy — and personally closes the hires that change a trajectory. Scope: a sub-org's pipeline.</t>
+          <t>Depth: Drives hiring strategy across teams; builds the interviewing bar. Evidenced by: Sets the hiring bar across a domain -- rubric library, debrief standards, a bar-raiser bench -- so teams they do not run make comparable decisions. Scope: a domain (cross-team).</t>
         </is>
       </c>
       <c r="J18" s="4" t="inlineStr">
         <is>
-          <t>Depth: Sets the function's talent-acquisition strategy — where to compete for people and on what basis — with recruiting and finance partners, holding the bar under growth pressure. Scope: a function's brand and bar.</t>
+          <t>Depth: Drives hiring strategy across teams; builds the interviewing bar. Evidenced by: Builds the hiring machinery a sub-org hires through -- interviewer training, bar-raiser pools, leveling guides, sourcing strategy. Scope: a sub-org.</t>
         </is>
       </c>
       <c r="K18" s="4" t="inlineStr">
         <is>
-          <t>Depth: Makes the org a destination for the people it most needs — visible externally, credible internally — and personally recruits the leadership that changes the company's capability. Scope: org-wide talent brand.</t>
+          <t>Depth: Sets the org's talent strategy. Evidenced by: Sets the function's talent-acquisition strategy -- where to compete for people and on what basis -- holding the bar under growth pressure. Scope: a function.</t>
+        </is>
+      </c>
+      <c r="L18" s="4" t="inlineStr">
+        <is>
+          <t>Depth: Shapes company-wide talent philosophy. Evidenced by: Makes the org a destination for the people it most needs, and personally recruits the leadership that changes its capability. Scope: org-wide.</t>
         </is>
       </c>
     </row>
@@ -1761,37 +1852,42 @@
       </c>
       <c r="E19" s="4" t="inlineStr">
         <is>
-          <t>Tuckman, Developmental Sequence in Small Groups (1965)</t>
+          <t>Ramps new people to productivity fast and leads teams through formation stages — launches, merges, and resets — deliberately rather than enduring them.</t>
         </is>
       </c>
       <c r="F19" s="4" t="inlineStr">
         <is>
-          <t>Depth: Runs a 30/60/90 onboarding with named buddies and early wins; new hires ship in their first weeks and say so in check-ins. Scope: one team's ramp.</t>
+          <t>Tuckman, Developmental Sequence in Small Groups, Psychological Bulletin 63(6), 384-399 (1965) — teams predictably move through forming, storming, norming, and performing, and leaders can shorten the trough</t>
         </is>
       </c>
       <c r="G19" s="4" t="inlineStr">
         <is>
-          <t>Depth: Reads a team's formation stage and intervenes on it — resets norms after a merge, names storming in the room instead of managing it by email. Scope: a critical team through churn and growth.</t>
+          <t>Depth: Runs a 30/60/90 onboarding with named buddies and early wins; new hires ship in their first weeks and say so in check-ins. Scope: one team.</t>
         </is>
       </c>
       <c r="H19" s="4" t="inlineStr">
         <is>
-          <t>Depth: Builds the onboarding and team-launch playbook a domain uses; teams they do not run start faster because of materials and rituals they created. Scope: cross-team.</t>
+          <t>Depth: Reads a team's formation stage and intervenes on it — resets norms after a merge, names storming in the room instead of managing it by email. Scope: a complex / critical team.</t>
         </is>
       </c>
       <c r="I19" s="4" t="inlineStr">
         <is>
-          <t>Depth: Stands up whole new teams — mission, first hires, norms, interfaces — repeatedly, and coaches leaders through their first team formations. Scope: a sub-org's growth mechanics.</t>
+          <t>Depth: Builds the onboarding and team-launch playbook multiple teams use; teams start faster because of materials and rituals they created, and stands up whole new teams repeatedly. Evidenced by: Cuts a domain's median time-to-first-contribution with a ramp template teams outside their own org start copying unprompted. Scope: a domain (cross-team).</t>
         </is>
       </c>
       <c r="J19" s="4" t="inlineStr">
         <is>
-          <t>Depth: Designs how a function absorbs step-change growth — acquisitions, new sites, doubled headcount — without culture dilution; integration plans carry named cultural mechanisms. Scope: a function.</t>
+          <t>Depth: Builds the onboarding and team-launch playbook multiple teams use; teams start faster because of materials and rituals they created, and stands up whole new teams repeatedly. Evidenced by: Stands up whole new teams -- mission, first hires, norms, interfaces -- repeatedly, and coaches leaders through their first team formations. Scope: a sub-org.</t>
         </is>
       </c>
       <c r="K19" s="4" t="inlineStr">
         <is>
-          <t>Depth: Makes team formation an org-wide capability — the org spins up new groups predictably without heroics — and audits that the machinery still works. Scope: org-wide.</t>
+          <t>Depth: Designs how an organization absorbs step-change growth — acquisitions, new sites, doubled headcount — without culture dilution; integration plans carry named cultural mechanisms. Evidenced by: Runs an acquired team through its first 90 days without losing a person to the culture clash that sank the last integration. Scope: a function.</t>
+        </is>
+      </c>
+      <c r="L19" s="4" t="inlineStr">
+        <is>
+          <t>Depth: Makes team formation an organization-wide capability — new groups spin up predictably without heroics — and audits that the machinery still works. Evidenced by: Audits the org's team-formation machinery on a cadence and finds -- and fixes -- the playbook step that quietly stopped working two reorgs ago. Scope: org-wide.</t>
         </is>
       </c>
     </row>
@@ -1818,37 +1914,42 @@
       </c>
       <c r="E20" s="4" t="inlineStr">
         <is>
-          <t>Whitmore, Coaching for Performance (1992); Google Project Oxygen</t>
+          <t>Grows other people's capability.</t>
         </is>
       </c>
       <c r="F20" s="4" t="inlineStr">
         <is>
-          <t>Depth: Holds weekly one-on-ones that are coaching conversations, not status reads — asks before advising; each person has a live growth plan they co-wrote. Scope: every individual on one team.</t>
+          <t>Whitmore, Coaching for Performance: GROWing Human Potential and Purpose, 4th ed. (Nicholas Brealey, 2009; orig. 1992) — regular coaching, not status-checking, is the top driver of manager effectiveness</t>
         </is>
       </c>
       <c r="G20" s="4" t="inlineStr">
         <is>
-          <t>Depth: Coaches senior engineers and first-time leads through ambiguity they cannot solve for them — scoping staff-level work, brokering visibility — and is sought out as a coach beyond the team. Scope: a critical team's senior bench.</t>
+          <t>Depth: Coaches engineers with growth-oriented feedback; measurably improves a team's skill. Evidenced by: Holds one-on-ones that are coaching conversations, not status reads -- each person has a live growth plan they co-wrote. Scope: one team.</t>
         </is>
       </c>
       <c r="H20" s="4" t="inlineStr">
         <is>
-          <t>Depth: Coaches other people-leads on their coaching — sits in on their reviews on request; leaders demonstrably improve their practice after working with them, and people across the domain cite their questions as the turning point. Scope: cross-team leadership bench.</t>
+          <t>Depth: Coaches engineers with growth-oriented feedback; measurably improves a team's skill. Evidenced by: Coaches senior engineers and first-time leads through ambiguity they cannot solve for them, and is sought out as a coach beyond the team. Scope: a complex / critical team.</t>
         </is>
       </c>
       <c r="I20" s="4" t="inlineStr">
         <is>
-          <t>Depth: Builds coaching capability at scale — manager forums, feedback training, calibration on what good coaching looks like — that a sub-org adopts and keeps running without them. Scope: a sub-org.</t>
+          <t>Depth: Develops future leads across teams; shapes hiring and onboarding. Evidenced by: Coaches other people-leads on their coaching, sitting in on their reviews on request; leaders demonstrably improve after working with them. Scope: a domain (cross-team).</t>
         </is>
       </c>
       <c r="J20" s="4" t="inlineStr">
         <is>
-          <t>Depth: Develops senior leaders across a function, including peers who seek their counsel, and sponsors development systems rather than only coaching personally. Scope: a function's leadership pipeline.</t>
+          <t>Depth: Develops future leads across teams; shapes hiring and onboarding. Evidenced by: Builds coaching capability at scale -- manager forums, calibration on what good coaching looks like -- that a sub-org adopts and keeps running. Scope: a sub-org.</t>
         </is>
       </c>
       <c r="K20" s="4" t="inlineStr">
         <is>
-          <t>Depth: Sets the org-wide philosophy and systems for talent growth, and the org's leaders visibly coach because the top does. Scope: org-wide leadership culture.</t>
+          <t>Depth: Develops senior engineers and leaders; builds culture deliberately. Evidenced by: Develops senior leaders across a function, including peers who seek their counsel, and sponsors development systems rather than only coaching personally. Scope: a function.</t>
+        </is>
+      </c>
+      <c r="L20" s="4" t="inlineStr">
+        <is>
+          <t>Depth: Develops the next generation of top talent; legacy outlasts tenure. Evidenced by: Sets the org-wide philosophy and systems for talent growth; the org's leaders visibly coach because the top does. Scope: org-wide.</t>
         </is>
       </c>
     </row>
@@ -1875,37 +1976,42 @@
       </c>
       <c r="E21" s="4" t="inlineStr">
         <is>
-          <t>Scott, Radical Candor (2017); SBI model (CCL)</t>
+          <t>Gives and receives honest, useful feedback.</t>
         </is>
       </c>
       <c r="F21" s="4" t="inlineStr">
         <is>
-          <t>Depth: Gives specific, behavior-anchored feedback within days — kind and clear, not brutal or vague — and listens to understand, soliciting dissent; feedback flows both directions in their one-on-ones. Scope: one team.</t>
+          <t>Scott, Radical Candor: Be a Kick-Ass Boss Without Losing Your Humanity (St. Martin's Press, 2017) — caring personally while challenging directly beats both ruinous empathy and obnoxious aggression</t>
         </is>
       </c>
       <c r="G21" s="4" t="inlineStr">
         <is>
-          <t>Depth: Creates feedback-rich norms on a complex team and handles the hardest feedback conversations well — hears what is not said, and turns hard feedback into changed behavior within weeks. Scope: a critical team.</t>
+          <t>Depth: Gives growth-oriented feedback that changes behavior; coaches through feedback. Evidenced by: Gives specific, behavior-anchored feedback within days, and listens to understand by soliciting dissent in one-on-ones. Scope: one team.</t>
         </is>
       </c>
       <c r="H21" s="4" t="inlineStr">
         <is>
-          <t>Depth: Builds a candor culture across a domain — models seeking and acting on critical feedback at scale, setting feedback norms teams they do not run follow. Scope: cross-team norms.</t>
+          <t>Depth: Gives growth-oriented feedback that changes behavior; coaches through feedback. Evidenced by: Creates feedback-rich norms on a complex team and turns hard feedback into changed behavior within weeks. Scope: a complex / critical team.</t>
         </is>
       </c>
       <c r="I21" s="4" t="inlineStr">
         <is>
-          <t>Depth: Institutionalizes feedback norms across a sub-org through mechanisms — training, calibration on feedback quality — that outlast their attention. Scope: a sub-org.</t>
+          <t>Depth: Builds feedback norms that raise the bar across teams. Evidenced by: Builds a candor culture across a domain, setting feedback norms teams they do not run follow. Scope: a domain (cross-team).</t>
         </is>
       </c>
       <c r="J21" s="4" t="inlineStr">
         <is>
-          <t>Depth: Coaches at the executive seam — peers and senior leaders take their feedback on leadership behavior, delivered candidly and in private. Scope: a function's leadership.</t>
+          <t>Depth: Builds feedback norms that raise the bar across teams. Evidenced by: Institutionalizes feedback norms across a sub-org through training and calibration mechanisms that outlast their attention. Scope: a sub-org.</t>
         </is>
       </c>
       <c r="K21" s="4" t="inlineStr">
         <is>
-          <t>Depth: Models candor at the top — publicly requests, receives, and acts on hard feedback; the org's norms of directness trace to their visible example. Scope: org-wide.</t>
+          <t>Depth: Sets the org's culture of candor and growth. Evidenced by: Coaches at the executive seam -- peers and senior leaders take their feedback on leadership behavior, delivered candidly and in private. Scope: a function.</t>
+        </is>
+      </c>
+      <c r="L21" s="4" t="inlineStr">
+        <is>
+          <t>Depth: Models and defines feedback culture company-wide. Evidenced by: Models candor at the top -- publicly requests, receives, and acts on hard feedback -- and the org's norms of directness trace to it. Scope: org-wide.</t>
         </is>
       </c>
     </row>
@@ -1932,37 +2038,42 @@
       </c>
       <c r="E22" s="4" t="inlineStr">
         <is>
-          <t>Grove, High Output Management (1983)</t>
+          <t>Setting expectations, evaluating performance, and addressing under-performance fairly and clearly.</t>
         </is>
       </c>
       <c r="F22" s="4" t="inlineStr">
         <is>
-          <t>Depth: Sets explicit expectations per person and level, documents evidence continuously, and delivers reviews with no surprises — underperformance is named early with a concrete support plan. Scope: their direct team.</t>
+          <t>Grove, High Output Management (Random House, 1983) — a manager's output is the team's output, so managing performance is the core lever</t>
         </is>
       </c>
       <c r="G22" s="4" t="inlineStr">
         <is>
-          <t>Depth: Handles the hard cases — brilliant-but-corrosive, long-tenured-but-plateaued — with documented, humane processes that end in change or exit inside a quarter or two, and writes promotion cases that survive committee. Scope: a critical team's full performance range.</t>
+          <t>Depth: Independently manages underperformance and difficult cases through to clear resolution. Evidenced by: Addresses an underperforming report directly with a documented, humane plan rather than letting it drift. Scope: one team.</t>
         </is>
       </c>
       <c r="H22" s="4" t="inlineStr">
         <is>
-          <t>Depth: Runs calibration across teams so the same work earns the same rating regardless of manager, contesting both inflation and harshness with specifics; coaches managers they do not oversee through their first improvement plans. Scope: cross-team fairness.</t>
+          <t>Depth: Independently manages underperformance and difficult cases through to clear resolution. Evidenced by: Handles the hard cases -- brilliant-but-corrosive, long-tenured-but-plateaued -- with documented processes that end in change or exit inside a quarter or two. Scope: a complex / critical team.</t>
         </is>
       </c>
       <c r="I22" s="4" t="inlineStr">
         <is>
-          <t>Depth: Designs a sub-org's performance system — rubrics, promotion bars, calibration protocols, appeal paths — and audits its outcomes for drift and bias; hard calls happen earlier because the system backs the people making them. Scope: a sub-org.</t>
+          <t>Depth: Defines accountability practices other managers adopt and coaches them through hard cases. Evidenced by: Runs calibration across teams so the same work earns the same rating regardless of manager, contesting both inflation and harshness. Scope: a domain (cross-team).</t>
         </is>
       </c>
       <c r="J22" s="4" t="inlineStr">
         <is>
-          <t>Depth: Holds senior leaders to the same standard as everyone else — visibly acts on underperformance at high levels, where the cost of avoidance is largest. Scope: a function's leadership accountability.</t>
+          <t>Depth: Defines accountability practices other managers adopt and coaches them through hard cases. Evidenced by: Designs a sub-org's performance system and audits its outcomes for drift and bias, so hard calls happen earlier. Scope: a sub-org.</t>
         </is>
       </c>
       <c r="K22" s="4" t="inlineStr">
         <is>
-          <t>Depth: Sets the org's performance philosophy — what is rewarded, tolerated, and exited — and applies it to the most senior and most protected people first. Scope: org-wide standards.</t>
+          <t>Depth: Sets the org's performance philosophy and anticipates systemic accountability gaps. Evidenced by: Holds senior leaders to the same standard as everyone else, visibly acting on underperformance at high levels. Scope: a function.</t>
+        </is>
+      </c>
+      <c r="L22" s="4" t="inlineStr">
+        <is>
+          <t>Depth: Defines what fair, effective performance management means and influences the field externally. Evidenced by: Sets the org's performance philosophy -- what is rewarded, tolerated, and exited -- applying it to the most senior people first. Scope: org-wide.</t>
         </is>
       </c>
     </row>
@@ -1989,37 +2100,42 @@
       </c>
       <c r="E23" s="4" t="inlineStr">
         <is>
-          <t>Hewlett, Forget a Mentor, Find a Sponsor (2013)</t>
+          <t>Growing engineers through development plans, advancement opportunities, and active sponsorship.</t>
         </is>
       </c>
       <c r="F23" s="4" t="inlineStr">
         <is>
-          <t>Depth: Knows each person's aspirations, creates stretch scope, and gives honest promotion guidance; sponsors deserving people in calibration rather than just advising them. Scope: one team's careers.</t>
+          <t>Hewlett, Forget a Mentor, Find a Sponsor: The New Way to Fast-Track Your Career (Harvard Business Review Press, 2013) — sponsorship -- spending capital on stretch, visibility, advocacy -- moves careers where mentoring alone does not</t>
         </is>
       </c>
       <c r="G23" s="4" t="inlineStr">
         <is>
-          <t>Depth: Sponsors people into senior and lead roles — writes compelling cases and spends real capital advocating beyond their own team. Scope: a critical team's senior transitions.</t>
+          <t>Depth: Coaches direct reports on standard career growth with normal review. Evidenced by: Knows each person's aspirations, creates stretch scope, and gives honest promotion guidance. Scope: one team.</t>
         </is>
       </c>
       <c r="H23" s="4" t="inlineStr">
         <is>
-          <t>Depth: Owns fair, consistent advancement across a domain, sponsoring senior ICs and emerging leaders into scope they would not get alone. Scope: cross-team advancement.</t>
+          <t>Depth: Independently sponsors people into stretch roles and navigates complex growth paths. Evidenced by: Sponsors people into senior and lead roles, writing compelling cases and spending real capital advocating beyond the team. Scope: a complex / critical team.</t>
         </is>
       </c>
       <c r="I23" s="4" t="inlineStr">
         <is>
-          <t>Depth: Builds career-path and recognition systems a sub-org adopts, so growth does not require leaving, and audits promotion rates by cohort for equity. Scope: a sub-org.</t>
+          <t>Depth: Defines career-development practices others adopt and unblocks the toughest growth cases. Evidenced by: Owns fair, consistent advancement across a domain, sponsoring senior ICs and emerging leaders into scope they would not get alone. Scope: a domain (cross-team).</t>
         </is>
       </c>
       <c r="J23" s="4" t="inlineStr">
         <is>
-          <t>Depth: Shapes the function's leveling and advancement architecture with people-team partners, sponsoring high-potential leaders into visibility before vacancies force it. Scope: a function.</t>
+          <t>Depth: Defines career-development practices others adopt and unblocks the toughest growth cases. Evidenced by: Builds career-path and recognition systems a sub-org adopts, so growth does not require leaving, and audits promotion rates by cohort. Scope: a sub-org.</t>
         </is>
       </c>
       <c r="K23" s="4" t="inlineStr">
         <is>
-          <t>Depth: Shapes advancement systems org-wide; the org's promotion decisions still mean something years later, and its leaders credit named sponsorship. Scope: org-wide.</t>
+          <t>Depth: Sets the org's talent-development strategy and anticipates future capability needs. Evidenced by: Shapes the function's leveling and advancement architecture, sponsoring high-potential leaders into visibility before vacancies force it. Scope: a function.</t>
+        </is>
+      </c>
+      <c r="L23" s="4" t="inlineStr">
+        <is>
+          <t>Depth: Defines exemplary career sponsorship for the discipline and is externally recognized for it. Evidenced by: Shapes advancement systems org-wide; the org's promotion decisions still mean something years later. Scope: org-wide.</t>
         </is>
       </c>
     </row>
@@ -2046,37 +2162,42 @@
       </c>
       <c r="E24" s="4" t="inlineStr">
         <is>
-          <t>Charan, Drotter &amp; Noel, The Leadership Pipeline (2001)</t>
+          <t>Owns frameworks for identifying, developing, and retaining critical and high-potential talent.</t>
         </is>
       </c>
       <c r="F24" s="4" t="inlineStr">
         <is>
-          <t>Depth: Names their own successor risk and grows a deputy — delegating real ownership as development, not offloading; someone can cover their vacation without incident. Scope: one team's bench.</t>
+          <t>Charan, Drotter &amp; Noel, The Leadership Pipeline: How to Build the Leadership-Powered Company, 2nd Edition (Jossey-Bass, 2010) — each leadership passage requires new skills and values, so benches must be built deliberately</t>
         </is>
       </c>
       <c r="G24" s="4" t="inlineStr">
         <is>
-          <t>Depth: Builds bench depth on purpose — tech-lead rotations, stretch scopes with safety nets — so the team survives its strongest engineer's departure; people they grew succeed after moving elsewhere, and say so. Scope: a critical team as a leadership incubator.</t>
+          <t>Depth: Runs standard talent-review and succession cycles independently for defined populations. Evidenced by: Names their own successor risk and grows a deputy -- delegating real ownership as development, not offloading. Scope: one team.</t>
         </is>
       </c>
       <c r="H24" s="4" t="inlineStr">
         <is>
-          <t>Depth: Maintains a live succession slate for every key seat in a domain and exports leaders to other parts of the org rather than hoarding them. Scope: a domain's bench.</t>
+          <t>Depth: Designs succession approaches for critical, ambiguous roles and resolves contested talent calls. Evidenced by: Builds bench depth on purpose -- tech-lead rotations, stretch scopes with safety nets -- so the team survives its strongest engineer's departure. Scope: a complex / critical team.</t>
         </is>
       </c>
       <c r="I24" s="4" t="inlineStr">
         <is>
-          <t>Depth: Runs talent reviews that end in moves — promotions, rotations, exits — not just ratings, and builds development mechanisms like acting-role assignments a sub-org adopts. Scope: sub-org pipeline health.</t>
+          <t>Depth: Defines talent-management and succession frameworks that other practitioners adopt. Evidenced by: Maintains a live succession slate for every key seat in a domain and exports leaders to other parts of the org rather than hoarding them. Scope: a domain (cross-team).</t>
         </is>
       </c>
       <c r="J24" s="4" t="inlineStr">
         <is>
-          <t>Depth: Ensures every critical role in the function has a named, developing successor, reviewing succession with executives before vacancies force it. Scope: a function.</t>
+          <t>Depth: Defines talent-management and succession frameworks that other practitioners adopt. Evidenced by: Runs talent reviews that end in moves, not just ratings, and builds acting-role development mechanisms a sub-org adopts. Scope: a sub-org.</t>
         </is>
       </c>
       <c r="K24" s="4" t="inlineStr">
         <is>
-          <t>Depth: Builds the pipeline the org promotes from, including the bench for the top jobs and their own; top seats fill internally more often than not. Scope: org-wide.</t>
+          <t>Depth: Sets enterprise succession strategy and anticipates future leadership and capability gaps. Evidenced by: Ensures every critical role in the function has a named, developing successor, reviewed with executives before vacancies force it. Scope: a function.</t>
+        </is>
+      </c>
+      <c r="L24" s="4" t="inlineStr">
+        <is>
+          <t>Depth: Defines leading practice for talent management and succession across the profession. Evidenced by: Builds the pipeline the org promotes from, including the bench for the top jobs and their own. Scope: org-wide.</t>
         </is>
       </c>
     </row>
@@ -2103,37 +2224,42 @@
       </c>
       <c r="E25" s="4" t="inlineStr">
         <is>
-          <t>Edmondson, The Fearless Organization (2018); Project Aristotle</t>
+          <t>Creates the conditions where people raise problems, dissent, and admit mistakes without penalty; reads and repairs team-health signals (conflict, burnout risk, on-call load).</t>
         </is>
       </c>
       <c r="F25" s="4" t="inlineStr">
         <is>
-          <t>Depth: Responds to bad news by thanking the messenger and models fallibility — says "I was wrong" in front of the team; the quietest person speaks in their meetings, and interruption and ridicule get shut down on the spot. Scope: one team's meetings and channels.</t>
+          <t>Edmondson, The Fearless Organization: Creating Psychological Safety in the Workplace for Learning, Innovation, and Growth (Wiley, 2018) — psychological safety is the top predictor of team effectiveness, and every other team behavior depends on it</t>
         </is>
       </c>
       <c r="G25" s="4" t="inlineStr">
         <is>
-          <t>Depth: Rebuilds safety where it is damaged — post-incident, post-layoff, post-conflict — measurably; dissent shows up in decision records again, and dissenters are visibly protected from consequences. Scope: a critical team under pressure.</t>
+          <t>Depth: Sustains safety through pressure (incidents, deadlines, change); repairs damaged trust; the team measurably speaks up (postmortems name real causes). Evidenced by: Responds to bad news by thanking the messenger and models fallibility, saying 'I was wrong' in front of the team under real pressure. Scope: one team.</t>
         </is>
       </c>
       <c r="H25" s="4" t="inlineStr">
         <is>
-          <t>Depth: Reads safety across teams from signals — who speaks in reviews, what surfaces in retros versus hallways — and coaches the leads whose teams have gone quiet; runs pre-mortems and challenge sessions others adopt. Scope: a domain's speak-up climate.</t>
+          <t>Depth: Sustains safety through pressure (incidents, deadlines, change); repairs damaged trust; the team measurably speaks up (postmortems name real causes). Evidenced by: Rebuilds safety where it is damaged post-incident or post-conflict; dissenters are visibly protected from consequences. Scope: a complex / critical team.</t>
         </is>
       </c>
       <c r="I25" s="4" t="inlineStr">
         <is>
-          <t>Depth: Builds channels through which bad news travels up fast — skip-levels, anonymous paths, incident amnesty — and proves they are safe by what happens to the people who use them. Scope: a sub-org's information flow.</t>
+          <t>Depth: Diagnoses and fixes systemic safety failures across teams; other leaders seek their help on entrenched conflict and burnout patterns. Evidenced by: Reads safety across teams from signals -- who speaks in reviews, what surfaces in retros versus hallways -- and coaches the leads whose teams have gone quiet. Scope: a domain (cross-team).</t>
         </is>
       </c>
       <c r="J25" s="4" t="inlineStr">
         <is>
-          <t>Depth: Makes dissent safe in executive rooms — invites challenge to their own proposals in front of others and rewards the challengers; kills shoot-the-messenger behavior among senior leaders where it happens. Scope: a function's leadership culture.</t>
+          <t>Depth: Diagnoses and fixes systemic safety failures across teams; other leaders seek their help on entrenched conflict and burnout patterns. Evidenced by: Builds channels through which bad news travels up fast -- skip-levels, anonymous paths, incident amnesty -- and proves they are safe. Scope: a sub-org.</t>
         </is>
       </c>
       <c r="K25" s="4" t="inlineStr">
         <is>
-          <t>Depth: Makes it safe to tell the org's most powerful people they are wrong — including themselves, publicly; the org's biggest failures produce learning documents, not scapegoats. Scope: org-wide culture.</t>
+          <t>Depth: Sets the org's team-health bar and mechanisms; safety practices they designed are adopted org-wide. Evidenced by: Makes dissent safe in executive rooms, inviting challenge to their own proposals and rewarding the challengers. Scope: a function.</t>
+        </is>
+      </c>
+      <c r="L25" s="4" t="inlineStr">
+        <is>
+          <t>Depth: Shapes how the industry thinks about team health; published practices others implement. Evidenced by: Makes it safe to tell the org's most powerful people they are wrong, including themselves, publicly. Scope: org-wide.</t>
         </is>
       </c>
     </row>
@@ -2160,37 +2286,42 @@
       </c>
       <c r="E26" s="4" t="inlineStr">
         <is>
-          <t>Deci &amp; Ryan, Self-Determination Theory (2000); Herzberg (1968)</t>
+          <t>Builds durable intrinsic motivation: removes dissatisfiers, feeds autonomy/mastery/purpose, recognizes well.</t>
         </is>
       </c>
       <c r="F26" s="4" t="inlineStr">
         <is>
-          <t>Depth: Knows what motivates each person and matches work to it — removing dissatisfiers and feeding autonomy, mastery, and purpose; catches disengagement in work patterns before the survey does, and regrettable attrition is rare and predicted. Scope: one team.</t>
+          <t>Deci &amp; Ryan, The "What" and "Why" of Goal Pursuits: Human Needs and the Self-Determination of Behavior, Psychological Inquiry 11(4), 227-268 (2000) — autonomy, mastery, and purpose drive durable engagement more than extrinsic rewards</t>
         </is>
       </c>
       <c r="G26" s="4" t="inlineStr">
         <is>
-          <t>Depth: Keeps a critical team engaged through grind — long migrations, incident sieges — by restoring autonomy and purpose where they have eroded; re-recruits key people proactively, before the resignation letter. Scope: a high-pressure team.</t>
+          <t>Depth: Sustains engagement through hard stretches; diagnoses systemic motivation problems (not just individuals) and fixes the conditions. Evidenced by: Catches disengagement across the whole team's morale during a demanding stretch, and fixes the driving condition rather than giving one-off pep talks. Scope: one team.</t>
         </is>
       </c>
       <c r="H26" s="4" t="inlineStr">
         <is>
-          <t>Depth: Reads attrition and engagement patterns across teams and fixes the systemic causes — career stagnation, meaningless work — not the symptoms; managers across the domain apply the playbook to their own teams. Scope: cross-team engagement.</t>
+          <t>Depth: Sustains engagement through hard stretches; diagnoses systemic motivation problems (not just individuals) and fixes the conditions. Evidenced by: Keeps a critical team engaged through grind by restoring autonomy and purpose where they have eroded, re-recruiting key people proactively. Scope: a complex / critical team.</t>
         </is>
       </c>
       <c r="I26" s="4" t="inlineStr">
         <is>
-          <t>Depth: Builds the conditions of motivation into a sub-org's operating model — team autonomy, mastery paths, recognition systems — and measures their effect rather than their activity. Scope: a sub-org.</t>
+          <t>Depth: Builds engagement mechanisms other teams adopt; reverses disengagement trends beyond their own span. Evidenced by: Reads attrition and engagement patterns across teams and fixes the systemic causes; managers across the domain apply the playbook to their own teams. Scope: a domain (cross-team).</t>
         </is>
       </c>
       <c r="J26" s="4" t="inlineStr">
         <is>
-          <t>Depth: Acts publicly on function-level engagement results — survey outcomes drive visible changes, and tells executives the truth when money is masking a meaning problem. Scope: a function.</t>
+          <t>Depth: Builds engagement mechanisms other teams adopt; reverses disengagement trends beyond their own span. Evidenced by: Builds the conditions of motivation into a sub-org's operating model and measures their effect rather than their activity. Scope: a sub-org.</t>
         </is>
       </c>
       <c r="K26" s="4" t="inlineStr">
         <is>
-          <t>Depth: Builds an employee value proposition people join and stay for — the story engineers tell friends is the one leadership tells — with regrettable attrition of critical people treated as a serious incident. Scope: org-wide.</t>
+          <t>Depth: Owns the engagement strategy for a function; conditions they designed show up in retention and survey trends. Evidenced by: Acts publicly on function-level engagement results, and tells executives the truth when money is masking a meaning problem. Scope: a function.</t>
+        </is>
+      </c>
+      <c r="L26" s="4" t="inlineStr">
+        <is>
+          <t>Depth: Advances the practice of engagement in the field; frameworks others cite and use. Evidenced by: Builds an employee value proposition people join and stay for; regrettable attrition of critical people is treated as a serious incident. Scope: org-wide.</t>
         </is>
       </c>
     </row>
@@ -2217,37 +2348,42 @@
       </c>
       <c r="E27" s="4" t="inlineStr">
         <is>
-          <t>Ely &amp; Thomas, Cultural Diversity at Work (2001)</t>
+          <t>Runs diversity, equity, and inclusion strategy, programs, and accountability measures.</t>
         </is>
       </c>
       <c r="F27" s="4" t="inlineStr">
         <is>
-          <t>Depth: Runs inclusive meetings and decisions — every voice heard, bias mitigated in hiring and reviews; airtime and credit are tracked, not assumed. Scope: one team.</t>
+          <t>Hunt, Prince, Dixon-Fyle &amp; Yee, Diversity Wins: How Inclusion Matters (McKinsey &amp; Company, 2020) — diverse teams outperform only under an integration-and-learning climate where people belong and can contribute</t>
         </is>
       </c>
       <c r="G27" s="4" t="inlineStr">
         <is>
-          <t>Depth: Builds inclusion into a critical team's norms and senior-IC growth — closes equity gaps in scope and visibility and mentors others in inclusive leadership. Scope: a critical team.</t>
+          <t>Depth: Runs standard DEI programs independently and tracks routine progress measures. Evidenced by: Runs inclusive meetings and decisions -- every voice heard, bias mitigated in hiring and reviews -- with airtime and credit tracked, not assumed. Scope: one team.</t>
         </is>
       </c>
       <c r="H27" s="4" t="inlineStr">
         <is>
-          <t>Depth: Owns inclusive practice and equitable outcomes across a domain — addresses systemic barriers and builds diverse pipelines; promotion and pay patterns are audited, not assumed. Scope: cross-team.</t>
+          <t>Depth: Designs DEI interventions for complex, sensitive challenges under significant ambiguity. Evidenced by: Builds inclusion into a critical team's norms and senior-IC growth, closing equity gaps in scope and visibility. Scope: a complex / critical team.</t>
         </is>
       </c>
       <c r="I27" s="4" t="inlineStr">
         <is>
-          <t>Depth: Builds inclusion mechanisms — meeting norms, promotion audits, pay-equity checks — that a sub-org adopts and reports on. Scope: a sub-org.</t>
+          <t>Depth: Defines DEI program frameworks and measurement approaches that other practitioners adopt. Evidenced by: Owns inclusive practice and equitable outcomes across a domain, addressing systemic barriers and auditing promotion and pay patterns. Scope: a domain (cross-team).</t>
         </is>
       </c>
       <c r="J27" s="4" t="inlineStr">
         <is>
-          <t>Depth: Sets inclusion strategy and accountability for a function, intervening on systemic patterns rather than the loudest case. Scope: a function.</t>
+          <t>Depth: Defines DEI program frameworks and measurement approaches that other practitioners adopt. Evidenced by: Builds inclusion mechanisms -- meeting norms, promotion audits, pay-equity checks -- that a sub-org adopts and reports on. Scope: a sub-org.</t>
         </is>
       </c>
       <c r="K27" s="4" t="inlineStr">
         <is>
-          <t>Depth: Champions an inclusive culture org-wide — the org's belonging outcomes are measured, published, and owned at the top. Scope: org-wide.</t>
+          <t>Depth: Sets enterprise DEI strategy and anticipates shifts in equity expectations and regulation. Evidenced by: Sets inclusion strategy and accountability for a function, intervening on systemic patterns rather than the loudest case. Scope: a function.</t>
+        </is>
+      </c>
+      <c r="L27" s="4" t="inlineStr">
+        <is>
+          <t>Depth: Pioneers DEI practice recognized externally as authoritative across the field. Evidenced by: Champions an inclusive culture org-wide; the org's belonging outcomes are measured, published, and owned at the top. Scope: org-wide.</t>
         </is>
       </c>
     </row>
@@ -2274,37 +2410,42 @@
       </c>
       <c r="E28" s="4" t="inlineStr">
         <is>
-          <t>Majors, The Engineer/Manager Pendulum (2017); Fournier (2017)</t>
+          <t>Retains enough hands-on technical depth to earn engineers' trust, ask the questions that change designs, and judge technical work without doing it.</t>
         </is>
       </c>
       <c r="F28" s="4" t="inlineStr">
         <is>
-          <t>Depth: Understands the team's systems well enough to review designs, probe trade-offs, and triage incidents — earns technical respect without taking the keyboard. Scope: one team's systems.</t>
+          <t>Fournier, The Manager's Path (O'Reilly, 2017) — a manager who cannot evaluate technical work loses the team's trust and cannot coach staff engineers</t>
         </is>
       </c>
       <c r="G28" s="4" t="inlineStr">
         <is>
-          <t>Depth: Maintains depth across a critical system's stack and hardest problems — a credible thought-partner to staff engineers, pairing them with the business context they need to choose well. Scope: a critical system and its senior ICs.</t>
+          <t>Depth: Maintains depth across a complex system's stack and hardest problems; a credible thought-partner to the most senior engineers, pairing them with the context they need. Evidenced by: Asks the one design-review question that makes a senior engineer redo their approach, without being the one who could have written the code. Scope: one team.</t>
         </is>
       </c>
       <c r="H28" s="4" t="inlineStr">
         <is>
-          <t>Depth: Retains broad technical credibility across a domain — credible on its hardest cross-team technical questions, staying current enough to ask the question that changes a design. Scope: a domain.</t>
+          <t>Depth: Maintains depth across a complex system's stack and hardest problems; a credible thought-partner to the most senior engineers, pairing them with the context they need. Evidenced by: Is the person a staff engineer brings a genuinely hard call to before committing to it, on a system outside their own team. Scope: a complex / critical team.</t>
         </is>
       </c>
       <c r="I28" s="4" t="inlineStr">
         <is>
-          <t>Depth: Sustains strategic technical credibility across a sub-org — credible with the principal engineers and architects who set the bar, and backs their judgment publicly. Scope: a sub-org.</t>
+          <t>Depth: Retains broad credibility across a multi-team domain — credible on its hardest cross-cutting technical questions, current enough to ask the question that changes a design. Evidenced by: Gets pulled into a cross-team design dispute specifically because both sides trust their read of the trade-off. Scope: a domain (cross-team).</t>
         </is>
       </c>
       <c r="J28" s="4" t="inlineStr">
         <is>
-          <t>Depth: Maintains the credibility to guide a function's technology direction — translates architectural risk into business terms without distortion. Scope: a function.</t>
+          <t>Depth: Retains broad credibility across a multi-team domain — credible on its hardest cross-cutting technical questions, current enough to ask the question that changes a design. Evidenced by: Sustains strategic technical credibility across a sub-org, credible with the principal engineers and architects who set the bar. Scope: a sub-org.</t>
         </is>
       </c>
       <c r="K28" s="4" t="inlineStr">
         <is>
-          <t>Depth: Sustains credibility across the org's technology landscape — engineers trust their technical judgment because it survives contact with detail. Scope: org-wide.</t>
+          <t>Depth: Sustains the credibility to guide an organization's technology direction; translates architectural risk into business terms without distortion, and senior technologists accept the judgment. Evidenced by: Talks a CFO out of a cost-cutting call by reframing the architectural risk in terms that survive the CFO's own scrutiny. Scope: a function.</t>
+        </is>
+      </c>
+      <c r="L28" s="4" t="inlineStr">
+        <is>
+          <t>Depth: Sustains the credibility to guide an organization's technology direction; translates architectural risk into business terms without distortion, and senior technologists accept the judgment. Evidenced by: Sustains credibility across the org's technology landscape; engineers trust their judgment because it survives contact with detail. Scope: org-wide.</t>
         </is>
       </c>
     </row>
@@ -2331,37 +2472,42 @@
       </c>
       <c r="E29" s="4" t="inlineStr">
         <is>
-          <t>Larson, An Elegant Puzzle (2019); Wardley Maps (2016)</t>
+          <t>Shapes technical direction beyond own work.</t>
         </is>
       </c>
       <c r="F29" s="4" t="inlineStr">
         <is>
-          <t>Depth: Reserves and defends explicit capacity for technical investment each quarter — names what debt costs in incidents and velocity, and challenges the build-first instinct with a written cost-of-ownership comparison before the team writes custom infrastructure. Scope: one team's technical budget.</t>
+          <t>Larson, An Elegant Puzzle: Systems of Engineering Management (Stripe Press, 2019) — the platform-versus-feature allocation is a strategy decision managers make whether or not they make it consciously</t>
         </is>
       </c>
       <c r="G29" s="4" t="inlineStr">
         <is>
-          <t>Depth: Writes the technical investment case for a critical system — sunset, rewrite, or double down — with costed options; makes reversible technology choices fast and irreversible ones deliberately, with spikes and exit criteria. Scope: a critical system's trajectory.</t>
+          <t>Depth: Influences component-level decisions through credibility. Evidenced by: Reserves and defends explicit capacity for technical investment each quarter, naming what debt costs in incidents and velocity. Scope: one team.</t>
         </is>
       </c>
       <c r="H29" s="4" t="inlineStr">
         <is>
-          <t>Depth: Aligns technical direction across a domain — shared platform bets, deprecation calendars, convergence of overlapping technology — through cases teams they do not run choose to fund, positioning each choice on differentiation versus commodity. Scope: cross-team technical portfolio.</t>
+          <t>Depth: Sets technical direction for a domain; others align to their calls. Evidenced by: Writes the technical investment case for a critical system with costed options, and makes reversible choices fast, irreversible ones deliberately. Scope: a complex / critical team.</t>
         </is>
       </c>
       <c r="I29" s="4" t="inlineStr">
         <is>
-          <t>Depth: Balances a sub-org's build-buy-adopt portfolio and sequences platform migrations across years, running an investment review so choices compound instead of fragmenting; the sub-org's systems get simpler while shipping more. Scope: a sub-org's technical estate.</t>
+          <t>Depth: Shapes how multiple teams approach problems; trusted tiebreaker. Evidenced by: Aligns technical direction across a domain -- shared platform bets, deprecation calendars -- through cases teams they do not run choose to fund. Scope: a domain (cross-team).</t>
         </is>
       </c>
       <c r="J29" s="4" t="inlineStr">
         <is>
-          <t>Depth: Puts technical strategy on the executive agenda in business terms — capability unlocked, risk retired, cost curve bent — and wins multi-year funding for unglamorous foundations, setting the function's build/buy/partner doctrine. Scope: a function.</t>
+          <t>Depth: Shapes how multiple teams approach problems; trusted tiebreaker. Evidenced by: Balances a sub-org's build-buy-adopt portfolio and sequences platform migrations across years, running an investment review so choices compound. Scope: a sub-org.</t>
         </is>
       </c>
       <c r="K29" s="4" t="inlineStr">
         <is>
-          <t>Depth: Makes the org's defining technical bets — the platform choices competitors respond to — and communicates them so thousands of local decisions align; answers for their decade-scale consequences publicly. Scope: org-wide, externally visible.</t>
+          <t>Depth: Influences org-wide technical strategy. Evidenced by: Puts technical strategy on the executive agenda in business terms and wins multi-year funding for unglamorous foundations. Scope: a function.</t>
+        </is>
+      </c>
+      <c r="L29" s="4" t="inlineStr">
+        <is>
+          <t>Depth: Influences company strategic direction through insight. Evidenced by: Makes the org's defining technical bets and communicates them so thousands of local decisions align. Scope: org-wide.</t>
         </is>
       </c>
     </row>
@@ -2388,37 +2534,42 @@
       </c>
       <c r="E30" s="4" t="inlineStr">
         <is>
-          <t>Cagan, Inspired (2008)</t>
+          <t>Connects technical work to user and business value.</t>
         </is>
       </c>
       <c r="F30" s="4" t="inlineStr">
         <is>
-          <t>Depth: Explains how the team's work serves customers and the business, and the key constraints it operates under — including regulated-industry constraints where they apply. Scope: one team's product surface.</t>
+          <t>Cagan, INSPIRED: How to Create Tech Products Customers Love, 2nd Edition (Wiley, 2018) — engineering decisions are only as good as their grasp of product, customer, economics, and regulatory context</t>
         </is>
       </c>
       <c r="G30" s="4" t="inlineStr">
         <is>
-          <t>Depth: Connects a critical system's work to business value and cost — makes cost- and compliance-aware trade-offs stakeholders recognize as commercially literate. Scope: a critical system.</t>
+          <t>Depth: Frames own work in user/business outcomes, not just tasks. Evidenced by: Explains how the team's work serves customers and the business, and the key constraints it operates under. Scope: one team.</t>
         </is>
       </c>
       <c r="H30" s="4" t="inlineStr">
         <is>
-          <t>Depth: Owns the business, customer, and regulatory case for a domain, aligning its technical work to outcomes and constraints; product partners treat their reasoning as native. Scope: a domain.</t>
+          <t>Depth: Treats their area as a product; uses metrics to decide what to build for a domain. Evidenced by: Connects a critical system's work to business value and cost, making trade-offs stakeholders recognize as commercially literate. Scope: a complex / critical team.</t>
         </is>
       </c>
       <c r="I30" s="4" t="inlineStr">
         <is>
-          <t>Depth: Aligns multiple teams' work to business and regulatory strategy through the leaders running them — investment cases read in market terms first. Scope: a sub-org.</t>
+          <t>Depth: Expert at aligning technical bets with product strategy across teams. Evidenced by: Owns the business, customer, and regulatory case for a domain, aligning its technical work to outcomes and constraints. Scope: a domain (cross-team).</t>
         </is>
       </c>
       <c r="J30" s="4" t="inlineStr">
         <is>
-          <t>Depth: Shapes how engineering serves company strategy — owns the function's business fluency, and engineering choices trace to unit economics and customer outcomes. Scope: a function.</t>
+          <t>Depth: Expert at aligning technical bets with product strategy across teams. Evidenced by: Aligns multiple teams' work to business and regulatory strategy through the leaders running them; investment cases read in market terms first. Scope: a sub-org.</t>
         </is>
       </c>
       <c r="K30" s="4" t="inlineStr">
         <is>
-          <t>Depth: Connects org-wide engineering to company and market strategy — the org's technical direction reads as a business thesis. Scope: org-wide.</t>
+          <t>Depth: Sets product direction for an org's technical surface. Evidenced by: Shapes how engineering serves company strategy, owning the function's business fluency. Scope: a function.</t>
+        </is>
+      </c>
+      <c r="L30" s="4" t="inlineStr">
+        <is>
+          <t>Depth: Shapes how the company creates value through technical products. Evidenced by: Connects org-wide engineering to company and market strategy; the org's technical direction reads as a business thesis. Scope: org-wide.</t>
         </is>
       </c>
     </row>
@@ -2445,37 +2596,42 @@
       </c>
       <c r="E31" s="4" t="inlineStr">
         <is>
-          <t>Conway (1968); Nygard, Documenting Architecture Decisions (2011)</t>
+          <t>Evaluates and justifies design options against competing quality attributes and constraints.</t>
         </is>
       </c>
       <c r="F31" s="4" t="inlineStr">
         <is>
-          <t>Depth: Runs design review as a real gate — asks the trade-off and failure-mode questions that change designs — while leaving the decision with the engineers who own it; consequential decisions get recorded with alternatives considered. Scope: one team's designs.</t>
+          <t>Conway, How Do Committees Invent?, Datamation 14(4), 28-31 (1968) — leaders shape architecture through decision processes and team boundaries even when they never write the design doc</t>
         </is>
       </c>
       <c r="G31" s="4" t="inlineStr">
         <is>
-          <t>Depth: Spots architecture risk in a critical system before it ships — coupling, scale cliffs, single points of failure — and gets it addressed without designing it themselves, naming the trade-offs the decision-makers must own. Scope: a critical system.</t>
+          <t>Depth: Evaluates standard trade-offs independently for routine architectural choices. Evidenced by: Runs design review as a real gate -- asks the trade-off and failure-mode questions that change designs -- while leaving the decision with the engineers who own it. Scope: one team.</t>
         </is>
       </c>
       <c r="H31" s="4" t="inlineStr">
         <is>
-          <t>Depth: Installs the decision mechanisms a domain designs by — decision records, RFC review, architecture forums — that teams they do not run use; catches mismatches between team shape and target architecture early. Scope: cross-team technical governance.</t>
+          <t>Depth: Structures and defends trade-off decisions for ambiguous, high-stakes designs autonomously. Evidenced by: Spots architecture risk in a critical system before it ships, and gets it addressed without designing it themselves. Scope: a complex / critical team.</t>
         </is>
       </c>
       <c r="I31" s="4" t="inlineStr">
         <is>
-          <t>Depth: Pairs org design with architecture direction deliberately — reshaping team boundaries so the target system becomes the path of least resistance; the sub-org's principal engineers set direction inside guardrails they negotiated together. Scope: a sub-org.</t>
+          <t>Depth: Defines trade-off analysis methods and decision frameworks others adopt. Evidenced by: Installs the decision mechanisms a domain designs by -- decision records, RFC review, architecture forums -- that teams they do not run use. Scope: a domain (cross-team).</t>
         </is>
       </c>
       <c r="J31" s="4" t="inlineStr">
         <is>
-          <t>Depth: Holds the line on function-wide architectural coherence — few platforms, deliberate exceptions with expiry dates — without becoming the bottleneck. Scope: a function.</t>
+          <t>Depth: Defines trade-off analysis methods and decision frameworks others adopt. Evidenced by: Pairs org design with architecture direction deliberately, reshaping team boundaries so the target system becomes the path of least resistance. Scope: a sub-org.</t>
         </is>
       </c>
       <c r="K31" s="4" t="inlineStr">
         <is>
-          <t>Depth: Answers for the org's technical integrity to the board and customers — knows where the liabilities are buried and funds the excavations, with a decision record showing the bets were reasoned, not fashionable. Scope: org-wide systems.</t>
+          <t>Depth: Sets how the organization makes architectural trade-offs, anticipating future tensions. Evidenced by: Holds the line on function-wide architectural coherence -- few platforms, deliberate exceptions with expiry dates -- without becoming the bottleneck. Scope: a function.</t>
+        </is>
+      </c>
+      <c r="L31" s="4" t="inlineStr">
+        <is>
+          <t>Depth: Advances trade-off-analysis practice recognized across the industry. Evidenced by: Answers for the org's technical integrity to the board and customers, knowing where the liabilities are buried and funding the excavations. Scope: org-wide.</t>
         </is>
       </c>
     </row>
@@ -2502,37 +2658,42 @@
       </c>
       <c r="E32" s="4" t="inlineStr">
         <is>
-          <t>Humble &amp; Farley, Continuous Delivery (2010)</t>
+          <t>Keeps code healthy, modular and maintainable.</t>
         </is>
       </c>
       <c r="F32" s="4" t="inlineStr">
         <is>
-          <t>Depth: Holds the quality bar in practice — tests, review discipline, definition of done — and does not waive it under deadline pressure without a written, expiring exception. Scope: one team's standard.</t>
+          <t>Humble &amp; Farley, Continuous Delivery: Reliable Software Releases through Build Test and Deployment Automation (Addison-Wesley, 2010) — quality is a property of the system of work, and managers own the system of work</t>
         </is>
       </c>
       <c r="G32" s="4" t="inlineStr">
         <is>
-          <t>Depth: Raises the bar on a system where it has slipped — testability, deploy safety, review quality — while shipping continues, and measures the change in escaped defects and change-fail rate. Scope: a critical codebase.</t>
+          <t>Depth: Writes clean, documented, modular code; gives useful review feedback. Evidenced by: Holds the quality bar in practice and does not waive it under deadline pressure without a written, expiring exception. Scope: one team.</t>
         </is>
       </c>
       <c r="H32" s="4" t="inlineStr">
         <is>
-          <t>Depth: Harmonizes standards across teams by making the best team's practice everyone's default — documented, tooled, adopted because it is easier; exceptions exist and each is justified in writing. Scope: a domain's engineering practice.</t>
+          <t>Depth: Designs for maintainability; leads refactors of problem areas; review feedback teaches. Evidenced by: Raises the bar on a system where it has slipped, while shipping continues, and measures the change in escaped defects and change-fail rate. Scope: a complex / critical team.</t>
         </is>
       </c>
       <c r="I32" s="4" t="inlineStr">
         <is>
-          <t>Depth: Builds the paved road — golden paths, shared tooling, quality gates in the pipeline — that makes a sub-org's standard the path of least resistance, funded as a first-class budget line. Scope: a sub-org.</t>
+          <t>Depth: Expert in code health at scale (shared libraries, deprecations, large migrations). Evidenced by: Harmonizes standards across teams by making the best team's practice everyone's default -- documented, tooled, adopted because it is easier. Scope: a domain (cross-team).</t>
         </is>
       </c>
       <c r="J32" s="4" t="inlineStr">
         <is>
-          <t>Depth: Publishes the function's engineering bar and reports honestly against it to executives, including where it is not met, winning the cost-of-quality trade explicitly rather than smuggling it into estimates. Scope: a function's reputation for quality.</t>
+          <t>Depth: Expert in code health at scale (shared libraries, deprecations, large migrations). Evidenced by: Builds the paved road -- golden paths, shared tooling, quality gates in the pipeline -- funded as a first-class budget line. Scope: a sub-org.</t>
         </is>
       </c>
       <c r="K32" s="4" t="inlineStr">
         <is>
-          <t>Depth: Makes engineering excellence part of the org's external identity — visible in the reliability customers experience, postmortems worth publishing, and the talent it attracts. Scope: org-wide.</t>
+          <t>Depth: Shapes org-wide engineering standards for long-lived codebases. Evidenced by: Publishes the function's engineering bar and reports honestly against it to executives, including where it is not met. Scope: a function.</t>
+        </is>
+      </c>
+      <c r="L32" s="4" t="inlineStr">
+        <is>
+          <t>Depth: Defines what good engineering looks like company-wide; externally recognized. Evidenced by: Makes engineering excellence part of the org's external identity, visible in the reliability customers experience. Scope: org-wide.</t>
         </is>
       </c>
     </row>
@@ -2549,7 +2710,7 @@
       </c>
       <c r="C33" s="4" t="inlineStr">
         <is>
-          <t>Technical Debt &amp; Risk Stewardship</t>
+          <t>Technical Debt &amp; Modernization</t>
         </is>
       </c>
       <c r="D33" s="6" t="inlineStr">
@@ -2559,37 +2720,42 @@
       </c>
       <c r="E33" s="4" t="inlineStr">
         <is>
-          <t>Cunningham, The WyCash Portfolio Management System (1992)</t>
+          <t>Surfaces, prices, and manages technical debt and technical risk as an economic portfolio — funding paydown structurally and setting the speed-versus-soundness posture explicitly.</t>
         </is>
       </c>
       <c r="F33" s="4" t="inlineStr">
         <is>
-          <t>Depth: Keeps a visible debt register with the cost of carry noted and retires items on a cadence, defending a steady paydown allocation in planning rather than begging quarter by quarter. Scope: one team's codebases.</t>
+          <t>Cunningham, The WyCash Portfolio Management System, OOPSLA 1992 Experience Report — debt is a deliberate liability with interest, paid down on purpose, not neglected mess</t>
         </is>
       </c>
       <c r="G33" s="4" t="inlineStr">
         <is>
-          <t>Depth: Distinguishes debt worth carrying from debt that will detonate and sequences remediation by risk, pricing debt in incident and velocity terms stakeholders accept; lands a major consolidation without stopping the roadmap. Scope: a critical system.</t>
+          <t>Depth: Keeps a visible debt register with the cost of carry noted and defends a steady paydown allocation in planning rather than begging quarter by quarter. Evidenced by: Trades a feature slot for a paydown item in planning by pointing to the register entry showing what the debt has already cost in incidents. Scope: one team.</t>
         </is>
       </c>
       <c r="H33" s="4" t="inlineStr">
         <is>
-          <t>Depth: Makes debt legible across a domain — a shared taxonomy and reporting rhythm teams they do not run adopt — and aggregates cross-team risk: the shared library nobody owns, the migration half-finished in three places, owned and funded. Scope: cross-team quality economics.</t>
+          <t>Depth: Distinguishes debt worth carrying from debt that will detonate, sequences remediation by risk, and prices debt in incident and velocity terms stakeholders accept. Evidenced by: Lands a major consolidation that retires a chunk of debt without ever stopping the roadmap to do it. Scope: a complex / critical team.</t>
         </is>
       </c>
       <c r="I33" s="4" t="inlineStr">
         <is>
-          <t>Depth: Sets a sub-org's quality strategy — where to gold-plate, where to accept scrappy — and lands multi-quarter remediation programs against feature pressure, with debt stated in business terms: incident cost, velocity drag, security exposure. Scope: a sub-org's risk portfolio.</t>
+          <t>Depth: Makes debt legible across multiple teams — shared taxonomy, reporting rhythm — and gets cross-team risk (the shared library nobody owns, the half-finished migration) owned and funded. Evidenced by: Makes debt legible across a domain -- a shared taxonomy and reporting rhythm teams they do not run adopt -- and aggregates cross-team risk. Scope: a domain (cross-team).</t>
         </is>
       </c>
       <c r="J33" s="4" t="inlineStr">
         <is>
-          <t>Depth: Carries the function's technical risk onto the executive risk register — top exposures known, sized, owned, and trending — and prevents the quarterly raid on foundational capacity. Scope: a function.</t>
+          <t>Depth: Makes debt legible across multiple teams — shared taxonomy, reporting rhythm — and gets cross-team risk (the shared library nobody owns, the half-finished migration) owned and funded. Evidenced by: Sets a sub-org's quality strategy and lands multi-quarter remediation programs against feature pressure, debt stated in business terms. Scope: a sub-org.</t>
         </is>
       </c>
       <c r="K33" s="4" t="inlineStr">
         <is>
-          <t>Depth: Sets the org's speed-versus-soundness dial explicitly — declares where the org will accept debt for velocity and where it never will — and holds it under growth pressure. Scope: org-wide.</t>
+          <t>Depth: Carries technical risk onto the executive risk register — top exposures known, sized, owned, trending — and lands multi-quarter remediation programs against feature pressure. Evidenced by: Gets a multi-quarter remediation program funded against direct feature-roadmap competition by putting it on the executive risk register. Scope: a function.</t>
+        </is>
+      </c>
+      <c r="L33" s="4" t="inlineStr">
+        <is>
+          <t>Depth: Sets an organization's speed-versus-soundness posture explicitly — where debt is accepted for velocity and where it never is — and holds it under growth pressure. Evidenced by: Publicly names the class of debt the org will always carry for speed, so no team wastes a quarter trying to fix what leadership already decided to accept. Scope: org-wide.</t>
         </is>
       </c>
     </row>
@@ -2616,37 +2782,42 @@
       </c>
       <c r="E34" s="4" t="inlineStr">
         <is>
-          <t>Minto, The Pyramid Principle (1987)</t>
+          <t>Conveys ideas clearly to the right audience.</t>
         </is>
       </c>
       <c r="F34" s="4" t="inlineStr">
         <is>
-          <t>Depth: Writes updates and decision docs that lead with the answer and fit on a page; runs meetings that start with a purpose and end with owners and dates. Scope: one team's information flow.</t>
+          <t>Minto, The Minto Pyramid Principle: Logic in Writing, Thinking, and Problem Solving (Minto International, 1996) — lead with the answer, group the supporting arguments, order them logically</t>
         </is>
       </c>
       <c r="G34" s="4" t="inlineStr">
         <is>
-          <t>Depth: Makes complex technical situations legible to non-engineers without dumbing them down — an incident narrative a customer team can use, a trade-off memo a product partner can decide on. Scope: a critical team's external interface.</t>
+          <t>Depth: Writes clear design notes, runbooks and PRs; explains trade-offs without overselling. Evidenced by: Writes updates and decision docs that lead with the answer and fit on a page, and runs meetings that end with owners and dates. Scope: one team.</t>
         </is>
       </c>
       <c r="H34" s="4" t="inlineStr">
         <is>
-          <t>Depth: Writes the documents cross-team decisions get made from — framing memos, options papers — that people cite weeks later; several teams execute against them without a clarifying meeting. Scope: domain-level discourse.</t>
+          <t>Depth: Writes design docs that drive decisions; translates technical risk for non-technical stakeholders. Evidenced by: Makes complex technical situations legible to non-engineers without dumbing them down -- an incident narrative a customer team can use. Scope: a complex / critical team.</t>
         </is>
       </c>
       <c r="I34" s="4" t="inlineStr">
         <is>
-          <t>Depth: Sets the writing norms — templates, pre-read culture, decision-doc formats — a sub-org adopts because their versions demonstrably work. Scope: a sub-org's document culture.</t>
+          <t>Depth: Expert at making complex capability/risk legible to executives without dumbing it down; RFCs align orgs. Evidenced by: Writes the documents cross-team decisions get made from -- framing memos, options papers -- that people cite weeks later. Scope: a domain (cross-team).</t>
         </is>
       </c>
       <c r="J34" s="4" t="inlineStr">
         <is>
-          <t>Depth: Delivers one message coherently across audiences — board slide, all-hands, engineering deep-dive — without the versions contradicting each other. Scope: a function's narrative.</t>
+          <t>Depth: Expert at making complex capability/risk legible to executives without dumbing it down; RFCs align orgs. Evidenced by: Sets the writing norms -- templates, pre-read culture, decision-doc formats -- a sub-org adopts because their versions demonstrably work. Scope: a sub-org.</t>
         </is>
       </c>
       <c r="K34" s="4" t="inlineStr">
         <is>
-          <t>Depth: Gives the org its language — the phrases and frames people use to explain the strategy to each other — and lands hard messages with clarity and humanity. Scope: org-wide and external.</t>
+          <t>Depth: Strategy memos leadership acts on; org-wide and external reach. Evidenced by: Delivers one message coherently across audiences -- board slide, all-hands, engineering deep-dive -- without the versions contradicting each other. Scope: a function.</t>
+        </is>
+      </c>
+      <c r="L34" s="4" t="inlineStr">
+        <is>
+          <t>Depth: A clarifying voice at company scale; externally recognized. Evidenced by: Gives the org its language -- the phrases people use to explain the strategy to each other -- and lands hard messages with clarity and humanity. Scope: org-wide.</t>
         </is>
       </c>
     </row>
@@ -2673,37 +2844,42 @@
       </c>
       <c r="E35" s="4" t="inlineStr">
         <is>
-          <t>Duarte, HBR Guide to Persuasive Presentations (2012)</t>
+          <t>Communicates upward and to executive audiences — answer-first briefings, decision-ready framing, and composure under hostile questioning.</t>
         </is>
       </c>
       <c r="F35" s="4" t="inlineStr">
         <is>
-          <t>Depth: Reports upward with the headline and the ask first — never burying the slip in paragraph four; no surprise reaches their leadership from someone else. Scope: their management chain and immediate stakeholders.</t>
+          <t>Duarte, HBR Guide to Persuasive Presentations (Harvard Business Review Press, 2012) — decisions above a leader are made on how the case is communicated, not only on its merits</t>
         </is>
       </c>
       <c r="G35" s="4" t="inlineStr">
         <is>
-          <t>Depth: Briefs senior leaders under fire — facts, impact, options, and a recommendation inside the first two minutes; their one-pagers get forwarded unedited. Scope: executive-facing moments for a critical program.</t>
+          <t>Depth: Reports upward answer-first with a specific ask; escalates early with options attached, so no surprise reaches leadership from someone else. Evidenced by: Reports upward with the headline and the ask first, never burying the slip in paragraph four. Scope: one team.</t>
         </is>
       </c>
       <c r="H35" s="4" t="inlineStr">
         <is>
-          <t>Depth: Builds the case for a cross-team investment and lands it with an executive audience — pre-wired with the skeptics, sized in business terms, honest about risk; preps other managers for executive rooms. Scope: domain-level asks and narratives.</t>
+          <t>Depth: Briefs senior leaders under pressure — facts, impact, options, and a recommendation inside the first two minutes; one-pagers get forwarded unedited. Evidenced by: Turns a skeptical VP's contested launch review into a green light in one sitting, opening with the recommendation before the data. Scope: a complex / critical team.</t>
         </is>
       </c>
       <c r="I35" s="4" t="inlineStr">
         <is>
-          <t>Depth: Runs the operating reviews a sub-org communicates through — the packet, the rhythm, the follow-through — managing a portfolio of executive stakeholders with different agendas and keeping commitments to all of them consistent. Scope: a sub-org's upward interface.</t>
+          <t>Depth: Builds and lands investment cases with executive audiences — pre-wired with skeptics, sized in business terms, honest about risk; coaches others for executive rooms and runs the operating reviews an organization communicates through. Evidenced by: Builds the case for a cross-team investment and lands it with an executive audience, pre-wired with the skeptics and honest about risk. Scope: a domain (cross-team).</t>
         </is>
       </c>
       <c r="J35" s="4" t="inlineStr">
         <is>
-          <t>Depth: Operates the executive room as a peer — advances a position, absorbs hostile questioning without defensiveness, and changes the room's decision more often than not. Scope: a function's voice at the top table.</t>
+          <t>Depth: Operates the executive room as a peer — advances positions, absorbs hostile questioning without defensiveness, and changes the room's decision more often than not. Evidenced by: Runs the operating reviews a sub-org communicates through, managing a portfolio of executive stakeholders with different agendas. Scope: a sub-org.</t>
         </is>
       </c>
       <c r="K35" s="4" t="inlineStr">
         <is>
-          <t>Depth: Speaks for the org's technical reality to boards, investors, and press — candid about bad news, precise about trade-offs; the org's credibility survives their appearances. Scope: org-wide and external.</t>
+          <t>Depth: Operates the executive room as a peer — advances positions, absorbs hostile questioning without defensiveness, and changes the room's decision more often than not. Evidenced by: Walks into a hostile budget review as the only voice defending the function's headcount ask, and leaves with it approved. Scope: a function.</t>
+        </is>
+      </c>
+      <c r="L35" s="4" t="inlineStr">
+        <is>
+          <t>Depth: Speaks for an organization's technical reality to boards, investors, and press; trusted with the messages that cannot be delegated, and organizational credibility survives the appearances. Evidenced by: Fronts the org's response to a public outage for press and investors, and the org's credibility holds through it. Scope: org-wide.</t>
         </is>
       </c>
     </row>
@@ -2730,37 +2906,42 @@
       </c>
       <c r="E36" s="4" t="inlineStr">
         <is>
-          <t>Freeman, Strategic Management: A Stakeholder Approach (1984)</t>
+          <t>Aligning leadership and cross-functional stakeholders around product direction and trade-offs.</t>
         </is>
       </c>
       <c r="F36" s="4" t="inlineStr">
         <is>
-          <t>Depth: Runs a genuine triad with product and design — shared goals, early involvement, no surprise commitments — and closes the loop when things change. Scope: one team's partner set.</t>
+          <t>Freeman, Strategic Management: A Stakeholder Approach (Pitman, 1984) — engineering leaders sit in a web of product, design, sales, support, and operations whose trust is built deliberately</t>
         </is>
       </c>
       <c r="G36" s="4" t="inlineStr">
         <is>
-          <t>Depth: Maps and works a critical program's stakeholders — who needs consultation versus information — and repairs a damaged partnership by resetting expectations and rebuilding credibility with delivered commitments. Scope: a program's stakeholder web.</t>
+          <t>Depth: Manages routine stakeholder relationships and communications with normal review. Evidenced by: Runs a genuine triad with product and design -- shared goals, early involvement, no surprise commitments -- and closes the loop when things change. Scope: one team.</t>
         </is>
       </c>
       <c r="H36" s="4" t="inlineStr">
         <is>
-          <t>Depth: Treats their peer group as their first team — argues hard in the room, backs the decision outside it — and builds durable cross-functional relationships: sales, support, and operations bring them bad news early. Scope: a domain's partner ecosystem.</t>
+          <t>Depth: Independently aligns conflicting stakeholders and navigates tense executive conversations. Evidenced by: Maps and works a critical program's stakeholders, and repairs a damaged partnership by resetting expectations and rebuilding credibility. Scope: a complex / critical team.</t>
         </is>
       </c>
       <c r="I36" s="4" t="inlineStr">
         <is>
-          <t>Depth: Designs how a sub-org interfaces with the rest of the business — intake paths, escalation contracts, joint planning and shared metrics — so partnership survives personnel changes. Scope: a sub-org's external seams.</t>
+          <t>Depth: Defines stakeholder-engagement approaches others adopt and brokers the hardest alignment. Evidenced by: Treats their peer group as their first team -- argues hard in the room, backs the decision outside it -- and builds durable cross-functional relationships. Scope: a domain (cross-team).</t>
         </is>
       </c>
       <c r="J36" s="4" t="inlineStr">
         <is>
-          <t>Depth: Forms function-to-function alliances with product, sales, finance, and legal — reciprocal, durable, tested in a crisis — trading short-term losses for long-term trust deliberately. Scope: cross-functional executive web.</t>
+          <t>Depth: Defines stakeholder-engagement approaches others adopt and brokers the hardest alignment. Evidenced by: Designs how a sub-org interfaces with the rest of the business -- intake paths, escalation contracts, joint planning -- so partnership survives personnel changes. Scope: a sub-org.</t>
         </is>
       </c>
       <c r="K36" s="4" t="inlineStr">
         <is>
-          <t>Depth: Stewards the org's most consequential external relationships — key customers, strategic partners, board stakeholders — and models one-company leadership, resolving function-versus-function conflicts by company interest even at cost to their own area. Scope: org-wide and external.</t>
+          <t>Depth: Sets executive-engagement strategy and anticipates leadership concerns before they arise. Evidenced by: Forms function-to-function alliances with product, sales, finance, and legal -- reciprocal, durable, tested in a crisis. Scope: a function.</t>
+        </is>
+      </c>
+      <c r="L36" s="4" t="inlineStr">
+        <is>
+          <t>Depth: Defines exemplary stakeholder management for the discipline and is externally credible on it. Evidenced by: Stewards the org's most consequential external relationships and models one-company leadership, resolving conflicts by company interest. Scope: org-wide.</t>
         </is>
       </c>
     </row>
@@ -2787,37 +2968,42 @@
       </c>
       <c r="E37" s="4" t="inlineStr">
         <is>
-          <t>Cohen &amp; Bradford, Influence Without Authority (1989)</t>
+          <t>Wins outcomes across organizational seams with no formal mandate — exchange in others' currencies, coalition-building, and earned credibility.</t>
         </is>
       </c>
       <c r="F37" s="4" t="inlineStr">
         <is>
-          <t>Depth: Wins cooperation from adjacent teams by trading in their currencies — timing help, review effort, shared credit — rather than escalating. Scope: one team's dependencies.</t>
+          <t>Cohen &amp; Bradford, Influence Without Authority, 3rd ed. (Wiley, 2017) — from Director up, nearly everything a leader needs done is done by people who do not answer to them</t>
         </is>
       </c>
       <c r="G37" s="4" t="inlineStr">
         <is>
-          <t>Depth: Secures priority from other teams for a critical program with no borrowed authority — builds the case in the other team's terms and repays visibly. Scope: a program's dependency network.</t>
+          <t>Depth: Wins cooperation from adjacent teams by trading in their currencies — timing help, review effort, shared credit — rather than escalating. Scope: one team.</t>
         </is>
       </c>
       <c r="H37" s="4" t="inlineStr">
         <is>
-          <t>Depth: Moves a domain to a shared position with no mandate — assembles the coalition, converts the skeptic whose objection is best — and the position holds after they stop pushing. Scope: cross-team direction.</t>
+          <t>Depth: Secures priority from other teams for an initiative with no borrowed authority; builds the case in the other party's terms and repays visibly. Evidenced by: Gets a dependency bumped ahead of another team's roadmap item by making the case in that team's own success metrics, not theirs. Scope: a complex / critical team.</t>
         </is>
       </c>
       <c r="I37" s="4" t="inlineStr">
         <is>
-          <t>Depth: Shifts sub-org-level outcomes through people two seams away — standards groups, principal engineers, partner leaders — who advocate the position as their own. Scope: a sub-org's ecosystem.</t>
+          <t>Depth: Moves a multi-team domain to a shared position with no mandate — assembles the coalition, converts the best-argued skeptic — and the position holds after they stop pushing. Evidenced by: Turns the domain's most vocal skeptic of a shared direction into the person who pitches it to the next skeptic. Scope: a domain (cross-team).</t>
         </is>
       </c>
       <c r="J37" s="4" t="inlineStr">
         <is>
-          <t>Depth: Influences peer executives and their organizations — lands function-shaping decisions while holding a minority of the formal power in the room. Scope: cross-functional.</t>
+          <t>Depth: Moves a multi-team domain to a shared position with no mandate — assembles the coalition, converts the best-argued skeptic — and the position holds after they stop pushing. Evidenced by: Shifts sub-org-level outcomes through people two seams away who advocate the position as their own. Scope: a sub-org.</t>
         </is>
       </c>
       <c r="K37" s="4" t="inlineStr">
         <is>
-          <t>Depth: Shapes industry and market context in the org's favor — standards bodies, open source, talent narratives — so external forces push where the org wants to go. Scope: beyond the org.</t>
+          <t>Depth: Shifts organization-level outcomes through people several seams away who advocate the position as their own; lands decisions while holding a minority of the formal power in the room. Evidenced by: Influences peer executives and their organizations, landing function-shaping decisions while holding a minority of the formal power in the room. Scope: a function.</t>
+        </is>
+      </c>
+      <c r="L37" s="4" t="inlineStr">
+        <is>
+          <t>Depth: Shapes industry and market context in the organization's favor — standards bodies, open ecosystems, talent narratives — so external forces push where the organization wants to go. Evidenced by: Gets an external standards body to adopt a pattern the org championed, so competitors now build to terms the org set. Scope: org-wide.</t>
         </is>
       </c>
     </row>
@@ -2844,37 +3030,42 @@
       </c>
       <c r="E38" s="4" t="inlineStr">
         <is>
-          <t>Fisher &amp; Ury, Getting to Yes (1981); Lencioni (2002)</t>
+          <t>Navigates conflict toward good decisions.</t>
         </is>
       </c>
       <c r="F38" s="4" t="inlineStr">
         <is>
-          <t>Depth: Surfaces simmering disagreement early and mediates it to interests — names the tension, separates people from positions, drives to an agreement both sides can state fairly. Scope: within one team and its nearest neighbors.</t>
+          <t>Fisher &amp; Ury, Getting to Yes: Negotiating Agreement Without Giving In (Penguin, 1981) — healthy organizations fight about ideas in the open, and unresolved conflict is one of the most expensive latencies an org carries</t>
         </is>
       </c>
       <c r="G38" s="4" t="inlineStr">
         <is>
-          <t>Depth: Negotiates commitments under pressure — scope, deadlines, contested interfaces — reaching agreements both sides keep, with the trade documented; reframes turf disputes as interface-design problems. Scope: a critical team's boundaries and stakes.</t>
+          <t>Depth: Works through disagreement to a decision without damaging relationships. Evidenced by: Surfaces simmering disagreement early and mediates it to interests, separating people from positions and driving to an agreement both sides can state fairly. Scope: one team.</t>
         </is>
       </c>
       <c r="H38" s="4" t="inlineStr">
         <is>
-          <t>Depth: Resolves lead-to-lead conflicts others route around as a trusted broker — finds the interest-based trade and teaches the parties to resolve the next one themselves; people bring them conflicts they are not even party to. Scope: cross-team disputes in a domain.</t>
+          <t>Depth: Mediates technical disputes in their domain; finds the path that holds up. Evidenced by: Negotiates commitments under pressure -- scope, deadlines, contested interfaces -- reaching agreements both sides keep, with the trade documented. Scope: a complex / critical team.</t>
         </is>
       </c>
       <c r="I38" s="4" t="inlineStr">
         <is>
-          <t>Depth: Redesigns the structures that generate recurring conflict — misaligned incentives, ambiguous ownership — instead of re-mediating the same fight, and designs escalation paths so conflicts resolve at the lowest capable level. Scope: a sub-org's conflict system.</t>
+          <t>Depth: Resolves high-stakes disagreements between senior stakeholders across orgs. Evidenced by: Resolves lead-to-lead conflicts others route around as a trusted broker, and teaches the parties to resolve the next one themselves. Scope: a domain (cross-team).</t>
         </is>
       </c>
       <c r="J38" s="4" t="inlineStr">
         <is>
-          <t>Depth: Negotiates function-level conflicts — budget splits, shared-platform terms, charter boundaries — with peer executives and external parties, keeping the relationships intact afterward. Scope: a function's seams.</t>
+          <t>Depth: Resolves high-stakes disagreements between senior stakeholders across orgs. Evidenced by: Redesigns the structures that generate recurring conflict, and designs escalation paths so conflicts resolve at the lowest capable level. Scope: a sub-org.</t>
         </is>
       </c>
       <c r="K38" s="4" t="inlineStr">
         <is>
-          <t>Depth: Turns the org's biggest ideological fights — build versus buy, centralize versus embed — into decision processes the losing side calls fair. Scope: org-wide.</t>
+          <t>Depth: Designs the decision processes the org uses to resolve conflict. Evidenced by: Negotiates function-level conflicts -- budget splits, shared-platform terms, charter boundaries -- keeping the relationships intact afterward. Scope: a function.</t>
+        </is>
+      </c>
+      <c r="L38" s="4" t="inlineStr">
+        <is>
+          <t>Depth: Sets the company norm for principled disagreement. Evidenced by: Turns the org's biggest ideological fights into decision processes the losing side calls fair. Scope: org-wide.</t>
         </is>
       </c>
     </row>
@@ -2901,37 +3092,42 @@
       </c>
       <c r="E39" s="4" t="inlineStr">
         <is>
-          <t>Grove, High Output Management (1983); Drucker (1967)</t>
+          <t>Spends leadership time where it multiplies — deliberate calendar design, high-leverage intervention choice, and systematic abandonment of low-value work.</t>
         </is>
       </c>
       <c r="F39" s="4" t="inlineStr">
         <is>
-          <t>Depth: Runs a deliberate calendar that matches stated priorities — one-on-ones, deep work, and team time protected; low-leverage meetings declined with alternatives — and ends each week with the highest-leverage actions done. Scope: their own week and one team's operating rhythm.</t>
+          <t>Grove, High Output Management (Random House, 1983) — a manager's output is the leveraged output of everyone they touch, and time is the one non-renewable resource</t>
         </is>
       </c>
       <c r="G39" s="4" t="inlineStr">
         <is>
-          <t>Depth: Prunes their own involvement ruthlessly as complexity grows — automates, delegates, or kills recurring work every quarter — and models a sustainable pace through crunch; peers copy the operating cadence. Scope: a complex team's demands on one person.</t>
+          <t>Depth: Runs a deliberate calendar that matches stated priorities — protected one-on-ones, deep work, and team time; declines low-leverage meetings with alternatives offered. Evidenced by: Runs a deliberate calendar that matches stated priorities, and ends each week with the highest-leverage actions done. Scope: one team.</t>
         </is>
       </c>
       <c r="H39" s="4" t="inlineStr">
         <is>
-          <t>Depth: Chooses interventions by multiplier across a domain — the review that shapes ten decisions, the doc that aligns three roadmaps — and declines the rest by policy, not mood; audits their own time quarterly and publishes the changes. Scope: cross-team attention allocation.</t>
+          <t>Depth: Prunes their own involvement ruthlessly as complexity grows — automates, delegates, or kills recurring work every quarter — and models sustainable pace through crunch. Evidenced by: Kills a recurring review meeting that only they found valuable, once they notice no one else has opened the notes in a month. Scope: a complex / critical team.</t>
         </is>
       </c>
       <c r="I39" s="4" t="inlineStr">
         <is>
-          <t>Depth: Designs their own role top-down from the sub-org's constraints — spends time only where they are the unique unlock — and declines demands that do not map to strategy, visibly and with reasons. Scope: a sub-org's scarcest resource, senior attention.</t>
+          <t>Depth: Chooses interventions by multiplier across many teams — the review that shapes ten decisions, the document that aligns three roadmaps — declining the rest by policy; audits their time and publishes the changes. Evidenced by: Chooses interventions by multiplier across a domain -- the review that shapes ten decisions -- and declines the rest by policy, not mood. Scope: a domain (cross-team).</t>
         </is>
       </c>
       <c r="J39" s="4" t="inlineStr">
         <is>
-          <t>Depth: Allocates attention at function scale like a portfolio — deep on two things, delegated on twenty — and says which is which out loud. Scope: a function.</t>
+          <t>Depth: Chooses interventions by multiplier across many teams — the review that shapes ten decisions, the document that aligns three roadmaps — declining the rest by policy; audits their time and publishes the changes. Evidenced by: Designs their own role top-down from the sub-org's constraints, spending time only where they are the unique unlock. Scope: a sub-org.</t>
         </is>
       </c>
       <c r="K39" s="4" t="inlineStr">
         <is>
-          <t>Depth: Spends presence deliberately as an org-wide signal — where they show up moves priorities — and guards the org's focus: limits concurrent top priorities and abandons stale initiatives by name. Scope: org-wide.</t>
+          <t>Depth: Allocates attention like a portfolio at organizational scale — deep on the few places they are the unique unlock, delegated on the rest — and says which is which out loud. Evidenced by: Tells the function plainly which two initiatives get their personal attention this half and which twenty do not. Scope: a function.</t>
+        </is>
+      </c>
+      <c r="L39" s="4" t="inlineStr">
+        <is>
+          <t>Depth: Spends presence deliberately as an organizational signal — where they show up moves priorities — and guards the organization's focus by limiting concurrent top priorities and abandoning stale initiatives by name. Evidenced by: Skips a well-attended launch review on principle, and the org reads the absence correctly as 'this isn't actually a top priority.' Scope: org-wide.</t>
         </is>
       </c>
     </row>
@@ -2958,37 +3154,42 @@
       </c>
       <c r="E40" s="4" t="inlineStr">
         <is>
-          <t>Marquet, Turn the Ship Around! (2012)</t>
+          <t>Hands over whole outcomes with context and calibrated support, pushes decision rights to where the information lives, and builds organizations that run on intent rather than presence.</t>
         </is>
       </c>
       <c r="F40" s="4" t="inlineStr">
         <is>
-          <t>Depth: Delegates whole outcomes with context and check-in contracts matched to each person's readiness — not tasks with instructions — and resists snatching work back when it wobbles. Scope: work within one team.</t>
+          <t>Marquet, Turn the Ship Around!: A True Story of Turning Followers into Leaders (Portfolio/Penguin, 2013; orig. 2012) — leadership scales by pushing authority to where the information is, creating leaders rather than followers</t>
         </is>
       </c>
       <c r="G40" s="4" t="inlineStr">
         <is>
-          <t>Depth: Hands ownership of a critical, visible workstream to someone not yet proven and scaffolds them to success — letting them keep the credit publicly; the team runs a week without them and nothing stalls. Scope: a complex team's critical path.</t>
+          <t>Depth: Delegates whole outcomes with context and check-in contracts matched to each person's readiness — and resists snatching work back when it wobbles. Scope: one team.</t>
         </is>
       </c>
       <c r="H40" s="4" t="inlineStr">
         <is>
-          <t>Depth: Pushes decisions down across a domain — publishes decision rights so teams stop escalating what they can decide themselves; their involvement is exception-based, and everyone knows which is which. Scope: cross-team decision flow.</t>
+          <t>Depth: Hands ownership of critical, visible work to someone not yet proven and scaffolds them to success, letting them keep the credit; the team runs a week without them and nothing stalls. Evidenced by: Goes on a two-week vacation from a critical workstream they handed off, and it ships on schedule without them. Scope: a complex / critical team.</t>
         </is>
       </c>
       <c r="I40" s="4" t="inlineStr">
         <is>
-          <t>Depth: Builds a sub-org that runs on mechanisms rather than their presence — delegated authorities with audit trails, pre-declared tripwires for taking back control. Scope: a sub-org that does not queue on them.</t>
+          <t>Depth: Pushes decisions down across multiple teams — publishes decision rights so teams stop escalating what they can decide themselves; involvement is exception-based, and everyone knows which is which. Evidenced by: Publishes a one-page decision-rights map that stops three different teams escalating the same class of call to them every week. Scope: a domain (cross-team).</t>
         </is>
       </c>
       <c r="J40" s="4" t="inlineStr">
         <is>
-          <t>Depth: Grants senior leaders genuinely consequential authority and holds them to outcomes, not methods; the function's decisions get faster as it grows, not slower. Scope: a function.</t>
+          <t>Depth: Pushes decisions down across multiple teams — publishes decision rights so teams stop escalating what they can decide themselves; involvement is exception-based, and everyone knows which is which. Evidenced by: Builds a sub-org that runs on mechanisms rather than their presence, with pre-declared tripwires for taking back control. Scope: a sub-org.</t>
         </is>
       </c>
       <c r="K40" s="4" t="inlineStr">
         <is>
-          <t>Depth: Runs the org on intent — direction and guardrails clear enough that leaders act correctly without asking — and treats every upward escalation as a design flaw to fix. Scope: org-wide autonomy architecture.</t>
+          <t>Depth: Builds organizations that run on mechanisms rather than presence — delegated authorities with audit trails, pre-declared tripwires — and grants leaders consequential authority held to outcomes, not methods. Evidenced by: Grants senior leaders genuinely consequential authority and holds them to outcomes, not methods; the function's decisions get faster as it grows. Scope: a function.</t>
+        </is>
+      </c>
+      <c r="L40" s="4" t="inlineStr">
+        <is>
+          <t>Depth: Runs an organization on intent — direction and guardrails clear enough that leaders act correctly without asking — and treats every upward escalation as a design flaw to fix. Evidenced by: Treats a director's request to escalate a call the director was empowered to make as a bug in the org design, not a normal Tuesday. Scope: org-wide.</t>
         </is>
       </c>
     </row>
@@ -3015,37 +3216,42 @@
       </c>
       <c r="E41" s="4" t="inlineStr">
         <is>
-          <t>Eurich, Insight (2017); Lombardo &amp; Eichinger (2000)</t>
+          <t>Seeks external feedback on their own behavior, knows their failure patterns, and extracts lessons from first-time situations fast enough to lead credibly in them.</t>
         </is>
       </c>
       <c r="F41" s="4" t="inlineStr">
         <is>
-          <t>Depth: Asks for feedback on their own management and changes visibly in response — "you said X, I changed Y" — and approaches first-time situations as learnable, keeping a running list of their own failure patterns. Scope: their own practice, witnessed by one team.</t>
+          <t>Eurich, What Self-Awareness Really Is (and How to Cultivate It), Harvard Business Review (2018) — accurate self-knowledge and the ability to learn from new experience predict leadership growth</t>
         </is>
       </c>
       <c r="G41" s="4" t="inlineStr">
         <is>
-          <t>Depth: Knows their failure modes under pressure and manages them in the moment — staffs deliberately against known weaknesses, seeking disconfirming input on their hardest calls before deciding. Scope: a critical team's exposure to their blind spots.</t>
+          <t>Depth: Asks for feedback on their own practice and changes visibly in response — "you said X, I changed Y" — keeping a running list of their own failure patterns. Evidenced by: Asks for feedback on their own management and changes visibly in response, and approaches first-time situations as learnable. Scope: one team.</t>
         </is>
       </c>
       <c r="H41" s="4" t="inlineStr">
         <is>
-          <t>Depth: Runs structured input on themselves — 360s, skip-level themes — and closes the loop publicly on what they heard and changed; retools openly for first-time challenges so others copy the learning method. Scope: signal gathered across a domain.</t>
+          <t>Depth: Knows their failure modes under pressure and manages them in the moment; staffs deliberately against known weaknesses and seeks disconfirming input before hard calls. Evidenced by: Pre-stages a co-lead for a call they know they tend to rush, because they have watched themselves rush it before. Scope: a complex / critical team.</t>
         </is>
       </c>
       <c r="I41" s="4" t="inlineStr">
         <is>
-          <t>Depth: Compensates deliberately for the seniority feedback vacuum — cultivates truth-tellers and rewards the bearer of unwelcome news about themselves; retires their own outdated playbook when the sub-org outgrows it. Scope: a sub-org's honest mirror.</t>
+          <t>Depth: Runs structured input on themselves — 360s, skip-level themes — and closes the loop publicly on what changed; retools openly for first-time challenges so others copy the learning method. Evidenced by: Runs a 360 and tells the org, in writing, the one thing it revealed that surprised them and what they are doing about it. Scope: a domain (cross-team).</t>
         </is>
       </c>
       <c r="J41" s="4" t="inlineStr">
         <is>
-          <t>Depth: Reinvents their leadership at function scale — lets go of the operator identity, learns governance and capital skills mid-flight — and says "I don't know" in rooms where pretending is the norm. Scope: a function watches and learns from it.</t>
+          <t>Depth: Runs structured input on themselves — 360s, skip-level themes — and closes the loop publicly on what changed; retools openly for first-time challenges so others copy the learning method. Evidenced by: Compensates deliberately for the seniority feedback vacuum, cultivating truth-tellers and rewarding the bearer of unwelcome news. Scope: a sub-org.</t>
         </is>
       </c>
       <c r="K41" s="4" t="inlineStr">
         <is>
-          <t>Depth: Institutionalizes challenge to their own judgment — red teams, protected dissent — and studies how their moods and offhand comments get amplified, regulating accordingly. Scope: an org-wide shadow, managed consciously.</t>
+          <t>Depth: Compensates deliberately for the seniority feedback vacuum — cultivates truth-tellers, rewards bearers of unwelcome news about themselves, and retires their own outdated playbook when the organization outgrows it. Evidenced by: Reinvents their leadership at function scale, letting go of the operator identity and saying 'I don't know' in rooms where pretending is the norm. Scope: a function.</t>
+        </is>
+      </c>
+      <c r="L41" s="4" t="inlineStr">
+        <is>
+          <t>Depth: Institutionalizes challenge to their own judgment — red teams, protected dissent — and manages how their moods and offhand comments get amplified across an organization. Evidenced by: Stands up a red-team review of their own biggest strategic bet and changes the bet when it finds a real hole. Scope: org-wide.</t>
         </is>
       </c>
     </row>
@@ -3072,37 +3278,42 @@
       </c>
       <c r="E42" s="4" t="inlineStr">
         <is>
-          <t>Loehr &amp; Schwartz, The Power of Full Engagement (2003)</t>
+          <t>Sustains effectiveness under prolonged pressure, recovers from setbacks, and designs sustainable pace into how teams operate rather than modeling heroics.</t>
         </is>
       </c>
       <c r="F42" s="4" t="inlineStr">
         <is>
-          <t>Depth: Stays effective and steady under pressure — recovers from setbacks, manages their own energy, and models a sustainable pace the team learns from watching, not from posters. Scope: one team's pace-setting example.</t>
+          <t>Loehr &amp; Schwartz, The Power of Full Engagement: Managing Energy, Not Time, Is the Key to High Performance and Personal Renewal (Free Press, 2003) — performance is a function of managed energy, not time, and sustainable pace beats heroics</t>
         </is>
       </c>
       <c r="G42" s="4" t="inlineStr">
         <is>
-          <t>Depth: Holds up through prolonged pressure — incident sieges, crunch, org turbulence — and helps the team stay resilient, refusing burnout-driven decisions and naming them when they appear. Scope: a critical team under sustained load.</t>
+          <t>Depth: Stays effective and steady under pressure — recovers from setbacks, manages their own energy, and models a sustainable pace others learn from watching. Evidenced by: Stays effective and steady under pressure, and models a sustainable pace the team learns from watching, not from posters. Scope: one team.</t>
         </is>
       </c>
       <c r="H42" s="4" t="inlineStr">
         <is>
-          <t>Depth: Builds resilience into how teams operate across a domain — on-call health, recovery time after pushes, load balancing between teams — and repairs burnout risk at scale. Scope: cross-team operating norms.</t>
+          <t>Depth: Holds up through prolonged pressure — incident sieges, crunch, organizational turbulence — helping the team stay resilient and refusing burnout-driven decisions. Evidenced by: Cancels a planned launch rather than run the team through a second consecutive crunch month, and says why out loud. Scope: a complex / critical team.</t>
         </is>
       </c>
       <c r="I42" s="4" t="inlineStr">
         <is>
-          <t>Depth: Models and protects sustainable pace across a sub-org, including through the leaders they develop; pace and recovery are designed into the operating rhythm, not left to heroics. Scope: a sub-org.</t>
+          <t>Depth: Builds resilience into how multiple teams operate — on-call health, recovery after pushes, load balancing — and repairs burnout risk at scale. Evidenced by: Notices two teams in a domain are both quietly running hot and rebalances on-call across them before either loses someone to burnout. Scope: a domain (cross-team).</t>
         </is>
       </c>
       <c r="J42" s="4" t="inlineStr">
         <is>
-          <t>Depth: Stewards organizational resilience at function scale — capacity buffers, crisis rotation, energy management for senior leaders — and holds the line when business pressure argues for permanent crunch. Scope: a function.</t>
+          <t>Depth: Builds resilience into how multiple teams operate — on-call health, recovery after pushes, load balancing — and repairs burnout risk at scale. Evidenced by: Models and protects sustainable pace across a sub-org, including through the leaders they develop; pace is designed in, not left to heroics. Scope: a sub-org.</t>
         </is>
       </c>
       <c r="K42" s="4" t="inlineStr">
         <is>
-          <t>Depth: Shapes a resilient, sustainable culture org-wide — the org absorbs shocks without breaking people, and the story of its hardest year is told without casualties as the moral. Scope: org-wide.</t>
+          <t>Depth: Stewards organizational resilience — capacity buffers, crisis rotation, energy management for senior leaders — and holds the line when business pressure argues for permanent crunch. Evidenced by: Pushes back when the business asks for a permanent on-call surge, and gets a capacity buffer funded instead. Scope: a function.</t>
+        </is>
+      </c>
+      <c r="L42" s="4" t="inlineStr">
+        <is>
+          <t>Depth: Shapes a resilient, sustainable culture across an organization; the organization absorbs shocks without breaking people, and the practice is referenced beyond it. Evidenced by: Shapes a resilient, sustainable culture org-wide; the story of the org's hardest year is told without casualties as the moral. Scope: org-wide.</t>
         </is>
       </c>
     </row>
@@ -3129,37 +3340,42 @@
       </c>
       <c r="E43" s="4" t="inlineStr">
         <is>
-          <t>Kahneman, Thinking, Fast and Slow (2011)</t>
+          <t>Makes sound calls with incomplete information.</t>
         </is>
       </c>
       <c r="F43" s="4" t="inlineStr">
         <is>
-          <t>Depth: Sizes the decision process to reversibility — quick calls on two-way doors, written option analysis on one-way doors — states assumptions and confidence levels, and sets a revisit date. Scope: one team's decisions, made at the pace the team needs.</t>
+          <t>Kahneman, Thinking, Fast and Slow (Farrar, Straus and Giroux, 2011) — judgment is systematically biased, and decision quality improves through process, not willpower</t>
         </is>
       </c>
       <c r="G43" s="4" t="inlineStr">
         <is>
-          <t>Depth: Structures high-stakes calls on incomplete data — options written, disconfirming evidence sought, dissent solicited before their own view is stated — names tripwires that trigger revisits and kills their own sunk-cost projects. Scope: a critical team's one-way doors.</t>
+          <t>Depth: Decides independently within their components; evaluates alternatives honestly. Evidenced by: Sizes the decision process to reversibility, stating assumptions and confidence levels and setting a revisit date. Scope: one team.</t>
         </is>
       </c>
       <c r="H43" s="4" t="inlineStr">
         <is>
-          <t>Depth: Installs debiasing mechanics across a domain — pre-mortems, red teams, decision journals reviewed against outcomes — and clarifies who decides what so cross-team decisions stop stalling in consensus. Scope: cross-team decision quality.</t>
+          <t>Depth: Makes architectural choices for a domain that hold up over months. Evidenced by: Structures high-stakes calls on incomplete data, naming tripwires that trigger revisits and killing their own sunk-cost projects. Scope: a complex / critical team.</t>
         </is>
       </c>
       <c r="I43" s="4" t="inlineStr">
         <is>
-          <t>Depth: Calibrates a sub-org's risk appetite decision by decision — pushes gamble-shy teams to bet and bet-happy teams to check — using a scored decision record, and separates decision quality from outcome luck in reviews. Scope: a sub-org's judgment culture.</t>
+          <t>Depth: Foresees second-order consequences; sets decision frameworks for teams. Evidenced by: Installs debiasing mechanics across a domain -- pre-mortems, decision journals reviewed against outcomes -- and clarifies who decides what. Scope: a domain (cross-team).</t>
         </is>
       </c>
       <c r="J43" s="4" t="inlineStr">
         <is>
-          <t>Depth: Makes function-level bets under genuine ambiguity — market shifts, platform discontinuities — sized so being wrong is survivable, showing the reasoning so the function learns even when the bet loses. Scope: a function.</t>
+          <t>Depth: Foresees second-order consequences; sets decision frameworks for teams. Evidenced by: Calibrates a sub-org's risk appetite decision by decision, using a scored decision record and separating decision quality from outcome luck. Scope: a sub-org.</t>
         </is>
       </c>
       <c r="K43" s="4" t="inlineStr">
         <is>
-          <t>Depth: Carries the org's irreversible decisions — the ones with no consensus and no precedent — with a process others trust even when they disagree with the call, and reserves only the genuine one-way doors. Scope: org-wide consequence.</t>
+          <t>Depth: Sets decision-making frameworks for the org. Evidenced by: Makes function-level bets under genuine ambiguity, sized so being wrong is survivable, showing the reasoning even when the bet loses. Scope: a function.</t>
+        </is>
+      </c>
+      <c r="L43" s="4" t="inlineStr">
+        <is>
+          <t>Depth: Visionary judgment; sees structural causes others miss. Evidenced by: Carries the org's irreversible decisions -- the ones with no consensus and no precedent -- with a process others trust even when they disagree. Scope: org-wide.</t>
         </is>
       </c>
     </row>
@@ -3186,37 +3402,42 @@
       </c>
       <c r="E44" s="4" t="inlineStr">
         <is>
-          <t>Mayer, Davis &amp; Schoorman (1995); ACM Code of Ethics (2018)</t>
+          <t>Earns and keeps trust through consistency and courage — keeping commitments, telling unwelcome truths, and holding the ethical line when it is costly.</t>
         </is>
       </c>
       <c r="F44" s="4" t="inlineStr">
         <is>
-          <t>Depth: Keeps commitments or renegotiates them before the deadline, never after — says the same thing in the room and out of it, owns mistakes unprompted, and tells stakeholders the true state of the project when the truth is unwelcome. Scope: one team's trust in its manager.</t>
+          <t>Mayer, Davis &amp; Schoorman, An Integrative Model of Organizational Trust, Academy of Management Review 20(3), 709-734 (1995) — trust is granted on perceived ability, benevolence, and integrity, and a leader's word is the currency every other competency spends</t>
         </is>
       </c>
       <c r="G44" s="4" t="inlineStr">
         <is>
-          <t>Depth: Holds the quality or safety line on a critical system under senior pressure — makes the unpopular-but-right call and absorbs the cost personally, protecting the engineer who raised the flag; handles sensitive information impeccably. Scope: a critical system's integrity.</t>
+          <t>Depth: Makes the unpopular-but-right call under pressure and absorbs the cost personally; protects the person who raised the flag and handles sensitive information impeccably. Evidenced by: Keeps commitments or renegotiates them before the deadline, never after, and owns mistakes unprompted. Scope: one team.</t>
         </is>
       </c>
       <c r="H44" s="4" t="inlineStr">
         <is>
-          <t>Depth: Serves as the honest broker across a domain — parties in a dispute accept their account of the facts — and carries uncomfortable systemic truths to the room where they can be fixed. Scope: cross-team credibility and ethical tone.</t>
+          <t>Depth: Makes the unpopular-but-right call under pressure and absorbs the cost personally; protects the person who raised the flag and handles sensitive information impeccably. Evidenced by: Holds the quality or safety line on a critical system under senior pressure, and protects the engineer who raised the flag. Scope: a complex / critical team.</t>
         </is>
       </c>
       <c r="I44" s="4" t="inlineStr">
         <is>
-          <t>Depth: Builds the mechanisms that make integrity cheap in a sub-org — ethics review in design, safe escalation with follow-through, fairness systems whose losers affirm the process — and applies them to their own decisions first. Scope: a sub-org's institutional fairness.</t>
+          <t>Depth: Serves as the honest broker across teams — disputing parties accept their account of the facts — and carries uncomfortable systemic truths to the room that can fix them. Evidenced by: Serves as the honest broker across a domain -- parties in a dispute accept their account of the facts. Scope: a domain (cross-team).</t>
         </is>
       </c>
       <c r="J44" s="4" t="inlineStr">
         <is>
-          <t>Depth: Stops function-level launches on ethical or safety grounds and defends the call upward with the business case for trust; corrects the record when convenient narratives are wrong. Scope: a function's public impact.</t>
+          <t>Depth: Serves as the honest broker across teams — disputing parties accept their account of the facts — and carries uncomfortable systemic truths to the room that can fix them. Evidenced by: Builds the mechanisms that make integrity cheap in a sub-org, and applies them to their own decisions first. Scope: a sub-org.</t>
         </is>
       </c>
       <c r="K44" s="4" t="inlineStr">
         <is>
-          <t>Depth: Holds the org's line with the board, investors, and market when the profitable path and the right path diverge — walks away from revenue, ships the hard disclosure — and how they handle the worst moments becomes the story the culture tells about itself. Scope: org-wide conscience, for years.</t>
+          <t>Depth: Builds mechanisms that make integrity cheap at scale — ethics review in design, safe escalation with follow-through, fairness systems whose losers affirm the process — and stops launches on ethical grounds with the business case for trust. Evidenced by: Stops function-level launches on ethical or safety grounds and defends the call upward with the business case for trust. Scope: a function.</t>
+        </is>
+      </c>
+      <c r="L44" s="4" t="inlineStr">
+        <is>
+          <t>Depth: Holds an organization's line when the profitable path and the right path diverge — the hard disclosure, the walked-away revenue — and those moments become the story the culture tells about itself. Evidenced by: Holds the org's line with the board and market when the profitable path and the right path diverge, and walks away from revenue. Scope: org-wide.</t>
         </is>
       </c>
     </row>
@@ -3420,7 +3641,7 @@
         <v>4</v>
       </c>
       <c r="M4" s="2" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="N4" s="2" t="n">
         <v>5</v>
@@ -3465,7 +3686,7 @@
         <v>4</v>
       </c>
       <c r="M5" s="2" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="N5" s="2" t="n">
         <v>5</v>
@@ -3932,7 +4153,7 @@
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>Process Design &amp; Continuous Improvement</t>
+          <t>Process &amp; Continuous Improvement</t>
         </is>
       </c>
       <c r="C16" s="2">
@@ -4787,7 +5008,7 @@
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>Technical Debt &amp; Risk Stewardship</t>
+          <t>Technical Debt &amp; Modernization</t>
         </is>
       </c>
       <c r="C35" s="2">
@@ -5330,424 +5551,1442 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A59"/>
+  <dimension ref="A1:D96"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="110" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="70" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="3" max="3"/>
+    <col width="45" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Sources</t>
+          <t>Framework</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Source</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Grounds</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Link</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="4" t="inlineStr">
         <is>
-          <t>ACM Code of Ethics and Professional Conduct (2018)</t>
+          <t>Strategy kernel (diagnosis, guiding policy, coherent action) as the test for real vs. bad strategy</t>
+        </is>
+      </c>
+      <c r="B2" s="4" t="inlineStr">
+        <is>
+          <t>Rumelt, Good Strategy Bad Strategy: The Difference and Why It Matters (Crown Business, 2011)</t>
+        </is>
+      </c>
+      <c r="C2" s="4" t="inlineStr">
+        <is>
+          <t>Strategy Formulation</t>
+        </is>
+      </c>
+      <c r="D2" s="4" t="inlineStr">
+        <is>
+          <t>https://www.penguinrandomhouse.com/books/198888/good-strategy-bad-strategy-by-richard-p-rumelt/</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="4" t="inlineStr">
         <is>
-          <t>Beyer, Jones, Petoff &amp; Murphy (eds.), Site Reliability Engineering: How Google Runs Production Systems (2016)</t>
+          <t>Published OKR mechanics (committed vs aspirational, cascading); anchors planning-cascade leveling</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>Doerr, Measure What Matters: How Google, Bono, and the Gates Foundation Rock the World with OKRs (Portfolio/Penguin, 2018)</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>Vision &amp; Goal Alignment</t>
+        </is>
+      </c>
+      <c r="D3" s="4" t="inlineStr">
+        <is>
+          <t>https://www.whatmatters.com/</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="4" t="inlineStr">
         <is>
-          <t>Brooks, The Mythical Man-Month (1975)</t>
+          <t>Eight-step model for leading organizational change through to durable adoption</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>Kotter, Leading Change (Harvard Business School Press, 1996)</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>Leading Change</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t>https://openlibrary.org/books/OL982607M/Leading_Change</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>Bungay, The Art of Action (2011)</t>
-        </is>
-      </c>
+          <t>Team boundaries; org-level team formation patterns</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>Skelton &amp; Pais, Team Topologies (IT Revolution, 2019)</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>Organizational &amp; Team Design</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>Cagan, Inspired: How to Create Products Customers Love (2008)</t>
-        </is>
-      </c>
+          <t>Directed opportunism / mission command applied to business execution across org gaps</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>Bungay, The Art of Action: How Leaders Close the Gaps between Plans, Actions and Results (Nicholas Brealey, 2011)</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>Driving Alignment &amp; Decision Clarity</t>
+        </is>
+      </c>
+      <c r="D6" s="4" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>Charan, Drotter &amp; Noel, The Leadership Pipeline (2001)</t>
-        </is>
-      </c>
+          <t>Origin of the Situational Leadership model: directing/coaching/supporting/delegating matched to follower readiness</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>Hersey &amp; Blanchard, Management of Organizational Behavior: Utilizing Human Resources (Prentice-Hall, 1969)</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>Situational &amp; Adaptive Leadership</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t>Cialdini, Influence: The Psychology of Persuasion (1984)</t>
+          <t>Estimation as a probabilistic forecast to calibrate, distinct from Code Complete</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>McConnell, Software Estimation: Demystifying the Black Art (Microsoft Press, 2006)</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="inlineStr">
+        <is>
+          <t>Planning &amp; Estimation</t>
+        </is>
+      </c>
+      <c r="D8" s="4" t="inlineStr">
+        <is>
+          <t>https://www.construx.com/store/software-estimation-demystifying-the-black-art/</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>CircleCI Engineering Competency Matrix (CC BY 4.0) — prose-register reference</t>
-        </is>
-      </c>
+          <t>Cost-of-delay and queueing-theory economics for prioritization decisions; verified via web search</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>Reinertsen, The Principles of Product Development Flow: Second Generation Lean Product Development (Celeritas, 2009)</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="inlineStr">
+        <is>
+          <t>Prioritization &amp; Trade-offs</t>
+        </is>
+      </c>
+      <c r="D9" s="4" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
         <is>
-          <t>Cohen &amp; Bradford, Influence Without Authority (1989)</t>
+          <t>Empirical linkage between deployment/release engineering maturity and organizational performance</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <t>Forsgren, Humble &amp; Kim, Accelerate: The Science of Lean Software and DevOps (IT Revolution Press, 2018)</t>
+        </is>
+      </c>
+      <c r="C10" s="4" t="inlineStr">
+        <is>
+          <t>Predictable Delivery &amp; Execution</t>
+        </is>
+      </c>
+      <c r="D10" s="4" t="inlineStr">
+        <is>
+          <t>https://itrevolution.com/product/accelerate/</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
         <is>
-          <t>Collins &amp; Porras, "Building Your Company's Vision" (Harvard Business Review, 1996)</t>
+          <t>Google's published postmortem/root-cause and diagnostic-tooling practice; anchors debugging leveling</t>
+        </is>
+      </c>
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t>Beyer, Jones, Petoff &amp; Murphy (eds.), Site Reliability Engineering: How Google Runs Production Systems (O'Reilly/Google, 2016)</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="inlineStr">
+        <is>
+          <t>Incident &amp; Reliability Leadership</t>
+        </is>
+      </c>
+      <c r="D11" s="4" t="inlineStr">
+        <is>
+          <t>https://sre.google/sre-book/table-of-contents/</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
         <is>
-          <t>Conway, "How Do Committees Invent?" (Datamation, 1968)</t>
+          <t>Six-function (incl. Govern) taxonomy for organizing enterprise cybersecurity risk strategy</t>
+        </is>
+      </c>
+      <c r="B12" s="4" t="inlineStr">
+        <is>
+          <t>NIST, The NIST Cybersecurity Framework (CSF) 2.0, NIST CSWP 29 (2024)</t>
+        </is>
+      </c>
+      <c r="C12" s="4" t="inlineStr">
+        <is>
+          <t>Risk Management &amp; Governance</t>
+        </is>
+      </c>
+      <c r="D12" s="4" t="inlineStr">
+        <is>
+          <t>https://csrc.nist.gov/pubs/cswp/29/the-nist-cybersecurity-framework-csf-20/final</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
         <is>
-          <t>Cunningham, "The WyCash Portfolio Management System" (OOPSLA, 1992)</t>
-        </is>
-      </c>
+          <t>14 points for management; continuous, systemic process improvement over inspection</t>
+        </is>
+      </c>
+      <c r="B13" s="4" t="inlineStr">
+        <is>
+          <t>Deming, Out of the Crisis (MIT Center for Advanced Engineering Study, 1986)</t>
+        </is>
+      </c>
+      <c r="C13" s="4" t="inlineStr">
+        <is>
+          <t>Process &amp; Continuous Improvement</t>
+        </is>
+      </c>
+      <c r="D13" s="4" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="4" t="inlineStr">
         <is>
-          <t>Deci &amp; Ryan, "Self-Determination Theory and the Facilitation of Intrinsic Motivation, Social Development, and Well-Being" (American Psychologist, 2000)</t>
+          <t>SPACE framework for developer productivity/DX measurement; 403 on automated fetch (bot-blocked) but title/venue confirmed via web search</t>
+        </is>
+      </c>
+      <c r="B14" s="4" t="inlineStr">
+        <is>
+          <t>Forsgren, Storey, Maddila, Zimmermann, Houck &amp; Butler, The SPACE of Developer Productivity, ACM Queue 19(1) (2021)</t>
+        </is>
+      </c>
+      <c r="C14" s="4" t="inlineStr">
+        <is>
+          <t>Developer Experience &amp; Flow</t>
+        </is>
+      </c>
+      <c r="D14" s="4" t="inlineStr">
+        <is>
+          <t>https://queue.acm.org/detail.cfm?id=3454124</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
         <is>
-          <t>Deming, Out of the Crisis (1986)</t>
+          <t>Adding manpower to a late project makes it later; coordination cost scales with headcount</t>
+        </is>
+      </c>
+      <c r="B15" s="4" t="inlineStr">
+        <is>
+          <t>Brooks, The Mythical Man-Month: Essays on Software Engineering, Anniversary ed. (Addison-Wesley, 1995; orig. 1975)</t>
+        </is>
+      </c>
+      <c r="C15" s="4" t="inlineStr">
+        <is>
+          <t>Capacity &amp; Headcount Planning</t>
+        </is>
+      </c>
+      <c r="D15" s="4" t="inlineStr">
+        <is>
+          <t>https://en.wikipedia.org/wiki/The_Mythical_Man-Month</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="4" t="inlineStr">
         <is>
-          <t>Drucker, The Effective Executive (1967)</t>
+          <t>38-competency leadership model incl. Financial Acumen; industry-standard leveling reference</t>
+        </is>
+      </c>
+      <c r="B16" s="4" t="inlineStr">
+        <is>
+          <t>Korn Ferry, Korn Ferry Leadership Architect Global Competency Framework (2014)</t>
+        </is>
+      </c>
+      <c r="C16" s="4" t="inlineStr">
+        <is>
+          <t>Budget &amp; Vendor Stewardship</t>
+        </is>
+      </c>
+      <c r="D16" s="4" t="inlineStr">
+        <is>
+          <t>https://www.kornferry.com/capabilities/talent-suite/korn-ferry-assess/leadership-architect</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="4" t="inlineStr">
         <is>
-          <t>Duarte, HBR Guide to Persuasive Presentations (2012)</t>
-        </is>
-      </c>
+          <t>Meta-analysis of 85 years of selection-method validity; grounds structured, evidence-based hiring judgment</t>
+        </is>
+      </c>
+      <c r="B17" s="4" t="inlineStr">
+        <is>
+          <t>Schmidt &amp; Hunter, The Validity and Utility of Selection Methods in Personnel Psychology, Psychological Bulletin 124(2), 262-274 (1998)</t>
+        </is>
+      </c>
+      <c r="C17" s="4" t="inlineStr">
+        <is>
+          <t>Hiring &amp; Selection</t>
+        </is>
+      </c>
+      <c r="D17" s="4" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="4" t="inlineStr">
         <is>
-          <t>Edmondson, The Fearless Organization (2018)</t>
+          <t>Forming-storming-norming-performing team stages</t>
+        </is>
+      </c>
+      <c r="B18" s="4" t="inlineStr">
+        <is>
+          <t>Tuckman, Developmental Sequence in Small Groups, Psychological Bulletin 63(6), 384-399 (1965)</t>
+        </is>
+      </c>
+      <c r="C18" s="4" t="inlineStr">
+        <is>
+          <t>Onboarding &amp; Team Formation</t>
+        </is>
+      </c>
+      <c r="D18" s="4" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1037/h0022100</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="4" t="inlineStr">
         <is>
-          <t>Ely &amp; Thomas, "Cultural Diversity at Work" (Administrative Science Quarterly, 2001)</t>
+          <t>GROW model; origin of the coach-not-tell manager stance</t>
+        </is>
+      </c>
+      <c r="B19" s="4" t="inlineStr">
+        <is>
+          <t>Whitmore, Coaching for Performance: GROWing Human Potential and Purpose, 4th ed. (Nicholas Brealey, 2009; orig. 1992)</t>
+        </is>
+      </c>
+      <c r="C19" s="4" t="inlineStr">
+        <is>
+          <t>Coaching &amp; Development</t>
+        </is>
+      </c>
+      <c r="D19" s="4" t="inlineStr">
+        <is>
+          <t>https://www.nicholasbrealey.com/coaching-for-performance/</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="4" t="inlineStr">
         <is>
-          <t>Eurich, Insight (2017)</t>
+          <t>Care-personally/challenge-directly feedback culture model; grounds org-scale feedback-culture leveling</t>
+        </is>
+      </c>
+      <c r="B20" s="4" t="inlineStr">
+        <is>
+          <t>Scott, Radical Candor: Be a Kick-Ass Boss Without Losing Your Humanity (St. Martin's Press, 2017)</t>
+        </is>
+      </c>
+      <c r="C20" s="4" t="inlineStr">
+        <is>
+          <t>Listening &amp; Feedback</t>
+        </is>
+      </c>
+      <c r="D20" s="4" t="inlineStr">
+        <is>
+          <t>https://www.radicalcandor.com/</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="4" t="inlineStr">
         <is>
-          <t>Fisher &amp; Ury, Getting to Yes (1981)</t>
+          <t>Origin of management-by-objectives cascading goal-setting that OKRs formalize</t>
+        </is>
+      </c>
+      <c r="B21" s="4" t="inlineStr">
+        <is>
+          <t>Grove, High Output Management (Random House, 1983)</t>
+        </is>
+      </c>
+      <c r="C21" s="4" t="inlineStr">
+        <is>
+          <t>Performance Management</t>
+        </is>
+      </c>
+      <c r="D21" s="4" t="inlineStr">
+        <is>
+          <t>https://www.penguinrandomhouse.com/books/163289/high-output-management-by-andrew-s-grove/</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="4" t="inlineStr">
         <is>
-          <t>Forsgren, Humble &amp; Kim, Accelerate: The Science of Lean Software and DevOps (2018)</t>
+          <t>Distinguishes sponsorship (advocacy, reputational risk) from mentorship (advice)</t>
+        </is>
+      </c>
+      <c r="B22" s="4" t="inlineStr">
+        <is>
+          <t>Hewlett, Forget a Mentor, Find a Sponsor: The New Way to Fast-Track Your Career (Harvard Business Review Press, 2013)</t>
+        </is>
+      </c>
+      <c r="C22" s="4" t="inlineStr">
+        <is>
+          <t>Career Development &amp; Sponsorship</t>
+        </is>
+      </c>
+      <c r="D22" s="4" t="inlineStr">
+        <is>
+          <t>https://www.barnesandnoble.com/w/forget-a-mentor-find-a-sponsor-sylvia-ann-hewlett/1114264520</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="4" t="inlineStr">
         <is>
-          <t>Forsgren et al., "The SPACE of Developer Productivity" (ACM Queue, 2021)</t>
+          <t>Six leadership 'passages' model; anchors talent-management and succession leveling</t>
+        </is>
+      </c>
+      <c r="B23" s="4" t="inlineStr">
+        <is>
+          <t>Charan, Drotter &amp; Noel, The Leadership Pipeline: How to Build the Leadership-Powered Company, 2nd Edition (Jossey-Bass, 2010)</t>
+        </is>
+      </c>
+      <c r="C23" s="4" t="inlineStr">
+        <is>
+          <t>Succession &amp; Leadership Pipeline</t>
+        </is>
+      </c>
+      <c r="D23" s="4" t="inlineStr">
+        <is>
+          <t>https://www.wiley.com/en-us/The+Leadership+Pipeline%3A+How+to+Build+the+Leadership-Powered+Company-p-9780787958527</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="4" t="inlineStr">
         <is>
-          <t>Fournier, The Manager's Path (2017)</t>
+          <t>Practitioner-facing extension of Edmondson's 1999 psychological-safety research to team leadership practice</t>
+        </is>
+      </c>
+      <c r="B24" s="4" t="inlineStr">
+        <is>
+          <t>Edmondson, The Fearless Organization: Creating Psychological Safety in the Workplace for Learning, Innovation, and Growth (Wiley, 2018)</t>
+        </is>
+      </c>
+      <c r="C24" s="4" t="inlineStr">
+        <is>
+          <t>Psychological Safety</t>
+        </is>
+      </c>
+      <c r="D24" s="4" t="inlineStr">
+        <is>
+          <t>https://www.wiley.com/en-us/The+Fearless+Organization%3A+Creating+Psychological+Safety+in+the+Workplace+for+Learning%2C+Innovation%2C+and+Growth-p-9781119477242</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="4" t="inlineStr">
         <is>
-          <t>Freeman, Strategic Management: A Stakeholder Approach (1984)</t>
+          <t>Autonomy, competence, relatedness drive durable engagement over extrinsic reward</t>
+        </is>
+      </c>
+      <c r="B25" s="4" t="inlineStr">
+        <is>
+          <t>Deci &amp; Ryan, The "What" and "Why" of Goal Pursuits: Human Needs and the Self-Determination of Behavior, Psychological Inquiry 11(4), 227-268 (2000)</t>
+        </is>
+      </c>
+      <c r="C25" s="4" t="inlineStr">
+        <is>
+          <t>Motivation, Engagement &amp; Retention</t>
+        </is>
+      </c>
+      <c r="D25" s="4" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1207/S15327965PLI1104_01</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="4" t="inlineStr">
         <is>
-          <t>Goldratt, The Goal (1984)</t>
+          <t>Connection timeout on automated fetch (blocked in this environment) but title/publisher/content confirmed via web search across mckinsey.com itself and multiple independent citing sources; anchors DEI leveling</t>
+        </is>
+      </c>
+      <c r="B26" s="4" t="inlineStr">
+        <is>
+          <t>Hunt, Prince, Dixon-Fyle &amp; Yee, Diversity Wins: How Inclusion Matters (McKinsey &amp; Company, 2020)</t>
+        </is>
+      </c>
+      <c r="C26" s="4" t="inlineStr">
+        <is>
+          <t>Inclusion &amp; Belonging</t>
+        </is>
+      </c>
+      <c r="D26" s="4" t="inlineStr">
+        <is>
+          <t>https://www.mckinsey.com/featured-insights/diversity-and-inclusion/diversity-wins-interactive</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="4" t="inlineStr">
         <is>
-          <t>Google re:Work, Project Aristotle team-effectiveness study (2015) — corroborates the Psychological Safety anchor</t>
+          <t>Progression from tech lead credibility through senior engineering leadership</t>
+        </is>
+      </c>
+      <c r="B27" s="4" t="inlineStr">
+        <is>
+          <t>Fournier, The Manager's Path (O'Reilly, 2017)</t>
+        </is>
+      </c>
+      <c r="C27" s="4" t="inlineStr">
+        <is>
+          <t>Technical Credibility</t>
+        </is>
+      </c>
+      <c r="D27" s="4" t="inlineStr">
+        <is>
+          <t>https://www.oreilly.com/library/view/the-managers-path/9781491973882/</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="4" t="inlineStr">
         <is>
-          <t>Google re:Work, Project Oxygen manager-behaviors study (2008) — corroborates the Coaching &amp; Development anchor</t>
+          <t>Sizing teams, technical strategy, and org design for engineering leadership</t>
+        </is>
+      </c>
+      <c r="B28" s="4" t="inlineStr">
+        <is>
+          <t>Larson, An Elegant Puzzle: Systems of Engineering Management (Stripe Press, 2019)</t>
+        </is>
+      </c>
+      <c r="C28" s="4" t="inlineStr">
+        <is>
+          <t>Technical Strategy &amp; Investment</t>
+        </is>
+      </c>
+      <c r="D28" s="4" t="inlineStr">
+        <is>
+          <t>https://press.stripe.com/an-elegant-puzzle</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="4" t="inlineStr">
         <is>
-          <t>Grove, High Output Management (1983)</t>
+          <t>SVPG discovery-risk framework (value/usability/feasibility/viability); PM domain-expertise and discovery-judgment anchor</t>
+        </is>
+      </c>
+      <c r="B29" s="4" t="inlineStr">
+        <is>
+          <t>Cagan, INSPIRED: How to Create Tech Products Customers Love, 2nd Edition (Wiley, 2018)</t>
+        </is>
+      </c>
+      <c r="C29" s="4" t="inlineStr">
+        <is>
+          <t>Domain &amp; Business Fluency</t>
+        </is>
+      </c>
+      <c r="D29" s="4" t="inlineStr">
+        <is>
+          <t>https://www.svpg.com/inspired-2nd-edition/</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="4" t="inlineStr">
         <is>
-          <t>Heifetz, Leadership Without Easy Answers (1994)</t>
+          <t>Conway's Law: system design mirrors the communication structure of the organization that builds it</t>
+        </is>
+      </c>
+      <c r="B30" s="4" t="inlineStr">
+        <is>
+          <t>Conway, How Do Committees Invent?, Datamation 14(4), 28-31 (1968)</t>
+        </is>
+      </c>
+      <c r="C30" s="4" t="inlineStr">
+        <is>
+          <t>Architecture &amp; Decision Oversight</t>
+        </is>
+      </c>
+      <c r="D30" s="4" t="inlineStr">
+        <is>
+          <t>https://www.melconway.com/Home/Committees_Paper.html</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="4" t="inlineStr">
         <is>
-          <t>Hersey &amp; Blanchard, Management of Organizational Behavior (1969)</t>
+          <t>Deployment pipeline environment-parity and release-automation discipline</t>
+        </is>
+      </c>
+      <c r="B31" s="4" t="inlineStr">
+        <is>
+          <t>Humble &amp; Farley, Continuous Delivery: Reliable Software Releases through Build Test and Deployment Automation (Addison-Wesley, 2010)</t>
+        </is>
+      </c>
+      <c r="C31" s="4" t="inlineStr">
+        <is>
+          <t>Engineering Standards &amp; Quality</t>
+        </is>
+      </c>
+      <c r="D31" s="4" t="inlineStr">
+        <is>
+          <t>https://continuousdelivery.com/</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="4" t="inlineStr">
         <is>
-          <t>Herzberg, "One More Time: How Do You Motivate Employees?" (Harvard Business Review, 1968)</t>
+          <t>Origin of the technical-debt metaphor (principal and accruing interest)</t>
+        </is>
+      </c>
+      <c r="B32" s="4" t="inlineStr">
+        <is>
+          <t>Cunningham, The WyCash Portfolio Management System, OOPSLA 1992 Experience Report</t>
+        </is>
+      </c>
+      <c r="C32" s="4" t="inlineStr">
+        <is>
+          <t>Technical Debt &amp; Modernization</t>
+        </is>
+      </c>
+      <c r="D32" s="4" t="inlineStr">
+        <is>
+          <t>https://c2.com/doc/oopsla92.html</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="4" t="inlineStr">
         <is>
-          <t>Hewlett, Forget a Mentor, Find a Sponsor (2013)</t>
+          <t>Answer-first, structured argument method; grounds executive-communication and design-doc leveling</t>
+        </is>
+      </c>
+      <c r="B33" s="4" t="inlineStr">
+        <is>
+          <t>Minto, The Minto Pyramid Principle: Logic in Writing, Thinking, and Problem Solving (Minto International, 1996)</t>
+        </is>
+      </c>
+      <c r="C33" s="4" t="inlineStr">
+        <is>
+          <t>Written &amp; Verbal Communication</t>
+        </is>
+      </c>
+      <c r="D33" s="4" t="inlineStr">
+        <is>
+          <t>https://www.barbaraminto.com/</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="4" t="inlineStr">
         <is>
-          <t>Humble &amp; Farley, Continuous Delivery (2010)</t>
+          <t>Structuring executive communication around audience needs, not speaker content</t>
+        </is>
+      </c>
+      <c r="B34" s="4" t="inlineStr">
+        <is>
+          <t>Duarte, HBR Guide to Persuasive Presentations (Harvard Business Review Press, 2012)</t>
+        </is>
+      </c>
+      <c r="C34" s="4" t="inlineStr">
+        <is>
+          <t>Executive &amp; Upward Communication</t>
+        </is>
+      </c>
+      <c r="D34" s="4" t="inlineStr">
+        <is>
+          <t>https://store.hbr.org/product/hbr-guide-to-persuasive-presentations/10058</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="4" t="inlineStr">
         <is>
-          <t>Kahneman, Thinking, Fast and Slow (2011)</t>
-        </is>
-      </c>
+          <t>Origin of stakeholder theory: managing for groups who affect or are affected by the organization</t>
+        </is>
+      </c>
+      <c r="B35" s="4" t="inlineStr">
+        <is>
+          <t>Freeman, Strategic Management: A Stakeholder Approach (Pitman, 1984)</t>
+        </is>
+      </c>
+      <c r="C35" s="4" t="inlineStr">
+        <is>
+          <t>Stakeholder Management &amp; Partnership</t>
+        </is>
+      </c>
+      <c r="D35" s="4" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" s="4" t="inlineStr">
         <is>
-          <t>Korn Ferry Leadership Architect competency library (2014) — comparison overlay only</t>
+          <t>Exchange Model of influence: trading in others' currencies absent formal authority</t>
+        </is>
+      </c>
+      <c r="B36" s="4" t="inlineStr">
+        <is>
+          <t>Cohen &amp; Bradford, Influence Without Authority, 3rd ed. (Wiley, 2017)</t>
+        </is>
+      </c>
+      <c r="C36" s="4" t="inlineStr">
+        <is>
+          <t>Influence Without Authority</t>
+        </is>
+      </c>
+      <c r="D36" s="4" t="inlineStr">
+        <is>
+          <t>https://www.wiley.com/en-us/Influence+Without+Authority,+3rd+Edition-p-9781119347712</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="4" t="inlineStr">
         <is>
-          <t>Kotter, Leading Change (1996); "What Leaders Really Do" (Harvard Business Review, 1990)</t>
+          <t>Principled negotiation: separating people from the problem, interests versus positions</t>
+        </is>
+      </c>
+      <c r="B37" s="4" t="inlineStr">
+        <is>
+          <t>Fisher &amp; Ury, Getting to Yes: Negotiating Agreement Without Giving In (Penguin, 1981)</t>
+        </is>
+      </c>
+      <c r="C37" s="4" t="inlineStr">
+        <is>
+          <t>Conflict Resolution &amp; Negotiation</t>
+        </is>
+      </c>
+      <c r="D37" s="4" t="inlineStr">
+        <is>
+          <t>https://www.pon.harvard.edu/shop/getting-to-yes-negotiating-agreement-without-giving-in/</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="4" t="inlineStr">
         <is>
-          <t>Larson, An Elegant Puzzle: Systems of Engineering Management (2019)</t>
-        </is>
-      </c>
+          <t>Leader-leader model: pushing authority and decision rights down to where the information is</t>
+        </is>
+      </c>
+      <c r="B38" s="4" t="inlineStr">
+        <is>
+          <t>Marquet, Turn the Ship Around!: A True Story of Turning Followers into Leaders (Portfolio/Penguin, 2013; orig. 2012)</t>
+        </is>
+      </c>
+      <c r="C38" s="4" t="inlineStr">
+        <is>
+          <t>Delegation &amp; Empowerment</t>
+        </is>
+      </c>
+      <c r="D38" s="4" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" s="4" t="inlineStr">
         <is>
-          <t>Lencioni, The Five Dysfunctions of a Team (2002)</t>
+          <t>Internal/external self-awareness distinction; feedback-seeking research across ~5,000 participants</t>
+        </is>
+      </c>
+      <c r="B39" s="4" t="inlineStr">
+        <is>
+          <t>Eurich, What Self-Awareness Really Is (and How to Cultivate It), Harvard Business Review (2018)</t>
+        </is>
+      </c>
+      <c r="C39" s="4" t="inlineStr">
+        <is>
+          <t>Self-Awareness &amp; Learning Agility</t>
+        </is>
+      </c>
+      <c r="D39" s="4" t="inlineStr">
+        <is>
+          <t>https://hbr.org/2018/01/what-self-awareness-really-is-and-how-to-cultivate-it</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="4" t="inlineStr">
         <is>
-          <t>Locke &amp; Latham, "Building a Practically Useful Theory of Goal Setting and Task Motivation" (American Psychologist, 2002)</t>
-        </is>
-      </c>
+          <t>Sustainable performance managed through energy (physical, emotional, mental, spiritual), not just time</t>
+        </is>
+      </c>
+      <c r="B40" s="4" t="inlineStr">
+        <is>
+          <t>Loehr &amp; Schwartz, The Power of Full Engagement: Managing Energy, Not Time, Is the Key to High Performance and Personal Renewal (Free Press, 2003)</t>
+        </is>
+      </c>
+      <c r="C40" s="4" t="inlineStr">
+        <is>
+          <t>Resilience &amp; Sustainable Pace</t>
+        </is>
+      </c>
+      <c r="D40" s="4" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" s="4" t="inlineStr">
         <is>
-          <t>Loehr &amp; Schwartz, The Power of Full Engagement (2003)</t>
+          <t>System 1 / System 2 reasoning; basis for structured decision-making under uncertainty</t>
+        </is>
+      </c>
+      <c r="B41" s="4" t="inlineStr">
+        <is>
+          <t>Kahneman, Thinking, Fast and Slow (Farrar, Straus and Giroux, 2011)</t>
+        </is>
+      </c>
+      <c r="C41" s="4" t="inlineStr">
+        <is>
+          <t>Decision-Making Under Uncertainty</t>
+        </is>
+      </c>
+      <c r="D41" s="4" t="inlineStr">
+        <is>
+          <t>https://en.wikipedia.org/wiki/Thinking,_Fast_and_Slow</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="4" t="inlineStr">
         <is>
-          <t>Lombardo &amp; Eichinger, "High Potentials as High Learners" (Human Resource Management, 2000)</t>
+          <t>Ability/benevolence/integrity model of trustworthiness; foundational organizational-trust theory</t>
+        </is>
+      </c>
+      <c r="B42" s="4" t="inlineStr">
+        <is>
+          <t>Mayer, Davis &amp; Schoorman, An Integrative Model of Organizational Trust, Academy of Management Review 20(3), 709-734 (1995)</t>
+        </is>
+      </c>
+      <c r="C42" s="4" t="inlineStr">
+        <is>
+          <t>Ethics, Integrity &amp; Trust</t>
+        </is>
+      </c>
+      <c r="D42" s="4" t="inlineStr">
+        <is>
+          <t>https://people.wku.edu/richard.miller/Mayer%20Trust%20article.pdf</t>
         </is>
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="4" t="inlineStr">
-        <is>
-          <t>Majors, "The Engineer/Manager Pendulum" (2017)</t>
-        </is>
-      </c>
+      <c r="A43" s="4" t="inlineStr"/>
+      <c r="B43" s="4" t="inlineStr">
+        <is>
+          <t>Rumelt, Good Strategy Bad Strategy: The Difference and Why It Matters (Crown Business, 2011) — https://www.penguinrandomhouse.com/books/198888/good-strategy-bad-strategy-by-richard-p-rumelt/</t>
+        </is>
+      </c>
+      <c r="C43" s="4" t="inlineStr"/>
+      <c r="D43" s="4" t="inlineStr"/>
     </row>
     <row r="44">
-      <c r="A44" s="4" t="inlineStr">
-        <is>
-          <t>Marquet, Turn the Ship Around! (2012)</t>
-        </is>
-      </c>
+      <c r="A44" s="4" t="inlineStr"/>
+      <c r="B44" s="4" t="inlineStr">
+        <is>
+          <t>GitLab Handbook, Engineering Management Job Framework (accessed 2026-07) — https://handbook.gitlab.com/job-families/engineering/engineering-management/</t>
+        </is>
+      </c>
+      <c r="C44" s="4" t="inlineStr"/>
+      <c r="D44" s="4" t="inlineStr"/>
     </row>
     <row r="45">
-      <c r="A45" s="4" t="inlineStr">
-        <is>
-          <t>Mayer, Davis &amp; Schoorman, "An Integrative Model of Organizational Trust" (Academy of Management Review, 1995)</t>
-        </is>
-      </c>
+      <c r="A45" s="4" t="inlineStr"/>
+      <c r="B45" s="4" t="inlineStr">
+        <is>
+          <t>Doerr, Measure What Matters: How Google, Bono, and the Gates Foundation Rock the World with OKRs (Portfolio/Penguin, 2018) — https://www.whatmatters.com/</t>
+        </is>
+      </c>
+      <c r="C45" s="4" t="inlineStr"/>
+      <c r="D45" s="4" t="inlineStr"/>
     </row>
     <row r="46">
-      <c r="A46" s="4" t="inlineStr">
-        <is>
-          <t>McConnell, Software Estimation: Demystifying the Black Art (2006)</t>
-        </is>
-      </c>
+      <c r="A46" s="4" t="inlineStr"/>
+      <c r="B46" s="4" t="inlineStr">
+        <is>
+          <t>Kotter, Leading Change (Harvard Business School Press, 1996) — https://openlibrary.org/books/OL982607M/Leading_Change</t>
+        </is>
+      </c>
+      <c r="C46" s="4" t="inlineStr"/>
+      <c r="D46" s="4" t="inlineStr"/>
     </row>
     <row r="47">
-      <c r="A47" s="4" t="inlineStr">
-        <is>
-          <t>Minto, The Pyramid Principle (1987)</t>
-        </is>
-      </c>
+      <c r="A47" s="4" t="inlineStr"/>
+      <c r="B47" s="4" t="inlineStr">
+        <is>
+          <t>Skelton &amp; Pais, Team Topologies (IT Revolution, 2019)</t>
+        </is>
+      </c>
+      <c r="C47" s="4" t="inlineStr"/>
+      <c r="D47" s="4" t="inlineStr"/>
     </row>
     <row r="48">
-      <c r="A48" s="4" t="inlineStr">
-        <is>
-          <t>Mitchell, Agle &amp; Wood, "Toward a Theory of Stakeholder Identification and Salience" (Academy of Management Review, 1997)</t>
-        </is>
-      </c>
+      <c r="A48" s="4" t="inlineStr"/>
+      <c r="B48" s="4" t="inlineStr">
+        <is>
+          <t>Bungay, The Art of Action: How Leaders Close the Gaps between Plans, Actions and Results (Nicholas Brealey, 2011)</t>
+        </is>
+      </c>
+      <c r="C48" s="4" t="inlineStr"/>
+      <c r="D48" s="4" t="inlineStr"/>
     </row>
     <row r="49">
-      <c r="A49" s="4" t="inlineStr">
-        <is>
-          <t>NIST Cybersecurity Framework (2014)</t>
-        </is>
-      </c>
+      <c r="A49" s="4" t="inlineStr"/>
+      <c r="B49" s="4" t="inlineStr">
+        <is>
+          <t>Hersey &amp; Blanchard, Management of Organizational Behavior: Utilizing Human Resources (Prentice-Hall, 1969)</t>
+        </is>
+      </c>
+      <c r="C49" s="4" t="inlineStr"/>
+      <c r="D49" s="4" t="inlineStr"/>
     </row>
     <row r="50">
-      <c r="A50" s="4" t="inlineStr">
-        <is>
-          <t>Nygard, "Documenting Architecture Decisions" (2011)</t>
-        </is>
-      </c>
+      <c r="A50" s="4" t="inlineStr"/>
+      <c r="B50" s="4" t="inlineStr">
+        <is>
+          <t>Heifetz, Grashow &amp; Linsky, The Practice of Adaptive Leadership (Harvard Business Press, 2009) — https://www.hks.harvard.edu/publications/practice-adaptive-leadership-tools-and-tactics-changing-your-organization-and-world</t>
+        </is>
+      </c>
+      <c r="C50" s="4" t="inlineStr"/>
+      <c r="D50" s="4" t="inlineStr"/>
     </row>
     <row r="51">
-      <c r="A51" s="4" t="inlineStr">
-        <is>
-          <t>Project Management Institute, PMBOK Guide (7th edition, 2021)</t>
-        </is>
-      </c>
+      <c r="A51" s="4" t="inlineStr"/>
+      <c r="B51" s="4" t="inlineStr">
+        <is>
+          <t>McConnell, Software Estimation: Demystifying the Black Art (Microsoft Press, 2006) — https://www.construx.com/store/software-estimation-demystifying-the-black-art/</t>
+        </is>
+      </c>
+      <c r="C51" s="4" t="inlineStr"/>
+      <c r="D51" s="4" t="inlineStr"/>
     </row>
     <row r="52">
-      <c r="A52" s="4" t="inlineStr">
-        <is>
-          <t>Reinertsen, The Principles of Product Development Flow (2009)</t>
-        </is>
-      </c>
+      <c r="A52" s="4" t="inlineStr"/>
+      <c r="B52" s="4" t="inlineStr">
+        <is>
+          <t>Reinertsen, The Principles of Product Development Flow: Second Generation Lean Product Development (Celeritas, 2009)</t>
+        </is>
+      </c>
+      <c r="C52" s="4" t="inlineStr"/>
+      <c r="D52" s="4" t="inlineStr"/>
     </row>
     <row r="53">
-      <c r="A53" s="4" t="inlineStr">
-        <is>
-          <t>Rumelt, Good Strategy Bad Strategy (2011)</t>
-        </is>
-      </c>
+      <c r="A53" s="4" t="inlineStr"/>
+      <c r="B53" s="4" t="inlineStr">
+        <is>
+          <t>Forsgren, Humble &amp; Kim, Accelerate: The Science of Lean Software and DevOps (IT Revolution Press, 2018) — https://itrevolution.com/product/accelerate/</t>
+        </is>
+      </c>
+      <c r="C53" s="4" t="inlineStr"/>
+      <c r="D53" s="4" t="inlineStr"/>
     </row>
     <row r="54">
-      <c r="A54" s="4" t="inlineStr">
-        <is>
-          <t>Schmidt &amp; Hunter, "The Validity and Utility of Selection Methods in Personnel Psychology" (Psychological Bulletin, 1998)</t>
-        </is>
-      </c>
+      <c r="A54" s="4" t="inlineStr"/>
+      <c r="B54" s="4" t="inlineStr">
+        <is>
+          <t>Beyer, Jones, Petoff &amp; Murphy (eds.), Site Reliability Engineering: How Google Runs Production Systems (O'Reilly/Google, 2016) — https://sre.google/sre-book/table-of-contents/</t>
+        </is>
+      </c>
+      <c r="C54" s="4" t="inlineStr"/>
+      <c r="D54" s="4" t="inlineStr"/>
     </row>
     <row r="55">
-      <c r="A55" s="4" t="inlineStr">
-        <is>
-          <t>Scott, Radical Candor (2017)</t>
-        </is>
-      </c>
+      <c r="A55" s="4" t="inlineStr"/>
+      <c r="B55" s="4" t="inlineStr">
+        <is>
+          <t>NIST, The NIST Cybersecurity Framework (CSF) 2.0, NIST CSWP 29 (2024) — https://csrc.nist.gov/pubs/cswp/29/the-nist-cybersecurity-framework-csf-20/final</t>
+        </is>
+      </c>
+      <c r="C55" s="4" t="inlineStr"/>
+      <c r="D55" s="4" t="inlineStr"/>
     </row>
     <row r="56">
-      <c r="A56" s="4" t="inlineStr">
-        <is>
-          <t>Skelton &amp; Pais, Team Topologies (2019)</t>
-        </is>
-      </c>
+      <c r="A56" s="4" t="inlineStr"/>
+      <c r="B56" s="4" t="inlineStr">
+        <is>
+          <t>Project Management Institute, A Guide to the Project Management Body of Knowledge (PMBOK Guide), 7th ed. (PMI, 2021) — https://www.pmi.org/standards/pmbok</t>
+        </is>
+      </c>
+      <c r="C56" s="4" t="inlineStr"/>
+      <c r="D56" s="4" t="inlineStr"/>
     </row>
     <row r="57">
-      <c r="A57" s="4" t="inlineStr">
-        <is>
-          <t>Tuckman, "Developmental Sequence in Small Groups" (Psychological Bulletin, 1965)</t>
-        </is>
-      </c>
+      <c r="A57" s="4" t="inlineStr"/>
+      <c r="B57" s="4" t="inlineStr">
+        <is>
+          <t>Forsgren, Storey, Maddila, Zimmermann, Houck &amp; Butler, The SPACE of Developer Productivity, ACM Queue 19(1) (2021) — https://queue.acm.org/detail.cfm?id=3454124</t>
+        </is>
+      </c>
+      <c r="C57" s="4" t="inlineStr"/>
+      <c r="D57" s="4" t="inlineStr"/>
     </row>
     <row r="58">
-      <c r="A58" s="4" t="inlineStr">
-        <is>
-          <t>Wardley, Wardley Maps (2016)</t>
-        </is>
-      </c>
+      <c r="A58" s="4" t="inlineStr"/>
+      <c r="B58" s="4" t="inlineStr">
+        <is>
+          <t>Deming, Out of the Crisis (MIT Center for Advanced Engineering Study, 1986)</t>
+        </is>
+      </c>
+      <c r="C58" s="4" t="inlineStr"/>
+      <c r="D58" s="4" t="inlineStr"/>
     </row>
     <row r="59">
-      <c r="A59" s="4" t="inlineStr">
-        <is>
-          <t>Whitmore, Coaching for Performance (1992)</t>
-        </is>
-      </c>
+      <c r="A59" s="4" t="inlineStr"/>
+      <c r="B59" s="4" t="inlineStr">
+        <is>
+          <t>Brooks, The Mythical Man-Month: Essays on Software Engineering, Anniversary ed. (Addison-Wesley, 1995; orig. 1975) — https://en.wikipedia.org/wiki/The_Mythical_Man-Month</t>
+        </is>
+      </c>
+      <c r="C59" s="4" t="inlineStr"/>
+      <c r="D59" s="4" t="inlineStr"/>
+    </row>
+    <row r="60">
+      <c r="A60" s="4" t="inlineStr"/>
+      <c r="B60" s="4" t="inlineStr">
+        <is>
+          <t>Korn Ferry, Korn Ferry Leadership Architect Global Competency Framework (2014) — https://www.kornferry.com/capabilities/talent-suite/korn-ferry-assess/leadership-architect</t>
+        </is>
+      </c>
+      <c r="C60" s="4" t="inlineStr"/>
+      <c r="D60" s="4" t="inlineStr"/>
+    </row>
+    <row r="61">
+      <c r="A61" s="4" t="inlineStr"/>
+      <c r="B61" s="4" t="inlineStr">
+        <is>
+          <t>Schmidt &amp; Hunter, The Validity and Utility of Selection Methods in Personnel Psychology, Psychological Bulletin 124(2), 262-274 (1998)</t>
+        </is>
+      </c>
+      <c r="C61" s="4" t="inlineStr"/>
+      <c r="D61" s="4" t="inlineStr"/>
+    </row>
+    <row r="62">
+      <c r="A62" s="4" t="inlineStr"/>
+      <c r="B62" s="4" t="inlineStr">
+        <is>
+          <t>Tuckman, Developmental Sequence in Small Groups, Psychological Bulletin 63(6), 384-399 (1965) — https://doi.org/10.1037/h0022100</t>
+        </is>
+      </c>
+      <c r="C62" s="4" t="inlineStr"/>
+      <c r="D62" s="4" t="inlineStr"/>
+    </row>
+    <row r="63">
+      <c r="A63" s="4" t="inlineStr"/>
+      <c r="B63" s="4" t="inlineStr">
+        <is>
+          <t>Whitmore, Coaching for Performance: GROWing Human Potential and Purpose, 4th ed. (Nicholas Brealey, 2009; orig. 1992) — https://www.nicholasbrealey.com/coaching-for-performance/</t>
+        </is>
+      </c>
+      <c r="C63" s="4" t="inlineStr"/>
+      <c r="D63" s="4" t="inlineStr"/>
+    </row>
+    <row r="64">
+      <c r="A64" s="4" t="inlineStr"/>
+      <c r="B64" s="4" t="inlineStr">
+        <is>
+          <t>Google re:Work, Following the Data: The Research Behind Great Managers (Project Oxygen research, accessed 2026-07) — https://rework.withgoogle.com/intl/en/guides/following-the-data-the-research-behind-great-managers</t>
+        </is>
+      </c>
+      <c r="C64" s="4" t="inlineStr"/>
+      <c r="D64" s="4" t="inlineStr"/>
+    </row>
+    <row r="65">
+      <c r="A65" s="4" t="inlineStr"/>
+      <c r="B65" s="4" t="inlineStr">
+        <is>
+          <t>Scott, Radical Candor: Be a Kick-Ass Boss Without Losing Your Humanity (St. Martin's Press, 2017) — https://www.radicalcandor.com/</t>
+        </is>
+      </c>
+      <c r="C65" s="4" t="inlineStr"/>
+      <c r="D65" s="4" t="inlineStr"/>
+    </row>
+    <row r="66">
+      <c r="A66" s="4" t="inlineStr"/>
+      <c r="B66" s="4" t="inlineStr">
+        <is>
+          <t>Grove, High Output Management (Random House, 1983) — https://www.penguinrandomhouse.com/books/163289/high-output-management-by-andrew-s-grove/</t>
+        </is>
+      </c>
+      <c r="C66" s="4" t="inlineStr"/>
+      <c r="D66" s="4" t="inlineStr"/>
+    </row>
+    <row r="67">
+      <c r="A67" s="4" t="inlineStr"/>
+      <c r="B67" s="4" t="inlineStr">
+        <is>
+          <t>Hewlett, Forget a Mentor, Find a Sponsor: The New Way to Fast-Track Your Career (Harvard Business Review Press, 2013) — https://www.barnesandnoble.com/w/forget-a-mentor-find-a-sponsor-sylvia-ann-hewlett/1114264520</t>
+        </is>
+      </c>
+      <c r="C67" s="4" t="inlineStr"/>
+      <c r="D67" s="4" t="inlineStr"/>
+    </row>
+    <row r="68">
+      <c r="A68" s="4" t="inlineStr"/>
+      <c r="B68" s="4" t="inlineStr">
+        <is>
+          <t>Charan, Drotter &amp; Noel, The Leadership Pipeline: How to Build the Leadership-Powered Company, 2nd Edition (Jossey-Bass, 2010) — https://www.wiley.com/en-us/The+Leadership+Pipeline%3A+How+to+Build+the+Leadership-Powered+Company-p-9780787958527</t>
+        </is>
+      </c>
+      <c r="C68" s="4" t="inlineStr"/>
+      <c r="D68" s="4" t="inlineStr"/>
+    </row>
+    <row r="69">
+      <c r="A69" s="4" t="inlineStr"/>
+      <c r="B69" s="4" t="inlineStr">
+        <is>
+          <t>Edmondson, The Fearless Organization: Creating Psychological Safety in the Workplace for Learning, Innovation, and Growth (Wiley, 2018) — https://www.wiley.com/en-us/The+Fearless+Organization%3A+Creating+Psychological+Safety+in+the+Workplace+for+Learning%2C+Innovation%2C+and+Growth-p-9781119477242</t>
+        </is>
+      </c>
+      <c r="C69" s="4" t="inlineStr"/>
+      <c r="D69" s="4" t="inlineStr"/>
+    </row>
+    <row r="70">
+      <c r="A70" s="4" t="inlineStr"/>
+      <c r="B70" s="4" t="inlineStr">
+        <is>
+          <t>Google re:Work, Guide: Understand Team Effectiveness (Project Aristotle research, accessed 2026-07) — https://rework.withgoogle.com/intl/en/guides/understand-team-effectiveness</t>
+        </is>
+      </c>
+      <c r="C70" s="4" t="inlineStr"/>
+      <c r="D70" s="4" t="inlineStr"/>
+    </row>
+    <row r="71">
+      <c r="A71" s="4" t="inlineStr"/>
+      <c r="B71" s="4" t="inlineStr">
+        <is>
+          <t>Deci &amp; Ryan, The "What" and "Why" of Goal Pursuits: Human Needs and the Self-Determination of Behavior, Psychological Inquiry 11(4), 227-268 (2000) — https://doi.org/10.1207/S15327965PLI1104_01</t>
+        </is>
+      </c>
+      <c r="C71" s="4" t="inlineStr"/>
+      <c r="D71" s="4" t="inlineStr"/>
+    </row>
+    <row r="72">
+      <c r="A72" s="4" t="inlineStr"/>
+      <c r="B72" s="4" t="inlineStr">
+        <is>
+          <t>Herzberg, One More Time: How Do You Motivate Employees?, Harvard Business Review 46(1), 53-62 (1968; HBR Classic reprint 2003) — https://hbr.org/2003/01/one-more-time-how-do-you-motivate-employees</t>
+        </is>
+      </c>
+      <c r="C72" s="4" t="inlineStr"/>
+      <c r="D72" s="4" t="inlineStr"/>
+    </row>
+    <row r="73">
+      <c r="A73" s="4" t="inlineStr"/>
+      <c r="B73" s="4" t="inlineStr">
+        <is>
+          <t>Hunt, Prince, Dixon-Fyle &amp; Yee, Diversity Wins: How Inclusion Matters (McKinsey &amp; Company, 2020) — https://www.mckinsey.com/featured-insights/diversity-and-inclusion/diversity-wins-interactive</t>
+        </is>
+      </c>
+      <c r="C73" s="4" t="inlineStr"/>
+      <c r="D73" s="4" t="inlineStr"/>
+    </row>
+    <row r="74">
+      <c r="A74" s="4" t="inlineStr"/>
+      <c r="B74" s="4" t="inlineStr">
+        <is>
+          <t>Fournier, The Manager's Path (O'Reilly, 2017) — https://www.oreilly.com/library/view/the-managers-path/9781491973882/</t>
+        </is>
+      </c>
+      <c r="C74" s="4" t="inlineStr"/>
+      <c r="D74" s="4" t="inlineStr"/>
+    </row>
+    <row r="75">
+      <c r="A75" s="4" t="inlineStr"/>
+      <c r="B75" s="4" t="inlineStr">
+        <is>
+          <t>SFIA Foundation, Skills Framework for the Information Age, version 9 (2024) — https://sfia-online.org/en/sfia-9</t>
+        </is>
+      </c>
+      <c r="C75" s="4" t="inlineStr"/>
+      <c r="D75" s="4" t="inlineStr"/>
+    </row>
+    <row r="76">
+      <c r="A76" s="4" t="inlineStr"/>
+      <c r="B76" s="4" t="inlineStr">
+        <is>
+          <t>Larson, An Elegant Puzzle: Systems of Engineering Management (Stripe Press, 2019) — https://press.stripe.com/an-elegant-puzzle</t>
+        </is>
+      </c>
+      <c r="C76" s="4" t="inlineStr"/>
+      <c r="D76" s="4" t="inlineStr"/>
+    </row>
+    <row r="77">
+      <c r="A77" s="4" t="inlineStr"/>
+      <c r="B77" s="4" t="inlineStr">
+        <is>
+          <t>Wardley, Wardley Maps: Topographical Intelligence in Business (2016, online book) — https://wardleymaps.com/</t>
+        </is>
+      </c>
+      <c r="C77" s="4" t="inlineStr"/>
+      <c r="D77" s="4" t="inlineStr"/>
+    </row>
+    <row r="78">
+      <c r="A78" s="4" t="inlineStr"/>
+      <c r="B78" s="4" t="inlineStr">
+        <is>
+          <t>Cagan, INSPIRED: How to Create Tech Products Customers Love, 2nd Edition (Wiley, 2018) — https://www.svpg.com/inspired-2nd-edition/</t>
+        </is>
+      </c>
+      <c r="C78" s="4" t="inlineStr"/>
+      <c r="D78" s="4" t="inlineStr"/>
+    </row>
+    <row r="79">
+      <c r="A79" s="4" t="inlineStr"/>
+      <c r="B79" s="4" t="inlineStr">
+        <is>
+          <t>Conway, How Do Committees Invent?, Datamation 14(4), 28-31 (1968) — https://www.melconway.com/Home/Committees_Paper.html</t>
+        </is>
+      </c>
+      <c r="C79" s="4" t="inlineStr"/>
+      <c r="D79" s="4" t="inlineStr"/>
+    </row>
+    <row r="80">
+      <c r="A80" s="4" t="inlineStr"/>
+      <c r="B80" s="4" t="inlineStr">
+        <is>
+          <t>Nygard, Documenting Architecture Decisions (Cognitect blog, 2011) — https://cognitect.com/blog/2011/11/15/documenting-architecture-decisions</t>
+        </is>
+      </c>
+      <c r="C80" s="4" t="inlineStr"/>
+      <c r="D80" s="4" t="inlineStr"/>
+    </row>
+    <row r="81">
+      <c r="A81" s="4" t="inlineStr"/>
+      <c r="B81" s="4" t="inlineStr">
+        <is>
+          <t>Humble &amp; Farley, Continuous Delivery: Reliable Software Releases through Build Test and Deployment Automation (Addison-Wesley, 2010) — https://continuousdelivery.com/</t>
+        </is>
+      </c>
+      <c r="C81" s="4" t="inlineStr"/>
+      <c r="D81" s="4" t="inlineStr"/>
+    </row>
+    <row r="82">
+      <c r="A82" s="4" t="inlineStr"/>
+      <c r="B82" s="4" t="inlineStr">
+        <is>
+          <t>Cunningham, The WyCash Portfolio Management System, OOPSLA 1992 Experience Report — https://c2.com/doc/oopsla92.html</t>
+        </is>
+      </c>
+      <c r="C82" s="4" t="inlineStr"/>
+      <c r="D82" s="4" t="inlineStr"/>
+    </row>
+    <row r="83">
+      <c r="A83" s="4" t="inlineStr"/>
+      <c r="B83" s="4" t="inlineStr">
+        <is>
+          <t>Minto, The Minto Pyramid Principle: Logic in Writing, Thinking, and Problem Solving (Minto International, 1996) — https://www.barbaraminto.com/</t>
+        </is>
+      </c>
+      <c r="C83" s="4" t="inlineStr"/>
+      <c r="D83" s="4" t="inlineStr"/>
+    </row>
+    <row r="84">
+      <c r="A84" s="4" t="inlineStr"/>
+      <c r="B84" s="4" t="inlineStr">
+        <is>
+          <t>Duarte, HBR Guide to Persuasive Presentations (Harvard Business Review Press, 2012) — https://store.hbr.org/product/hbr-guide-to-persuasive-presentations/10058</t>
+        </is>
+      </c>
+      <c r="C84" s="4" t="inlineStr"/>
+      <c r="D84" s="4" t="inlineStr"/>
+    </row>
+    <row r="85">
+      <c r="A85" s="4" t="inlineStr"/>
+      <c r="B85" s="4" t="inlineStr">
+        <is>
+          <t>Freeman, Strategic Management: A Stakeholder Approach (Pitman, 1984)</t>
+        </is>
+      </c>
+      <c r="C85" s="4" t="inlineStr"/>
+      <c r="D85" s="4" t="inlineStr"/>
+    </row>
+    <row r="86">
+      <c r="A86" s="4" t="inlineStr"/>
+      <c r="B86" s="4" t="inlineStr">
+        <is>
+          <t>Cohen &amp; Bradford, Influence Without Authority, 3rd ed. (Wiley, 2017) — https://www.wiley.com/en-us/Influence+Without+Authority,+3rd+Edition-p-9781119347712</t>
+        </is>
+      </c>
+      <c r="C86" s="4" t="inlineStr"/>
+      <c r="D86" s="4" t="inlineStr"/>
+    </row>
+    <row r="87">
+      <c r="A87" s="4" t="inlineStr"/>
+      <c r="B87" s="4" t="inlineStr">
+        <is>
+          <t>Fisher &amp; Ury, Getting to Yes: Negotiating Agreement Without Giving In (Penguin, 1981) — https://www.pon.harvard.edu/shop/getting-to-yes-negotiating-agreement-without-giving-in/</t>
+        </is>
+      </c>
+      <c r="C87" s="4" t="inlineStr"/>
+      <c r="D87" s="4" t="inlineStr"/>
+    </row>
+    <row r="88">
+      <c r="A88" s="4" t="inlineStr"/>
+      <c r="B88" s="4" t="inlineStr">
+        <is>
+          <t>Lencioni, The Five Dysfunctions of a Team: A Leadership Fable (Jossey-Bass, 2002) — https://openlibrary.org/works/OL3906183W/The_five_dysfunctions_of_a_team</t>
+        </is>
+      </c>
+      <c r="C88" s="4" t="inlineStr"/>
+      <c r="D88" s="4" t="inlineStr"/>
+    </row>
+    <row r="89">
+      <c r="A89" s="4" t="inlineStr"/>
+      <c r="B89" s="4" t="inlineStr">
+        <is>
+          <t>Drucker, The Effective Executive (Harper &amp; Row, 1967)</t>
+        </is>
+      </c>
+      <c r="C89" s="4" t="inlineStr"/>
+      <c r="D89" s="4" t="inlineStr"/>
+    </row>
+    <row r="90">
+      <c r="A90" s="4" t="inlineStr"/>
+      <c r="B90" s="4" t="inlineStr">
+        <is>
+          <t>Marquet, Turn the Ship Around!: A True Story of Turning Followers into Leaders (Portfolio/Penguin, 2013; orig. 2012)</t>
+        </is>
+      </c>
+      <c r="C90" s="4" t="inlineStr"/>
+      <c r="D90" s="4" t="inlineStr"/>
+    </row>
+    <row r="91">
+      <c r="A91" s="4" t="inlineStr"/>
+      <c r="B91" s="4" t="inlineStr">
+        <is>
+          <t>Eurich, What Self-Awareness Really Is (and How to Cultivate It), Harvard Business Review (2018) — https://hbr.org/2018/01/what-self-awareness-really-is-and-how-to-cultivate-it</t>
+        </is>
+      </c>
+      <c r="C91" s="4" t="inlineStr"/>
+      <c r="D91" s="4" t="inlineStr"/>
+    </row>
+    <row r="92">
+      <c r="A92" s="4" t="inlineStr"/>
+      <c r="B92" s="4" t="inlineStr">
+        <is>
+          <t>Lombardo &amp; Eichinger, The Career Architect Development Planner, 3rd ed. (Lominger, 2000)</t>
+        </is>
+      </c>
+      <c r="C92" s="4" t="inlineStr"/>
+      <c r="D92" s="4" t="inlineStr"/>
+    </row>
+    <row r="93">
+      <c r="A93" s="4" t="inlineStr"/>
+      <c r="B93" s="4" t="inlineStr">
+        <is>
+          <t>Loehr &amp; Schwartz, The Power of Full Engagement: Managing Energy, Not Time, Is the Key to High Performance and Personal Renewal (Free Press, 2003)</t>
+        </is>
+      </c>
+      <c r="C93" s="4" t="inlineStr"/>
+      <c r="D93" s="4" t="inlineStr"/>
+    </row>
+    <row r="94">
+      <c r="A94" s="4" t="inlineStr"/>
+      <c r="B94" s="4" t="inlineStr">
+        <is>
+          <t>Kahneman, Thinking, Fast and Slow (Farrar, Straus and Giroux, 2011) — https://en.wikipedia.org/wiki/Thinking,_Fast_and_Slow</t>
+        </is>
+      </c>
+      <c r="C94" s="4" t="inlineStr"/>
+      <c r="D94" s="4" t="inlineStr"/>
+    </row>
+    <row r="95">
+      <c r="A95" s="4" t="inlineStr"/>
+      <c r="B95" s="4" t="inlineStr">
+        <is>
+          <t>Mayer, Davis &amp; Schoorman, An Integrative Model of Organizational Trust, Academy of Management Review 20(3), 709-734 (1995) — https://people.wku.edu/richard.miller/Mayer%20Trust%20article.pdf</t>
+        </is>
+      </c>
+      <c r="C95" s="4" t="inlineStr"/>
+      <c r="D95" s="4" t="inlineStr"/>
+    </row>
+    <row r="96">
+      <c r="A96" s="4" t="inlineStr"/>
+      <c r="B96" s="4" t="inlineStr">
+        <is>
+          <t>ACM, ACM Code of Ethics and Professional Conduct (2018) — https://www.acm.org/code-of-ethics</t>
+        </is>
+      </c>
+      <c r="C96" s="4" t="inlineStr"/>
+      <c r="D96" s="4" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>